<commit_message>
chore: adoption report 2026-06-16 18:56 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -545,7 +545,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  Generado: 2026-06-15</t>
+          <t>Quarter: Q2 2026  |  Generado: 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -604,14 +604,14 @@
         <v>22</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>11828</v>
+        <v>11837</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>9405</v>
+        <v>9883</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>54%</t>
         </is>
       </c>
     </row>
@@ -657,14 +657,14 @@
         <v>23</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>12473</v>
+        <v>12482</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>10054</v>
+        <v>10532</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>54%</t>
         </is>
       </c>
     </row>
@@ -759,17 +759,17 @@
         <v>15</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>6228</v>
+        <v>6237</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>3912</v>
+        <v>4390</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>10140</v>
+        <v>10627</v>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>59%</t>
         </is>
       </c>
     </row>
@@ -1010,11 +1010,11 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Component 16</t>
+          <t>DirectionDown</t>
         </is>
       </c>
       <c r="D6" s="14" t="n">
-        <v>270</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -1030,11 +1030,11 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Botón Primario</t>
+          <t>Component 16</t>
         </is>
       </c>
       <c r="D7" s="14" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -1130,11 +1130,11 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Botón Primario</t>
         </is>
       </c>
       <c r="D12" s="14" t="n">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -1150,11 +1150,11 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>barras</t>
+          <t>DirectionUp</t>
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -1170,11 +1170,11 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>settings</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -1190,11 +1190,11 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>billetera</t>
+          <t>barras</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -1210,11 +1210,11 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>settings</t>
         </is>
       </c>
       <c r="D16" s="14" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -1230,11 +1230,11 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>billetera</t>
         </is>
       </c>
       <c r="D17" s="14" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
@@ -1250,11 +1250,11 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>create account</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="D18" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -1270,11 +1270,11 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D19" s="14" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -1290,11 +1290,11 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>create account</t>
         </is>
       </c>
       <c r="D20" s="14" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -1310,11 +1310,11 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>AGENDA</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -1852,22 +1852,22 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>54%</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
         <v>22</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>11828</v>
+        <v>11837</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>21233</v>
+        <v>21720</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-16 22:53 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -604,14 +604,14 @@
         <v>22</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>11837</v>
+        <v>11902</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>9883</v>
+        <v>9931</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>55%</t>
         </is>
       </c>
     </row>
@@ -657,10 +657,10 @@
         <v>23</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>12482</v>
+        <v>12547</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>10532</v>
+        <v>10580</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
@@ -827,17 +827,17 @@
         <v>1</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>1592</v>
+        <v>1657</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>511</v>
+        <v>559</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>2103</v>
+        <v>2216</v>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="D5" s="14" t="n">
-        <v>643</v>
+        <v>636</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="D15" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="D16" s="14" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="D17" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
@@ -1250,11 +1250,11 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D18" s="14" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="D19" s="14" t="n">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="D20" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -1857,17 +1857,17 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
         <v>22</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>11837</v>
+        <v>11902</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>21720</v>
+        <v>21833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-17 17:48 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -70,6 +70,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FF1D9E75"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="FFF5A623"/>
       <sz val="10"/>
     </font>
@@ -77,12 +83,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FF1A7FA8"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF1D9E75"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -143,16 +143,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -604,14 +604,14 @@
         <v>17</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>2437</v>
+        <v>2680</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>5545</v>
+        <v>5302</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>34%</t>
         </is>
       </c>
     </row>
@@ -633,14 +633,14 @@
         <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>1215</v>
+        <v>3647</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3557</v>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>25%</t>
+        <v>967</v>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
         </is>
       </c>
     </row>
@@ -659,17 +659,17 @@
         <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>1900</v>
+        <v>4743</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>8303</v>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>19%</t>
+        <v>2412</v>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>66%</t>
         </is>
       </c>
     </row>
@@ -688,17 +688,17 @@
         <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>25727</v>
+        <v>154195</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>179865</v>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>13%</t>
+        <v>26003</v>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>86%</t>
         </is>
       </c>
     </row>
@@ -720,14 +720,14 @@
         <v>5</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>6522</v>
+        <v>10174</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>7315</v>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>47%</t>
+        <v>3543</v>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>74%</t>
         </is>
       </c>
     </row>
@@ -749,14 +749,14 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>11902</v>
+        <v>13591</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>9931</v>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>55%</t>
+        <v>8241</v>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>62%</t>
         </is>
       </c>
     </row>
@@ -778,14 +778,14 @@
         <v>16</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>6110</v>
+        <v>10028</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>9633</v>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>39%</t>
+        <v>5579</v>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>64%</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
         <v>3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>3604</v>
+        <v>10104</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>10108</v>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>26%</t>
+        <v>2700</v>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
         </is>
       </c>
     </row>
@@ -836,38 +836,38 @@
         <v>6</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>343</v>
+        <v>1422</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>1464</v>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>19%</t>
+        <v>337</v>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>81%</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="D14" s="10" t="n">
-        <v>202</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>59760</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>235721</v>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>20%</t>
+      <c r="D14" s="11" t="n">
+        <v>188</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>210584</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>55084</v>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>79%</t>
         </is>
       </c>
     </row>
@@ -962,17 +962,17 @@
         <v>4</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>474</v>
+        <v>574</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>820</v>
+        <v>720</v>
       </c>
       <c r="G2" s="6" t="n">
         <v>1294</v>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>11</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>1950</v>
+        <v>2093</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>4706</v>
+        <v>4563</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>6656</v>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>31%</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       <c r="G4" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>55%</t>
         </is>
@@ -1098,17 +1098,17 @@
         <v>5</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>663</v>
+        <v>1037</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1047</v>
+        <v>665</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>1710</v>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>39%</t>
+        <v>1702</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>61%</t>
         </is>
       </c>
     </row>
@@ -1132,17 +1132,17 @@
         <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>552</v>
+        <v>2610</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2510</v>
+        <v>302</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>3062</v>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>18%</t>
+        <v>2912</v>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>90%</t>
         </is>
       </c>
     </row>
@@ -1166,17 +1166,17 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>342</v>
+        <v>1272</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>1253</v>
+        <v>275</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>1595</v>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>21%</t>
+        <v>1547</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -1197,20 +1197,20 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1558</v>
+        <v>3471</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>7050</v>
+        <v>2137</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>8608</v>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>18%</t>
+        <v>5608</v>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>62%</t>
         </is>
       </c>
     </row>
@@ -1231,20 +1231,20 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1446</v>
+        <v>0</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>16460</v>
+        <v>0</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>17906</v>
+        <v>0</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1268,17 +1268,17 @@
         <v>37</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>24281</v>
+        <v>154195</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>163405</v>
+        <v>26003</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>187686</v>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>13%</t>
+        <v>180198</v>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>86%</t>
         </is>
       </c>
     </row>
@@ -1302,17 +1302,17 @@
         <v>5</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>6522</v>
+        <v>10174</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>7315</v>
+        <v>3543</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>13837</v>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>47%</t>
+        <v>13717</v>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>74%</t>
         </is>
       </c>
     </row>
@@ -1336,17 +1336,17 @@
         <v>15</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>6237</v>
+        <v>7697</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>4390</v>
+        <v>2930</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>10627</v>
       </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>59%</t>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>72%</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1370,17 @@
         <v>6</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>4008</v>
+        <v>4145</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>4982</v>
+        <v>4844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>8990</v>
+        <v>8989</v>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>46%</t>
         </is>
       </c>
     </row>
@@ -1404,17 +1404,17 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1657</v>
+        <v>1749</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>559</v>
+        <v>467</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>2216</v>
       </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>75%</t>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
         </is>
       </c>
     </row>
@@ -1438,17 +1438,17 @@
         <v>1</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>1224</v>
+        <v>1508</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>963</v>
+        <v>679</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>2187</v>
       </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>56%</t>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>69%</t>
         </is>
       </c>
     </row>
@@ -1472,17 +1472,17 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1550</v>
+        <v>2007</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>1723</v>
+        <v>1266</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>3273</v>
       </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>47%</t>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>61%</t>
         </is>
       </c>
     </row>
@@ -1506,17 +1506,17 @@
         <v>1</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>645</v>
+        <v>825</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>649</v>
+        <v>469</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>1294</v>
       </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>50%</t>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>64%</t>
         </is>
       </c>
     </row>
@@ -1540,17 +1540,17 @@
         <v>2</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>1830</v>
+        <v>2329</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>2241</v>
+        <v>1742</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>4071</v>
       </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>45%</t>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>57%</t>
         </is>
       </c>
     </row>
@@ -1574,17 +1574,17 @@
         <v>11</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>861</v>
+        <v>3359</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>4057</v>
+        <v>1423</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>4918</v>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>18%</t>
+        <v>4782</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>70%</t>
         </is>
       </c>
     </row>
@@ -1639,20 +1639,20 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>2104</v>
+        <v>4525</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>4149</v>
+        <v>1006</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>6253</v>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>34%</t>
+        <v>5531</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -1676,17 +1676,17 @@
         <v>3</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>912</v>
+        <v>4204</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>4879</v>
+        <v>1427</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>5791</v>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>16%</t>
+        <v>5631</v>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1710,17 +1710,17 @@
         <v>14</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>588</v>
+        <v>1375</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>1080</v>
+        <v>267</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>1668</v>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>35%</t>
+        <v>1642</v>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>84%</t>
         </is>
       </c>
     </row>
@@ -1744,17 +1744,17 @@
         <v>6</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>343</v>
+        <v>1422</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>1464</v>
+        <v>337</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>1807</v>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>19%</t>
+        <v>1759</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>81%</t>
         </is>
       </c>
     </row>
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D8" s="14" t="n">
-        <v>204</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>shoppingcart</t>
         </is>
       </c>
       <c r="D9" s="14" t="n">
@@ -1973,11 +1973,11 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>shoppingcart</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="D10" s="14" t="n">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -1993,11 +1993,11 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="D11" s="14" t="n">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -2013,11 +2013,11 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>Star</t>
         </is>
       </c>
       <c r="D12" s="14" t="n">
-        <v>174</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Star</t>
+          <t>Bottom app bar</t>
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>162</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -2053,11 +2053,11 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Bottom app bar</t>
+          <t>documento simple</t>
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>138</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -2073,11 +2073,11 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>documento simple</t>
+          <t>Seguros card</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -2093,11 +2093,11 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Seguros card</t>
+          <t>sirena emergencia</t>
         </is>
       </c>
       <c r="D16" s="14" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -2133,11 +2133,11 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>sirena emergencia</t>
+          <t>informacion de poliza</t>
         </is>
       </c>
       <c r="D18" s="14" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -2213,11 +2213,11 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="D22" s="14" t="n">
-        <v>1500</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Suggested search (Deprecated)</t>
         </is>
       </c>
       <c r="D23" s="14" t="n">
-        <v>255</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
@@ -2253,11 +2253,11 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D24" s="14" t="n">
-        <v>250</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -2273,11 +2273,11 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Step 01</t>
         </is>
       </c>
       <c r="D25" s="14" t="n">
-        <v>196</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
@@ -2293,11 +2293,11 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Step 02</t>
         </is>
       </c>
       <c r="D26" s="14" t="n">
-        <v>150</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -2313,11 +2313,11 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>Step 03</t>
         </is>
       </c>
       <c r="D27" s="14" t="n">
-        <v>150</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>celda L</t>
         </is>
       </c>
       <c r="D28" s="14" t="n">
-        <v>95</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -2353,11 +2353,11 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Suggested search (Deprecated)</t>
+          <t>Step 04</t>
         </is>
       </c>
       <c r="D29" s="14" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
@@ -2373,11 +2373,11 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Step 05</t>
         </is>
       </c>
       <c r="D30" s="14" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
@@ -2393,11 +2393,11 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Step 01</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D31" s="14" t="n">
-        <v>59</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
@@ -2413,11 +2413,11 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Step 02</t>
+          <t>Upload icon</t>
         </is>
       </c>
       <c r="D32" s="14" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Step 03</t>
+          <t>Userflow</t>
         </is>
       </c>
       <c r="D33" s="14" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>ArrowLeft</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -2473,11 +2473,11 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>celda L</t>
+          <t>celda S</t>
         </is>
       </c>
       <c r="D35" s="14" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
@@ -2493,11 +2493,11 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Step 04</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
-        <v>39</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
@@ -2513,11 +2513,11 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Step 05</t>
+          <t>titulo-fila</t>
         </is>
       </c>
       <c r="D37" s="14" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>generate ai</t>
         </is>
       </c>
       <c r="D38" s="14" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
@@ -2553,11 +2553,11 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>More</t>
         </is>
       </c>
       <c r="D39" s="14" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
@@ -2573,11 +2573,11 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>arrow_carrousel</t>
         </is>
       </c>
       <c r="D40" s="14" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
@@ -2593,11 +2593,11 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Upload icon</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="D41" s="14" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
@@ -2613,11 +2613,11 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Menu Item</t>
         </is>
       </c>
       <c r="D42" s="14" t="n">
-        <v>3264</v>
+        <v>520</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="D43" s="14" t="n">
-        <v>640</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
@@ -2653,11 +2653,11 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="D44" s="14" t="n">
-        <v>544</v>
+        <v>103</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
@@ -2673,11 +2673,11 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>HealthAndSafe</t>
         </is>
       </c>
       <c r="D45" s="14" t="n">
-        <v>316</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
@@ -2693,11 +2693,11 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Notification Item</t>
         </is>
       </c>
       <c r="D46" s="14" t="n">
-        <v>276</v>
+        <v>75</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
@@ -2713,11 +2713,11 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>eye_close</t>
         </is>
       </c>
       <c r="D47" s="14" t="n">
-        <v>272</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="D48" s="14" t="n">
-        <v>272</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
@@ -2753,11 +2753,11 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D49" s="14" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
@@ -2773,11 +2773,11 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D50" s="14" t="n">
-        <v>160</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
@@ -2793,11 +2793,11 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D51" s="14" t="n">
-        <v>136</v>
+        <v>58</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
@@ -2813,11 +2813,11 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>time</t>
         </is>
       </c>
       <c r="D52" s="14" t="n">
-        <v>105</v>
+        <v>56</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>menu</t>
         </is>
       </c>
       <c r="D53" s="14" t="n">
-        <v>105</v>
+        <v>54</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
@@ -2853,11 +2853,11 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>HealthAndSafe</t>
+          <t>Beneficio | card</t>
         </is>
       </c>
       <c r="D54" s="14" t="n">
-        <v>96</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Notification Item</t>
+          <t>Apps</t>
         </is>
       </c>
       <c r="D55" s="14" t="n">
-        <v>93</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
@@ -2893,11 +2893,11 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>eye_close</t>
+          <t>Beneficio | card mobile</t>
         </is>
       </c>
       <c r="D56" s="14" t="n">
-        <v>93</v>
+        <v>42</v>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
@@ -2913,11 +2913,11 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>menu</t>
+          <t>Slider</t>
         </is>
       </c>
       <c r="D57" s="14" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="D58" s="14" t="n">
-        <v>61</v>
+        <v>38</v>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
@@ -2953,11 +2953,11 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>generate ai</t>
         </is>
       </c>
       <c r="D59" s="14" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
@@ -2973,11 +2973,11 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>Atajos | Beneficios (new)</t>
         </is>
       </c>
       <c r="D60" s="14" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
@@ -2993,11 +2993,11 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Apps</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D61" s="14" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
@@ -3013,11 +3013,11 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D62" s="14" t="n">
-        <v>96329</v>
+        <v>4980</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>celda S</t>
         </is>
       </c>
       <c r="D63" s="14" t="n">
-        <v>16943</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
@@ -3053,11 +3053,11 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>eye_close</t>
         </is>
       </c>
       <c r="D64" s="14" t="n">
-        <v>9112</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
@@ -3073,11 +3073,11 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Notification Item</t>
         </is>
       </c>
       <c r="D65" s="14" t="n">
-        <v>8640</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
@@ -3093,11 +3093,11 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>menu</t>
         </is>
       </c>
       <c r="D66" s="14" t="n">
-        <v>8256</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
@@ -3113,11 +3113,11 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="D67" s="14" t="n">
-        <v>5595</v>
+        <v>948</v>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Apps</t>
         </is>
       </c>
       <c r="D68" s="14" t="n">
-        <v>4319</v>
+        <v>793</v>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
@@ -3153,11 +3153,11 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>celda S</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="D69" s="14" t="n">
-        <v>2366</v>
+        <v>780</v>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
@@ -3173,11 +3173,11 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D70" s="14" t="n">
-        <v>2109</v>
+        <v>697</v>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
@@ -3193,11 +3193,11 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="D71" s="14" t="n">
-        <v>1868</v>
+        <v>692</v>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
@@ -3213,11 +3213,11 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>eye_close</t>
+          <t>tiktok</t>
         </is>
       </c>
       <c r="D72" s="14" t="n">
-        <v>1671</v>
+        <v>692</v>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Notification Item</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="D73" s="14" t="n">
-        <v>1536</v>
+        <v>692</v>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
@@ -3253,11 +3253,11 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>account</t>
         </is>
       </c>
       <c r="D74" s="14" t="n">
-        <v>1166</v>
+        <v>564</v>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
@@ -3273,11 +3273,11 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_badges_download</t>
         </is>
       </c>
       <c r="D75" s="14" t="n">
-        <v>1080</v>
+        <v>518</v>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
@@ -3293,11 +3293,11 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>call</t>
         </is>
       </c>
       <c r="D76" s="14" t="n">
-        <v>1080</v>
+        <v>514</v>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
@@ -3313,11 +3313,11 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>menu</t>
+          <t>Home_Header</t>
         </is>
       </c>
       <c r="D77" s="14" t="n">
-        <v>1019</v>
+        <v>511</v>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Action 1</t>
         </is>
       </c>
       <c r="D78" s="14" t="n">
-        <v>948</v>
+        <v>496</v>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
@@ -3353,11 +3353,11 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Apps</t>
+          <t>Action 2</t>
         </is>
       </c>
       <c r="D79" s="14" t="n">
-        <v>793</v>
+        <v>496</v>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
@@ -3373,11 +3373,11 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Menu_Mobile</t>
         </is>
       </c>
       <c r="D80" s="14" t="n">
-        <v>780</v>
+        <v>482</v>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1">
@@ -3393,11 +3393,11 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>titulo-fila</t>
         </is>
       </c>
       <c r="D81" s="14" t="n">
-        <v>697</v>
+        <v>433</v>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Pegar Icon</t>
         </is>
       </c>
       <c r="D82" s="14" t="n">
-        <v>1440</v>
+        <v>484</v>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>copy</t>
         </is>
       </c>
       <c r="D83" s="14" t="n">
-        <v>569</v>
+        <v>439</v>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
@@ -3453,11 +3453,11 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Pegar Icon</t>
+          <t>DirectionDown</t>
         </is>
       </c>
       <c r="D84" s="14" t="n">
-        <v>484</v>
+        <v>328</v>
       </c>
     </row>
     <row r="85" ht="20" customHeight="1">
@@ -3473,11 +3473,11 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>copy</t>
+          <t>DirectionRight</t>
         </is>
       </c>
       <c r="D85" s="14" t="n">
-        <v>439</v>
+        <v>268</v>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1">
@@ -3493,11 +3493,11 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>DirectionDown</t>
+          <t>power</t>
         </is>
       </c>
       <c r="D86" s="14" t="n">
-        <v>328</v>
+        <v>212</v>
       </c>
     </row>
     <row r="87" ht="20" customHeight="1">
@@ -3513,11 +3513,11 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>call</t>
         </is>
       </c>
       <c r="D87" s="14" t="n">
-        <v>306</v>
+        <v>153</v>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>DirectionRight</t>
+          <t>Option</t>
         </is>
       </c>
       <c r="D88" s="14" t="n">
-        <v>268</v>
+        <v>139</v>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
@@ -3553,11 +3553,11 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Component 9</t>
         </is>
       </c>
       <c r="D89" s="14" t="n">
-        <v>240</v>
+        <v>94</v>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
@@ -3573,11 +3573,11 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D90" s="14" t="n">
-        <v>228</v>
+        <v>93</v>
       </c>
     </row>
     <row r="91" ht="20" customHeight="1">
@@ -3593,11 +3593,11 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>power</t>
+          <t>Logo Horizontal</t>
         </is>
       </c>
       <c r="D91" s="14" t="n">
-        <v>212</v>
+        <v>73</v>
       </c>
     </row>
     <row r="92" ht="20" customHeight="1">
@@ -3613,11 +3613,11 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="D92" s="14" t="n">
-        <v>204</v>
+        <v>61</v>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D93" s="14" t="n">
-        <v>190</v>
+        <v>60</v>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
@@ -3653,11 +3653,11 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>Card Dashboard</t>
         </is>
       </c>
       <c r="D94" s="14" t="n">
-        <v>153</v>
+        <v>56</v>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1">
@@ -3673,11 +3673,11 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>mail</t>
         </is>
       </c>
       <c r="D95" s="14" t="n">
-        <v>150</v>
+        <v>47</v>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
@@ -3693,11 +3693,11 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Frame 1707479054</t>
         </is>
       </c>
       <c r="D96" s="14" t="n">
-        <v>139</v>
+        <v>46</v>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
@@ -3713,11 +3713,11 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Frame 1707479133</t>
         </is>
       </c>
       <c r="D97" s="14" t="n">
-        <v>120</v>
+        <v>44</v>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D98" s="14" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
@@ -3753,11 +3753,11 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Component 9</t>
+          <t>Indicator number</t>
         </is>
       </c>
       <c r="D99" s="14" t="n">
-        <v>94</v>
+        <v>32</v>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
@@ -3773,11 +3773,11 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D100" s="14" t="n">
-        <v>93</v>
+        <v>29</v>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
@@ -3793,11 +3793,11 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Logo Horizontal</t>
+          <t>informacion de poliza</t>
         </is>
       </c>
       <c r="D101" s="14" t="n">
-        <v>73</v>
+        <v>27</v>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D103" s="14" t="n">
-        <v>666</v>
+        <v>643</v>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
@@ -3853,11 +3853,11 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>DirectionDown</t>
         </is>
       </c>
       <c r="D104" s="14" t="n">
-        <v>646</v>
+        <v>311</v>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
@@ -3873,11 +3873,11 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Component 16</t>
         </is>
       </c>
       <c r="D105" s="14" t="n">
-        <v>636</v>
+        <v>270</v>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
@@ -3893,11 +3893,11 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>DirectionDown</t>
+          <t>Botón Primario</t>
         </is>
       </c>
       <c r="D106" s="14" t="n">
-        <v>311</v>
+        <v>180</v>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
@@ -3913,11 +3913,11 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Component 16</t>
+          <t>Dropdown filter page</t>
         </is>
       </c>
       <c r="D107" s="14" t="n">
-        <v>270</v>
+        <v>159</v>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Dropdown filter page</t>
+          <t>width fixed pagination</t>
         </is>
       </c>
       <c r="D108" s="14" t="n">
@@ -3953,11 +3953,11 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>width fixed pagination</t>
+          <t>Line Tracking Vertical</t>
         </is>
       </c>
       <c r="D109" s="14" t="n">
-        <v>159</v>
+        <v>135</v>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
@@ -3973,11 +3973,11 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Indicator Circle</t>
+          <t>DirectionUp</t>
         </is>
       </c>
       <c r="D110" s="14" t="n">
-        <v>135</v>
+        <v>116</v>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
@@ -3993,11 +3993,11 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Line Tracking Vertical</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="D111" s="14" t="n">
-        <v>135</v>
+        <v>115</v>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
@@ -4013,11 +4013,11 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Botón Primario</t>
+          <t>barras</t>
         </is>
       </c>
       <c r="D112" s="14" t="n">
-        <v>126</v>
+        <v>111</v>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>DirectionUp</t>
+          <t>settings</t>
         </is>
       </c>
       <c r="D113" s="14" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="114" ht="20" customHeight="1">
@@ -4053,11 +4053,11 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D114" s="14" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="115" ht="20" customHeight="1">
@@ -4073,11 +4073,11 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>barras</t>
+          <t>billetera</t>
         </is>
       </c>
       <c r="D115" s="14" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="116" ht="20" customHeight="1">
@@ -4093,11 +4093,11 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>settings</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D116" s="14" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="117" ht="20" customHeight="1">
@@ -4113,11 +4113,11 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>billetera</t>
+          <t>create account</t>
         </is>
       </c>
       <c r="D117" s="14" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="118" ht="20" customHeight="1">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D118" s="14" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="119" ht="20" customHeight="1">
@@ -4153,11 +4153,11 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>directionLeft</t>
         </is>
       </c>
       <c r="D119" s="14" t="n">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="120" ht="20" customHeight="1">
@@ -4173,11 +4173,11 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>create account</t>
+          <t>AGENDA</t>
         </is>
       </c>
       <c r="D120" s="14" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
     </row>
     <row r="121" ht="20" customHeight="1">
@@ -4193,11 +4193,11 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D121" s="14" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="122" ht="20" customHeight="1">
@@ -4213,11 +4213,11 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Menu Item</t>
         </is>
       </c>
       <c r="D122" s="14" t="n">
-        <v>1632</v>
+        <v>380</v>
       </c>
     </row>
     <row r="123" ht="20" customHeight="1">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="D123" s="14" t="n">
-        <v>635</v>
+        <v>352</v>
       </c>
     </row>
     <row r="124" ht="20" customHeight="1">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>celda</t>
         </is>
       </c>
       <c r="D124" s="14" t="n">
-        <v>380</v>
+        <v>312</v>
       </c>
     </row>
     <row r="125" ht="20" customHeight="1">
@@ -4273,11 +4273,11 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="D125" s="14" t="n">
-        <v>336</v>
+        <v>248</v>
       </c>
     </row>
     <row r="126" ht="20" customHeight="1">
@@ -4293,11 +4293,11 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>celda</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D126" s="14" t="n">
-        <v>312</v>
+        <v>224</v>
       </c>
     </row>
     <row r="127" ht="20" customHeight="1">
@@ -4313,11 +4313,11 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Property 33</t>
+          <t>02</t>
         </is>
       </c>
       <c r="D127" s="14" t="n">
-        <v>272</v>
+        <v>212</v>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>add</t>
         </is>
       </c>
       <c r="D128" s="14" t="n">
-        <v>272</v>
+        <v>159</v>
       </c>
     </row>
     <row r="129" ht="20" customHeight="1">
@@ -4353,11 +4353,11 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>01</t>
         </is>
       </c>
       <c r="D129" s="14" t="n">
-        <v>248</v>
+        <v>139</v>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
@@ -4373,11 +4373,11 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D130" s="14" t="n">
-        <v>212</v>
+        <v>119</v>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
@@ -4393,11 +4393,11 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>Toast</t>
         </is>
       </c>
       <c r="D131" s="14" t="n">
-        <v>210</v>
+        <v>118</v>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
@@ -4413,11 +4413,11 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D132" s="14" t="n">
-        <v>184</v>
+        <v>105</v>
       </c>
     </row>
     <row r="133" ht="20" customHeight="1">
@@ -4433,11 +4433,11 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>call</t>
         </is>
       </c>
       <c r="D133" s="14" t="n">
-        <v>174</v>
+        <v>104</v>
       </c>
     </row>
     <row r="134" ht="20" customHeight="1">
@@ -4453,11 +4453,11 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="D134" s="14" t="n">
-        <v>170</v>
+        <v>95</v>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
@@ -4473,11 +4473,11 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>add</t>
+          <t>Indicator Mobile</t>
         </is>
       </c>
       <c r="D135" s="14" t="n">
-        <v>159</v>
+        <v>86</v>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1">
@@ -4493,11 +4493,11 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="D136" s="14" t="n">
-        <v>153</v>
+        <v>81</v>
       </c>
     </row>
     <row r="137" ht="20" customHeight="1">
@@ -4513,11 +4513,11 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="D137" s="14" t="n">
-        <v>139</v>
+        <v>78</v>
       </c>
     </row>
     <row r="138" ht="20" customHeight="1">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Infotip</t>
         </is>
       </c>
       <c r="D138" s="14" t="n">
-        <v>136</v>
+        <v>57</v>
       </c>
     </row>
     <row r="139" ht="20" customHeight="1">
@@ -4553,11 +4553,11 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>Component 120</t>
         </is>
       </c>
       <c r="D139" s="14" t="n">
-        <v>136</v>
+        <v>56</v>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
@@ -4573,11 +4573,11 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Smile</t>
         </is>
       </c>
       <c r="D140" s="14" t="n">
-        <v>119</v>
+        <v>55</v>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
@@ -4593,11 +4593,11 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Toast</t>
+          <t>directionLeft</t>
         </is>
       </c>
       <c r="D141" s="14" t="n">
-        <v>106</v>
+        <v>55</v>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
@@ -4613,11 +4613,11 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D142" s="14" t="n">
-        <v>3135</v>
+        <v>280</v>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D143" s="14" t="n">
-        <v>1095</v>
+        <v>215</v>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
@@ -4653,11 +4653,11 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Property 33</t>
+          <t>CardProductPromo</t>
         </is>
       </c>
       <c r="D144" s="14" t="n">
-        <v>1058</v>
+        <v>200</v>
       </c>
     </row>
     <row r="145" ht="20" customHeight="1">
@@ -4673,11 +4673,11 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="D145" s="14" t="n">
-        <v>495</v>
+        <v>165</v>
       </c>
     </row>
     <row r="146" ht="20" customHeight="1">
@@ -4693,11 +4693,11 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Cotizar</t>
         </is>
       </c>
       <c r="D146" s="14" t="n">
-        <v>373</v>
+        <v>95</v>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
@@ -4713,11 +4713,11 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="D147" s="14" t="n">
-        <v>300</v>
+        <v>95</v>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>Close Icon</t>
         </is>
       </c>
       <c r="D148" s="14" t="n">
-        <v>270</v>
+        <v>88</v>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
@@ -4753,11 +4753,11 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Scroll</t>
         </is>
       </c>
       <c r="D149" s="14" t="n">
-        <v>264</v>
+        <v>73</v>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
@@ -4773,11 +4773,11 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>CardMenúMobile</t>
         </is>
       </c>
       <c r="D150" s="14" t="n">
-        <v>264</v>
+        <v>73</v>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
@@ -4793,11 +4793,11 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>CardProductPromo</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="D151" s="14" t="n">
-        <v>200</v>
+        <v>73</v>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
@@ -4813,11 +4813,11 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>CardMenú</t>
         </is>
       </c>
       <c r="D152" s="14" t="n">
-        <v>195</v>
+        <v>71</v>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D153" s="14" t="n">
-        <v>149</v>
+        <v>70</v>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
@@ -4853,11 +4853,11 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Cotizar</t>
+          <t>BotónCategoría</t>
         </is>
       </c>
       <c r="D154" s="14" t="n">
-        <v>105</v>
+        <v>69</v>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
@@ -4873,11 +4873,11 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>WithoutShieldHeart</t>
         </is>
       </c>
       <c r="D155" s="14" t="n">
-        <v>105</v>
+        <v>66</v>
       </c>
     </row>
     <row r="156" ht="20" customHeight="1">
@@ -4893,11 +4893,11 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Close Icon</t>
+          <t>ShieldHeart</t>
         </is>
       </c>
       <c r="D156" s="14" t="n">
-        <v>96</v>
+        <v>63</v>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
@@ -4913,11 +4913,11 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Scroll</t>
+          <t>Slider</t>
         </is>
       </c>
       <c r="D157" s="14" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Car</t>
         </is>
       </c>
       <c r="D158" s="14" t="n">
-        <v>77</v>
+        <v>47</v>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
@@ -4953,11 +4953,11 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>CardMenúMobile</t>
+          <t>_Link Icon</t>
         </is>
       </c>
       <c r="D159" s="14" t="n">
-        <v>73</v>
+        <v>45</v>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
@@ -4973,11 +4973,11 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="D160" s="14" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
@@ -4993,11 +4993,11 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>CardMenú</t>
+          <t>MedicalService</t>
         </is>
       </c>
       <c r="D161" s="14" t="n">
-        <v>71</v>
+        <v>45</v>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
@@ -5013,11 +5013,11 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D162" s="14" t="n">
-        <v>570</v>
+        <v>52</v>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Property 33</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D163" s="14" t="n">
-        <v>140</v>
+        <v>42</v>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
@@ -5053,11 +5053,11 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>icon</t>
         </is>
       </c>
       <c r="D164" s="14" t="n">
-        <v>90</v>
+        <v>24</v>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
@@ -5073,11 +5073,11 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>SecciónDescripción</t>
         </is>
       </c>
       <c r="D165" s="14" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
@@ -5093,11 +5093,11 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D166" s="14" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="167" ht="20" customHeight="1">
@@ -5113,11 +5113,11 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="D167" s="14" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
     </row>
     <row r="168" ht="20" customHeight="1">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>operador</t>
         </is>
       </c>
       <c r="D168" s="14" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1">
@@ -5153,11 +5153,11 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>compare_arrow</t>
+          <t>WithoutShieldHeart</t>
         </is>
       </c>
       <c r="D169" s="14" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
     </row>
     <row r="170" ht="20" customHeight="1">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>SeccionCanales</t>
         </is>
       </c>
       <c r="D170" s="14" t="n">
-        <v>42</v>
+        <v>12</v>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
@@ -5193,11 +5193,11 @@
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>PersonalInjuy</t>
         </is>
       </c>
       <c r="D171" s="14" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
@@ -5213,11 +5213,11 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>icon</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="D172" s="14" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>SecciónDescripción</t>
+          <t>LogosCollab</t>
         </is>
       </c>
       <c r="D173" s="14" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="174" ht="20" customHeight="1">
@@ -5253,11 +5253,11 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>CoberturasIconos</t>
         </is>
       </c>
       <c r="D174" s="14" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="175" ht="20" customHeight="1">
@@ -5273,11 +5273,11 @@
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Scroll</t>
         </is>
       </c>
       <c r="D175" s="14" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="176" ht="20" customHeight="1">
@@ -5293,11 +5293,11 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Complex</t>
         </is>
       </c>
       <c r="D176" s="14" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="177" ht="20" customHeight="1">
@@ -5313,11 +5313,11 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>operador</t>
+          <t>menu</t>
         </is>
       </c>
       <c r="D177" s="14" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="178" ht="20" customHeight="1">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>title_+_badges_download</t>
         </is>
       </c>
       <c r="D178" s="14" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179" ht="20" customHeight="1">
@@ -5353,11 +5353,11 @@
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Átomo mobile</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="D179" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
@@ -5373,11 +5373,11 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>SeccionCanales</t>
+          <t>tiktok</t>
         </is>
       </c>
       <c r="D180" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="181" ht="20" customHeight="1">
@@ -5393,11 +5393,11 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>PersonalInjuy</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="D181" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -5476,7 +5476,7 @@
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
@@ -5507,19 +5507,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>39%</t>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>64%</t>
         </is>
       </c>
       <c r="E3" s="6" t="n">
         <v>16</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>6110</v>
+        <v>10028</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>15743</v>
+        <v>15607</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -5538,19 +5538,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>19%</t>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>81%</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
         <v>6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>343</v>
+        <v>1422</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>1807</v>
+        <v>1759</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -5571,14 +5571,14 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2437</v>
+        <v>2680</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>7982</v>
@@ -5600,19 +5600,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>55%</t>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>62%</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
         <v>22</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>11902</v>
+        <v>13591</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>21833</v>
+        <v>21832</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -5631,19 +5631,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>13%</t>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>86%</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>25727</v>
+        <v>154195</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>205592</v>
+        <v>180198</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -5662,19 +5662,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>47%</t>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>74%</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
         <v>5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>6522</v>
+        <v>10174</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>13837</v>
+        <v>13717</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -5693,19 +5693,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>19%</t>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>66%</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1900</v>
+        <v>4743</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>10203</v>
+        <v>7155</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -5724,19 +5724,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>25%</t>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
         <v>12</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1215</v>
+        <v>3647</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4772</v>
+        <v>4614</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -5755,19 +5755,19 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>26%</t>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>3604</v>
+        <v>10104</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>13712</v>
+        <v>12804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-17 23:05 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -659,17 +659,17 @@
         <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>4743</v>
+        <v>7035</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2412</v>
+        <v>2896</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>66%</t>
+          <t>71%</t>
         </is>
       </c>
     </row>
@@ -688,13 +688,13 @@
         <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>154195</v>
+        <v>169195</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>26003</v>
+        <v>28141</v>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
@@ -804,13 +804,13 @@
         <v>3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10104</v>
+        <v>10619</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>2700</v>
+        <v>2826</v>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
@@ -857,17 +857,17 @@
         <v>24</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>210584</v>
+        <v>228391</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>55084</v>
+        <v>57832</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>80%</t>
         </is>
       </c>
     </row>
@@ -1197,20 +1197,20 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>3471</v>
+        <v>5763</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2137</v>
+        <v>2621</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>5608</v>
+        <v>8384</v>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>69%</t>
         </is>
       </c>
     </row>
@@ -1231,20 +1231,20 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0</v>
+        <v>2138</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>17138</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>88%</t>
         </is>
       </c>
     </row>
@@ -1639,16 +1639,16 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>4525</v>
+        <v>5041</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>1006</v>
+        <v>1132</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>5531</v>
+        <v>6173</v>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
@@ -1710,13 +1710,13 @@
         <v>14</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>267</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D42" s="14" t="n">
-        <v>520</v>
+        <v>640</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D43" s="14" t="n">
-        <v>130</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
@@ -2653,11 +2653,11 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D44" s="14" t="n">
-        <v>103</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
@@ -2673,11 +2673,11 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>HealthAndSafe</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="D45" s="14" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
@@ -2693,11 +2693,11 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Notification Item</t>
+          <t>HealthAndSafe</t>
         </is>
       </c>
       <c r="D46" s="14" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
@@ -2713,11 +2713,11 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>eye_close</t>
+          <t>Notification Item</t>
         </is>
       </c>
       <c r="D47" s="14" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>eye_close</t>
         </is>
       </c>
       <c r="D48" s="14" t="n">
-        <v>74</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
@@ -2753,11 +2753,11 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="D49" s="14" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
@@ -2773,11 +2773,11 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>menu</t>
         </is>
       </c>
       <c r="D50" s="14" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
@@ -2793,11 +2793,11 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D51" s="14" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
@@ -2813,11 +2813,11 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D52" s="14" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>menu</t>
+          <t>time</t>
         </is>
       </c>
       <c r="D53" s="14" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
@@ -2853,11 +2853,11 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Beneficio | card</t>
+          <t>Apps</t>
         </is>
       </c>
       <c r="D54" s="14" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Apps</t>
+          <t>Beneficio | card</t>
         </is>
       </c>
       <c r="D55" s="14" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
@@ -2893,11 +2893,11 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Beneficio | card mobile</t>
+          <t>Slider</t>
         </is>
       </c>
       <c r="D56" s="14" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
@@ -2913,11 +2913,11 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Slider</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="D57" s="14" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Beneficio | card mobile</t>
         </is>
       </c>
       <c r="D58" s="14" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
@@ -2953,11 +2953,11 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>generate ai</t>
+          <t>Banner | errores</t>
         </is>
       </c>
       <c r="D59" s="14" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
@@ -2973,11 +2973,11 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Atajos | Beneficios (new)</t>
+          <t>generate ai</t>
         </is>
       </c>
       <c r="D60" s="14" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
@@ -2993,11 +2993,11 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>download</t>
+          <t>account</t>
         </is>
       </c>
       <c r="D61" s="14" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="D62" s="14" t="n">
-        <v>4980</v>
+        <v>5595</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
@@ -3173,11 +3173,11 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="D70" s="14" t="n">
-        <v>697</v>
+        <v>769</v>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
@@ -3193,11 +3193,11 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>instagram</t>
+          <t>tiktok</t>
         </is>
       </c>
       <c r="D71" s="14" t="n">
-        <v>692</v>
+        <v>769</v>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
@@ -3213,11 +3213,11 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>tiktok</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="D72" s="14" t="n">
-        <v>692</v>
+        <v>769</v>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>youtube</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D73" s="14" t="n">
-        <v>692</v>
+        <v>697</v>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="D75" s="14" t="n">
-        <v>518</v>
+        <v>550</v>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="D76" s="14" t="n">
-        <v>514</v>
+        <v>523</v>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
@@ -4617,7 +4617,7 @@
         </is>
       </c>
       <c r="D142" s="14" t="n">
-        <v>280</v>
+        <v>304</v>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D143" s="14" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="D145" s="14" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="146" ht="20" customHeight="1">
@@ -4697,7 +4697,7 @@
         </is>
       </c>
       <c r="D146" s="14" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
@@ -4717,7 +4717,7 @@
         </is>
       </c>
       <c r="D147" s="14" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D148" s="14" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c r="D149" s="14" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
@@ -4773,11 +4773,11 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>CardMenúMobile</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D150" s="14" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
@@ -4793,7 +4793,7 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>CardMenúMobile</t>
         </is>
       </c>
       <c r="D151" s="14" t="n">
@@ -4813,11 +4813,11 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>CardMenú</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="D152" s="14" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>WithoutShieldHeart</t>
         </is>
       </c>
       <c r="D153" s="14" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
@@ -4853,11 +4853,11 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>BotónCategoría</t>
+          <t>CardMenú</t>
         </is>
       </c>
       <c r="D154" s="14" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
@@ -4873,11 +4873,11 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>ShieldHeart</t>
         </is>
       </c>
       <c r="D155" s="14" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="156" ht="20" customHeight="1">
@@ -4893,11 +4893,11 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>ShieldHeart</t>
+          <t>BotónCategoría</t>
         </is>
       </c>
       <c r="D156" s="14" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Car</t>
+          <t>_Link Icon</t>
         </is>
       </c>
       <c r="D158" s="14" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
@@ -4953,11 +4953,11 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>_Link Icon</t>
+          <t>_Button Icon</t>
         </is>
       </c>
       <c r="D159" s="14" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
@@ -4973,11 +4973,11 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Car</t>
         </is>
       </c>
       <c r="D160" s="14" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>MedicalService</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="D161" s="14" t="n">
@@ -5637,13 +5637,13 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>154195</v>
+        <v>169195</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>180198</v>
+        <v>197336</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -5695,17 +5695,17 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>66%</t>
+          <t>71%</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4743</v>
+        <v>7035</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>7155</v>
+        <v>9931</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -5761,13 +5761,13 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>10104</v>
+        <v>10619</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>12804</v>
+        <v>13445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-18 17:59 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -545,7 +545,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  Generado: 2026-06-17</t>
+          <t>Quarter: Q2 2026  |  Generado: 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -749,10 +749,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>13591</v>
+        <v>13615</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>8241</v>
+        <v>8209</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
@@ -775,13 +775,13 @@
         <v>6</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>10028</v>
+        <v>9789</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>5579</v>
+        <v>5487</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
@@ -804,17 +804,17 @@
         <v>3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>72</v>
+        <v>21</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10619</v>
+        <v>1842</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>2826</v>
+        <v>404</v>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -833,13 +833,13 @@
         <v>1</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1422</v>
+        <v>450</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>337</v>
+        <v>104</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -857,13 +857,13 @@
         <v>24</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>202</v>
+        <v>144</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>228391</v>
+        <v>218427</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>57832</v>
+        <v>55053</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
@@ -1404,17 +1404,17 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1749</v>
+        <v>1773</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>467</v>
+        <v>435</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>2216</v>
+        <v>2208</v>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>80%</t>
         </is>
       </c>
     </row>
@@ -1571,16 +1571,16 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>3359</v>
+        <v>3120</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>1423</v>
+        <v>1331</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>4782</v>
+        <v>4451</v>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
@@ -1639,16 +1639,16 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>5041</v>
+        <v>1842</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>1132</v>
+        <v>404</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>6173</v>
+        <v>2246</v>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
@@ -1673,20 +1673,20 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>4204</v>
+        <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>1427</v>
+        <v>0</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>5631</v>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>75%</t>
+        <v>0</v>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1707,20 +1707,20 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>1374</v>
+        <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>267</v>
+        <v>0</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>1641</v>
-      </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>84%</t>
+        <v>0</v>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1741,16 +1741,16 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>1422</v>
+        <v>450</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>337</v>
+        <v>104</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>1759</v>
+        <v>554</v>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="D111" s="14" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
@@ -4017,7 +4017,7 @@
         </is>
       </c>
       <c r="D112" s="14" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D113" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="114" ht="20" customHeight="1">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>billetera</t>
         </is>
       </c>
       <c r="D114" s="14" t="n">
@@ -4073,11 +4073,11 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>billetera</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D115" s="14" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="116" ht="20" customHeight="1">
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="D116" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="117" ht="20" customHeight="1">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="D117" s="14" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="118" ht="20" customHeight="1">
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="D122" s="14" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
     </row>
     <row r="123" ht="20" customHeight="1">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D123" s="14" t="n">
-        <v>352</v>
+        <v>336</v>
       </c>
     </row>
     <row r="124" ht="20" customHeight="1">
@@ -4293,11 +4293,11 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>02</t>
         </is>
       </c>
       <c r="D126" s="14" t="n">
-        <v>224</v>
+        <v>212</v>
       </c>
     </row>
     <row r="127" ht="20" customHeight="1">
@@ -4313,11 +4313,11 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D127" s="14" t="n">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
@@ -4373,11 +4373,11 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Toast</t>
         </is>
       </c>
       <c r="D130" s="14" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
@@ -4393,11 +4393,11 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Toast</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D131" s="14" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D133" s="14" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="134" ht="20" customHeight="1">
@@ -4453,11 +4453,11 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Indicator Mobile</t>
         </is>
       </c>
       <c r="D134" s="14" t="n">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
@@ -4473,11 +4473,11 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Indicator Mobile</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="D135" s="14" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1">
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="D136" s="14" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="137" ht="20" customHeight="1">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Infotip</t>
+          <t>torito</t>
         </is>
       </c>
       <c r="D138" s="14" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="139" ht="20" customHeight="1">
@@ -4553,11 +4553,11 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Component 120</t>
+          <t>Infotip</t>
         </is>
       </c>
       <c r="D139" s="14" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
@@ -4573,11 +4573,11 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Smile</t>
+          <t>Component 120</t>
         </is>
       </c>
       <c r="D140" s="14" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>directionLeft</t>
+          <t>Smile</t>
         </is>
       </c>
       <c r="D141" s="14" t="n">
@@ -4617,7 +4617,7 @@
         </is>
       </c>
       <c r="D142" s="14" t="n">
-        <v>304</v>
+        <v>78</v>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Cotizar</t>
         </is>
       </c>
       <c r="D143" s="14" t="n">
-        <v>217</v>
+        <v>30</v>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
@@ -4653,11 +4653,11 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>CardProductPromo</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="D144" s="14" t="n">
-        <v>200</v>
+        <v>30</v>
       </c>
     </row>
     <row r="145" ht="20" customHeight="1">
@@ -4673,11 +4673,11 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="D145" s="14" t="n">
-        <v>167</v>
+        <v>28</v>
       </c>
     </row>
     <row r="146" ht="20" customHeight="1">
@@ -4693,11 +4693,11 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Cotizar</t>
+          <t>Close Icon</t>
         </is>
       </c>
       <c r="D146" s="14" t="n">
-        <v>105</v>
+        <v>22</v>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
@@ -4713,11 +4713,11 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Scroll</t>
         </is>
       </c>
       <c r="D147" s="14" t="n">
-        <v>105</v>
+        <v>19</v>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Close Icon</t>
+          <t>_Link Icon</t>
         </is>
       </c>
       <c r="D148" s="14" t="n">
-        <v>96</v>
+        <v>18</v>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
@@ -4753,11 +4753,11 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Scroll</t>
+          <t>_Button Icon</t>
         </is>
       </c>
       <c r="D149" s="14" t="n">
-        <v>80</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
@@ -4773,11 +4773,11 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>submenu</t>
         </is>
       </c>
       <c r="D150" s="14" t="n">
-        <v>77</v>
+        <v>16</v>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
@@ -4793,11 +4793,11 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>CardMenúMobile</t>
+          <t>ShieldHeart</t>
         </is>
       </c>
       <c r="D151" s="14" t="n">
-        <v>73</v>
+        <v>15</v>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
@@ -4813,11 +4813,11 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>WithoutShieldHeart</t>
         </is>
       </c>
       <c r="D152" s="14" t="n">
-        <v>73</v>
+        <v>15</v>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>Link Stamp</t>
         </is>
       </c>
       <c r="D153" s="14" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
@@ -4853,11 +4853,11 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>CardMenú</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D154" s="14" t="n">
-        <v>71</v>
+        <v>8</v>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
@@ -4873,11 +4873,11 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>ShieldHeart</t>
+          <t>link</t>
         </is>
       </c>
       <c r="D155" s="14" t="n">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="156" ht="20" customHeight="1">
@@ -4893,11 +4893,11 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>BotónCategoría</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="D156" s="14" t="n">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
@@ -4913,11 +4913,11 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Slider</t>
+          <t>Link Details</t>
         </is>
       </c>
       <c r="D157" s="14" t="n">
-        <v>62</v>
+        <v>6</v>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>_Link Icon</t>
+          <t>account</t>
         </is>
       </c>
       <c r="D158" s="14" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
@@ -4953,11 +4953,11 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>_Button Icon</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="D159" s="14" t="n">
-        <v>49</v>
+        <v>6</v>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
@@ -4973,11 +4973,11 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Car</t>
+          <t>support</t>
         </is>
       </c>
       <c r="D160" s="14" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
@@ -4993,11 +4993,11 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D161" s="14" t="n">
-        <v>45</v>
+        <v>6</v>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="D162" s="14" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D163" s="14" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="D164" s="14" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
@@ -5073,11 +5073,11 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>SecciónDescripción</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D165" s="14" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
@@ -5093,11 +5093,11 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="D166" s="14" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="167" ht="20" customHeight="1">
@@ -5113,11 +5113,11 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>SecciónDescripción</t>
         </is>
       </c>
       <c r="D167" s="14" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="168" ht="20" customHeight="1">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>operador</t>
+          <t>LogosCollab</t>
         </is>
       </c>
       <c r="D168" s="14" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1">
@@ -5153,11 +5153,11 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>SeccionCanales</t>
         </is>
       </c>
       <c r="D169" s="14" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="170" ht="20" customHeight="1">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>SeccionCanales</t>
+          <t>WithoutShieldHeart</t>
         </is>
       </c>
       <c r="D170" s="14" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
@@ -5197,7 +5197,7 @@
         </is>
       </c>
       <c r="D171" s="14" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
@@ -5213,11 +5213,11 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>problema eléctrico</t>
         </is>
       </c>
       <c r="D172" s="14" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>LogosCollab</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="D173" s="14" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="174" ht="20" customHeight="1">
@@ -5253,11 +5253,11 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>CoberturasIconos</t>
+          <t>Complex</t>
         </is>
       </c>
       <c r="D174" s="14" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="175" ht="20" customHeight="1">
@@ -5273,11 +5273,11 @@
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Scroll</t>
+          <t>menu</t>
         </is>
       </c>
       <c r="D175" s="14" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176" ht="20" customHeight="1">
@@ -5293,11 +5293,11 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Complex</t>
+          <t>robo de autopartes</t>
         </is>
       </c>
       <c r="D176" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177" ht="20" customHeight="1">
@@ -5313,11 +5313,11 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>menu</t>
+          <t>operador</t>
         </is>
       </c>
       <c r="D177" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178" ht="20" customHeight="1">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>title_+_badges_download</t>
+          <t>CoberturasIconos</t>
         </is>
       </c>
       <c r="D178" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="179" ht="20" customHeight="1">
@@ -5353,11 +5353,11 @@
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>instagram</t>
+          <t>Scroll</t>
         </is>
       </c>
       <c r="D179" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
@@ -5373,11 +5373,11 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>tiktok</t>
+          <t>title_+_badges_download</t>
         </is>
       </c>
       <c r="D180" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="181" ht="20" customHeight="1">
@@ -5393,11 +5393,11 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>youtube</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="D181" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
@@ -5513,13 +5513,13 @@
         </is>
       </c>
       <c r="E3" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>10028</v>
+        <v>9789</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>15607</v>
+        <v>15276</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -5544,13 +5544,13 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1422</v>
+        <v>450</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>1759</v>
+        <v>554</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -5597,7 +5597,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -5609,10 +5609,10 @@
         <v>22</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>13591</v>
+        <v>13615</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>21832</v>
+        <v>21824</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -5752,22 +5752,22 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>72</v>
+        <v>21</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>10619</v>
+        <v>1842</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>13445</v>
+        <v>2246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-18 21:27 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -768,104 +768,249 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>9789</v>
+        <v>1508</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>5487</v>
+        <v>679</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>64%</t>
+          <t>69%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1842</v>
+        <v>2007</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>404</v>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>82%</t>
+        <v>1266</v>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>61%</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>825</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>469</v>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="7" t="n">
-        <v>450</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>104</v>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="E14" s="7" t="n">
+        <v>2329</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>1742</v>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>3120</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>1331</v>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>3684</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>10823</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>2882</v>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>1422</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>337</v>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>81%</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C19" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="D14" s="11" t="n">
-        <v>144</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>218427</v>
-      </c>
-      <c r="F14" s="11" t="n">
-        <v>55053</v>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="D19" s="11" t="n">
+        <v>207</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>232064</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>58961</v>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
         <is>
           <t>80%</t>
         </is>
@@ -873,9 +1018,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A19:B19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1426,7 +1571,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1460,7 +1605,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1494,7 +1639,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1528,7 +1673,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1562,7 +1707,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1596,7 +1741,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1605,20 +1750,20 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0</v>
+        <v>3684</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0</v>
+        <v>1197</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>4881</v>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1639,16 +1784,16 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>1842</v>
+        <v>5041</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>404</v>
+        <v>1132</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>2246</v>
+        <v>6173</v>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
@@ -1673,20 +1818,20 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0</v>
+        <v>4389</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0</v>
+        <v>1477</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>5866</v>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1707,20 +1852,20 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>0</v>
+        <v>1393</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>0</v>
+        <v>273</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>1666</v>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>84%</t>
         </is>
       </c>
     </row>
@@ -1741,16 +1886,16 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>450</v>
+        <v>1422</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>104</v>
+        <v>337</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>554</v>
+        <v>1759</v>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
@@ -1769,7 +1914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4208,16 +4353,16 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>01</t>
         </is>
       </c>
       <c r="D122" s="14" t="n">
-        <v>340</v>
+        <v>41</v>
       </c>
     </row>
     <row r="123" ht="20" customHeight="1">
@@ -4228,7 +4373,7 @@
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
@@ -4237,7 +4382,7 @@
         </is>
       </c>
       <c r="D123" s="14" t="n">
-        <v>336</v>
+        <v>36</v>
       </c>
     </row>
     <row r="124" ht="20" customHeight="1">
@@ -4248,16 +4393,16 @@
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>celda</t>
+          <t>Indicator Mobile</t>
         </is>
       </c>
       <c r="D124" s="14" t="n">
-        <v>312</v>
+        <v>31</v>
       </c>
     </row>
     <row r="125" ht="20" customHeight="1">
@@ -4268,16 +4413,16 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>torito</t>
         </is>
       </c>
       <c r="D125" s="14" t="n">
-        <v>248</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" ht="20" customHeight="1">
@@ -4288,16 +4433,16 @@
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>Infotip</t>
         </is>
       </c>
       <c r="D126" s="14" t="n">
-        <v>212</v>
+        <v>29</v>
       </c>
     </row>
     <row r="127" ht="20" customHeight="1">
@@ -4308,16 +4453,16 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>number_deskop</t>
         </is>
       </c>
       <c r="D127" s="14" t="n">
-        <v>210</v>
+        <v>24</v>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
@@ -4328,16 +4473,16 @@
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>add</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D128" s="14" t="n">
-        <v>159</v>
+        <v>23</v>
       </c>
     </row>
     <row r="129" ht="20" customHeight="1">
@@ -4348,16 +4493,16 @@
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D129" s="14" t="n">
-        <v>139</v>
+        <v>21</v>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
@@ -4368,16 +4513,16 @@
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Toast</t>
+          <t>eye_open</t>
         </is>
       </c>
       <c r="D130" s="14" t="n">
-        <v>118</v>
+        <v>18</v>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
@@ -4388,16 +4533,16 @@
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Step 01</t>
         </is>
       </c>
       <c r="D131" s="14" t="n">
-        <v>109</v>
+        <v>17</v>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
@@ -4408,16 +4553,16 @@
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Step 02</t>
         </is>
       </c>
       <c r="D132" s="14" t="n">
-        <v>105</v>
+        <v>17</v>
       </c>
     </row>
     <row r="133" ht="20" customHeight="1">
@@ -4428,16 +4573,16 @@
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>Step 03</t>
         </is>
       </c>
       <c r="D133" s="14" t="n">
-        <v>102</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134" ht="20" customHeight="1">
@@ -4448,16 +4593,16 @@
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Indicator Mobile</t>
+          <t>shield</t>
         </is>
       </c>
       <c r="D134" s="14" t="n">
-        <v>86</v>
+        <v>16</v>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
@@ -4468,16 +4613,16 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>tarjeta de crédito</t>
         </is>
       </c>
       <c r="D135" s="14" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1">
@@ -4488,16 +4633,16 @@
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>Póliza Salud</t>
         </is>
       </c>
       <c r="D136" s="14" t="n">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="137" ht="20" customHeight="1">
@@ -4508,16 +4653,16 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="D137" s="14" t="n">
-        <v>78</v>
+        <v>14</v>
       </c>
     </row>
     <row r="138" ht="20" customHeight="1">
@@ -4528,16 +4673,16 @@
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>torito</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="D138" s="14" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
     </row>
     <row r="139" ht="20" customHeight="1">
@@ -4548,16 +4693,16 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Infotip</t>
+          <t>call</t>
         </is>
       </c>
       <c r="D139" s="14" t="n">
-        <v>57</v>
+        <v>13</v>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
@@ -4568,16 +4713,16 @@
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Component 120</t>
+          <t>Toast</t>
         </is>
       </c>
       <c r="D140" s="14" t="n">
-        <v>56</v>
+        <v>12</v>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
@@ -4588,687 +4733,687 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Smile</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="D141" s="14" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="D142" s="14" t="n">
-        <v>78</v>
+        <v>149</v>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Cotizar</t>
+          <t>02</t>
         </is>
       </c>
       <c r="D143" s="14" t="n">
-        <v>30</v>
+        <v>105</v>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="D144" s="14" t="n">
-        <v>30</v>
+        <v>102</v>
       </c>
     </row>
     <row r="145" ht="20" customHeight="1">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>01</t>
         </is>
       </c>
       <c r="D145" s="14" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
     </row>
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Close Icon</t>
+          <t>add</t>
         </is>
       </c>
       <c r="D146" s="14" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Scroll</t>
+          <t>call</t>
         </is>
       </c>
       <c r="D147" s="14" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>_Link Icon</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="D148" s="14" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>_Button Icon</t>
+          <t>grid view</t>
         </is>
       </c>
       <c r="D149" s="14" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>submenu</t>
+          <t>Toast</t>
         </is>
       </c>
       <c r="D150" s="14" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>ShieldHeart</t>
+          <t>Infotip</t>
         </is>
       </c>
       <c r="D151" s="14" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>Smile</t>
         </is>
       </c>
       <c r="D152" s="14" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Link Stamp</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="D153" s="14" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="D154" s="14" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D155" s="14" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="156" ht="20" customHeight="1">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>eye_open</t>
         </is>
       </c>
       <c r="D156" s="14" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Link Details</t>
+          <t>torito</t>
         </is>
       </c>
       <c r="D157" s="14" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>account</t>
+          <t>tarjeta de crédito</t>
         </is>
       </c>
       <c r="D158" s="14" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>asset_promo</t>
         </is>
       </c>
       <c r="D159" s="14" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>Indicator Mobile</t>
         </is>
       </c>
       <c r="D160" s="14" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>download</t>
+          <t>Image Frame</t>
         </is>
       </c>
       <c r="D161" s="14" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>grid view</t>
+          <t>Slider Controls Glass</t>
         </is>
       </c>
       <c r="D162" s="14" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="D163" s="14" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>icon</t>
+          <t>Spinner</t>
         </is>
       </c>
       <c r="D164" s="14" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>icon</t>
         </is>
       </c>
       <c r="D165" s="14" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Caja formulario complex L M</t>
         </is>
       </c>
       <c r="D166" s="14" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="167" ht="20" customHeight="1">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>SecciónDescripción</t>
+          <t>Contenido desktop</t>
         </is>
       </c>
       <c r="D167" s="14" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>LogosCollab</t>
+          <t>Formulario L M complex</t>
         </is>
       </c>
       <c r="D168" s="14" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>SeccionCanales</t>
+          <t>Banner mobile</t>
         </is>
       </c>
       <c r="D169" s="14" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="170" ht="20" customHeight="1">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="D170" s="14" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>PersonalInjuy</t>
+          <t>Slider</t>
         </is>
       </c>
       <c r="D171" s="14" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>problema eléctrico</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="D172" s="14" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Contenido mobile</t>
         </is>
       </c>
       <c r="D173" s="14" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="174" ht="20" customHeight="1">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Complex</t>
+          <t>security</t>
         </is>
       </c>
       <c r="D174" s="14" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -5277,127 +5422,2127 @@
         </is>
       </c>
       <c r="D175" s="14" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>robo de autopartes</t>
+          <t>Complex</t>
         </is>
       </c>
       <c r="D176" s="14" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="177" ht="20" customHeight="1">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>operador</t>
+          <t>CajaFormulario</t>
         </is>
       </c>
       <c r="D177" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>CoberturasIconos</t>
+          <t>Carousel</t>
         </is>
       </c>
       <c r="D178" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Scroll</t>
+          <t>Card_Mobile_funciona 1</t>
         </is>
       </c>
       <c r="D179" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>title_+_badges_download</t>
+          <t>Card_Mobile_funciona 3</t>
         </is>
       </c>
       <c r="D180" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181" ht="20" customHeight="1">
       <c r="A181" s="4" t="inlineStr">
         <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>Auto Efectivo</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t>Card_Mobile_funciona 4</t>
+        </is>
+      </c>
+      <c r="D181" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="182" ht="20" customHeight="1">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t>grid view</t>
+        </is>
+      </c>
+      <c r="D182" s="14" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="183" ht="20" customHeight="1">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C183" s="4" t="inlineStr">
+        <is>
+          <t>Discount Badge</t>
+        </is>
+      </c>
+      <c r="D183" s="14" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="184" ht="20" customHeight="1">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>Slider Controls</t>
+        </is>
+      </c>
+      <c r="D184" s="14" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="A185" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C185" s="4" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="D185" s="14" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D186" s="14" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D187" s="14" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="188" ht="20" customHeight="1">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+      <c r="D188" s="14" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="189" ht="20" customHeight="1">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="D189" s="14" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D190" s="14" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="191" ht="20" customHeight="1">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>Smile</t>
+        </is>
+      </c>
+      <c r="D191" s="14" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="192" ht="20" customHeight="1">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="D192" s="14" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="193" ht="20" customHeight="1">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr">
+        <is>
+          <t>hoist</t>
+        </is>
+      </c>
+      <c r="D193" s="14" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="194" ht="20" customHeight="1">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>Indicator Mobile</t>
+        </is>
+      </c>
+      <c r="D194" s="14" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="195" ht="20" customHeight="1">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>emergency</t>
+        </is>
+      </c>
+      <c r="D195" s="14" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="196" ht="20" customHeight="1">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t>Commercial Chips</t>
+        </is>
+      </c>
+      <c r="D196" s="14" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="197" ht="20" customHeight="1">
+      <c r="A197" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C197" s="4" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="D197" s="14" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="198" ht="20" customHeight="1">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>call</t>
+        </is>
+      </c>
+      <c r="D198" s="14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="199" ht="20" customHeight="1">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>Step 01</t>
+        </is>
+      </c>
+      <c r="D199" s="14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="200" ht="20" customHeight="1">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>Step 02</t>
+        </is>
+      </c>
+      <c r="D200" s="14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="201" ht="20" customHeight="1">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>Step 03</t>
+        </is>
+      </c>
+      <c r="D201" s="14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="202" ht="20" customHeight="1">
+      <c r="A202" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C202" s="4" t="inlineStr">
+        <is>
+          <t>Menu Item</t>
+        </is>
+      </c>
+      <c r="D202" s="14" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="203" ht="20" customHeight="1">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>celda</t>
+        </is>
+      </c>
+      <c r="D203" s="14" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="204" ht="20" customHeight="1">
+      <c r="A204" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C204" s="4" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="D204" s="14" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="205" ht="20" customHeight="1">
+      <c r="A205" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C205" s="4" t="inlineStr">
+        <is>
+          <t>Menu title</t>
+        </is>
+      </c>
+      <c r="D205" s="14" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="206" ht="20" customHeight="1">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C206" s="4" t="inlineStr">
+        <is>
+          <t>Component 120</t>
+        </is>
+      </c>
+      <c r="D206" s="14" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="207" ht="20" customHeight="1">
+      <c r="A207" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C207" s="4" t="inlineStr">
+        <is>
+          <t>directionLeft</t>
+        </is>
+      </c>
+      <c r="D207" s="14" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="208" ht="20" customHeight="1">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>call</t>
+        </is>
+      </c>
+      <c r="D208" s="14" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="209" ht="20" customHeight="1">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="D209" s="14" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="210" ht="20" customHeight="1">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>Star</t>
+        </is>
+      </c>
+      <c r="D210" s="14" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="211" ht="20" customHeight="1">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>Topbar</t>
+        </is>
+      </c>
+      <c r="D211" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="212" ht="20" customHeight="1">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="D212" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="213" ht="20" customHeight="1">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="D213" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="214" ht="20" customHeight="1">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>youtube</t>
+        </is>
+      </c>
+      <c r="D214" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="215" ht="20" customHeight="1">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>LocationPin</t>
+        </is>
+      </c>
+      <c r="D215" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="216" ht="20" customHeight="1">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C216" s="4" t="inlineStr">
+        <is>
+          <t>Indicator Mobile</t>
+        </is>
+      </c>
+      <c r="D216" s="14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="217" ht="20" customHeight="1">
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B217" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C217" s="4" t="inlineStr">
+        <is>
+          <t>Step 01</t>
+        </is>
+      </c>
+      <c r="D217" s="14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="218" ht="20" customHeight="1">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>Bar Progress</t>
+        </is>
+      </c>
+      <c r="D218" s="14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="219" ht="20" customHeight="1">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C219" s="4" t="inlineStr">
+        <is>
+          <t>Step 02</t>
+        </is>
+      </c>
+      <c r="D219" s="14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="220" ht="20" customHeight="1">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>torito</t>
+        </is>
+      </c>
+      <c r="D220" s="14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="221" ht="20" customHeight="1">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="D221" s="14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="222" ht="20" customHeight="1">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="D222" s="14" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="223" ht="20" customHeight="1">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>Slider Controls</t>
+        </is>
+      </c>
+      <c r="D223" s="14" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="224" ht="20" customHeight="1">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="D224" s="14" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="225" ht="20" customHeight="1">
+      <c r="A225" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B225" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C225" s="4" t="inlineStr">
+        <is>
+          <t>Menu Item</t>
+        </is>
+      </c>
+      <c r="D225" s="14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="226" ht="20" customHeight="1">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>01 Info</t>
+        </is>
+      </c>
+      <c r="D226" s="14" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="227" ht="20" customHeight="1">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t>ArrowLeft</t>
+        </is>
+      </c>
+      <c r="D227" s="14" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="228" ht="20" customHeight="1">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="D228" s="14" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="229" ht="20" customHeight="1">
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="D229" s="14" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="230" ht="20" customHeight="1">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="D230" s="14" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="231" ht="20" customHeight="1">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t>menu</t>
+        </is>
+      </c>
+      <c r="D231" s="14" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="232" ht="20" customHeight="1">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>Chip Deleteable</t>
+        </is>
+      </c>
+      <c r="D232" s="14" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="233" ht="20" customHeight="1">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>correo electronico</t>
+        </is>
+      </c>
+      <c r="D233" s="14" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="234" ht="20" customHeight="1">
+      <c r="A234" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>Menu title</t>
+        </is>
+      </c>
+      <c r="D234" s="14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="235" ht="20" customHeight="1">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>addcircle</t>
+        </is>
+      </c>
+      <c r="D235" s="14" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="236" ht="20" customHeight="1">
+      <c r="A236" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B236" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C236" s="4" t="inlineStr">
+        <is>
+          <t>call</t>
+        </is>
+      </c>
+      <c r="D236" s="14" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="237" ht="20" customHeight="1">
+      <c r="A237" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B237" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>payments</t>
+        </is>
+      </c>
+      <c r="D237" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="238" ht="20" customHeight="1">
+      <c r="A238" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B238" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C238" s="4" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="D238" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="239" ht="20" customHeight="1">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr">
+        <is>
+          <t>generando ia</t>
+        </is>
+      </c>
+      <c r="D239" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="240" ht="20" customHeight="1">
+      <c r="A240" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C240" s="4" t="inlineStr">
+        <is>
+          <t>creditcard</t>
+        </is>
+      </c>
+      <c r="D240" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="241" ht="20" customHeight="1">
+      <c r="A241" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="C241" s="4" t="inlineStr">
+        <is>
+          <t>A.white</t>
+        </is>
+      </c>
+      <c r="D241" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="242" ht="20" customHeight="1">
+      <c r="A242" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C242" s="4" t="inlineStr">
+        <is>
+          <t>grid view</t>
+        </is>
+      </c>
+      <c r="D242" s="14" t="n">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="243" ht="20" customHeight="1">
+      <c r="A243" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B243" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C243" s="4" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D243" s="14" t="n">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="244" ht="20" customHeight="1">
+      <c r="A244" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C244" s="4" t="inlineStr">
+        <is>
+          <t>CardProductPromo</t>
+        </is>
+      </c>
+      <c r="D244" s="14" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="245" ht="20" customHeight="1">
+      <c r="A245" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr">
+        <is>
+          <t>Slider Controls</t>
+        </is>
+      </c>
+      <c r="D245" s="14" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="246" ht="20" customHeight="1">
+      <c r="A246" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C246" s="4" t="inlineStr">
+        <is>
+          <t>Cotizar</t>
+        </is>
+      </c>
+      <c r="D246" s="14" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="247" ht="20" customHeight="1">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B247" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="D247" s="14" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="248" ht="20" customHeight="1">
+      <c r="A248" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C248" s="4" t="inlineStr">
+        <is>
+          <t>Close Icon</t>
+        </is>
+      </c>
+      <c r="D248" s="14" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="249" ht="20" customHeight="1">
+      <c r="A249" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr">
+        <is>
+          <t>Scroll</t>
+        </is>
+      </c>
+      <c r="D249" s="14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="250" ht="20" customHeight="1">
+      <c r="A250" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr">
+        <is>
+          <t>CardMenúMobile</t>
+        </is>
+      </c>
+      <c r="D250" s="14" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="251" ht="20" customHeight="1">
+      <c r="A251" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B251" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C251" s="4" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="D251" s="14" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="252" ht="20" customHeight="1">
+      <c r="A252" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C252" s="4" t="inlineStr">
+        <is>
+          <t>CardMenú</t>
+        </is>
+      </c>
+      <c r="D252" s="14" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="253" ht="20" customHeight="1">
+      <c r="A253" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B253" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C253" s="4" t="inlineStr">
+        <is>
+          <t>Status Control</t>
+        </is>
+      </c>
+      <c r="D253" s="14" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="254" ht="20" customHeight="1">
+      <c r="A254" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C254" s="4" t="inlineStr">
+        <is>
+          <t>WithoutShieldHeart</t>
+        </is>
+      </c>
+      <c r="D254" s="14" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="255" ht="20" customHeight="1">
+      <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="inlineStr">
+        <is>
+          <t>ShieldHeart</t>
+        </is>
+      </c>
+      <c r="D255" s="14" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="256" ht="20" customHeight="1">
+      <c r="A256" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B256" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C256" s="4" t="inlineStr">
+        <is>
+          <t>BotónCategoría</t>
+        </is>
+      </c>
+      <c r="D256" s="14" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="257" ht="20" customHeight="1">
+      <c r="A257" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>Slider</t>
+        </is>
+      </c>
+      <c r="D257" s="14" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="258" ht="20" customHeight="1">
+      <c r="A258" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C258" s="4" t="inlineStr">
+        <is>
+          <t>_Link Icon</t>
+        </is>
+      </c>
+      <c r="D258" s="14" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="259" ht="20" customHeight="1">
+      <c r="A259" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B259" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C259" s="4" t="inlineStr">
+        <is>
+          <t>_Button Icon</t>
+        </is>
+      </c>
+      <c r="D259" s="14" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="260" ht="20" customHeight="1">
+      <c r="A260" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B260" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C260" s="4" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="D260" s="14" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="261" ht="20" customHeight="1">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="D261" s="14" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="262" ht="20" customHeight="1">
+      <c r="A262" s="4" t="inlineStr">
+        <is>
           <t>Embebidos</t>
         </is>
       </c>
-      <c r="B181" s="4" t="inlineStr">
+      <c r="B262" s="4" t="inlineStr">
         <is>
           <t>Embebidos</t>
         </is>
       </c>
-      <c r="C181" s="4" t="inlineStr">
+      <c r="C262" s="4" t="inlineStr">
+        <is>
+          <t>grid view</t>
+        </is>
+      </c>
+      <c r="D262" s="14" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="263" ht="20" customHeight="1">
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B263" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C263" s="4" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="D263" s="14" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="264" ht="20" customHeight="1">
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>icon</t>
+        </is>
+      </c>
+      <c r="D264" s="14" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="265" ht="20" customHeight="1">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>SecciónDescripción</t>
+        </is>
+      </c>
+      <c r="D265" s="14" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="266" ht="20" customHeight="1">
+      <c r="A266" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D266" s="14" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="267" ht="20" customHeight="1">
+      <c r="A267" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C267" s="4" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D267" s="14" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="268" ht="20" customHeight="1">
+      <c r="A268" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B268" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>operador</t>
+        </is>
+      </c>
+      <c r="D268" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="269" ht="20" customHeight="1">
+      <c r="A269" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C269" s="4" t="inlineStr">
+        <is>
+          <t>WithoutShieldHeart</t>
+        </is>
+      </c>
+      <c r="D269" s="14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="270" ht="20" customHeight="1">
+      <c r="A270" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B270" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C270" s="4" t="inlineStr">
+        <is>
+          <t>SeccionCanales</t>
+        </is>
+      </c>
+      <c r="D270" s="14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="271" ht="20" customHeight="1">
+      <c r="A271" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C271" s="4" t="inlineStr">
+        <is>
+          <t>PersonalInjuy</t>
+        </is>
+      </c>
+      <c r="D271" s="14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="272" ht="20" customHeight="1">
+      <c r="A272" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B272" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="D272" s="14" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="273" ht="20" customHeight="1">
+      <c r="A273" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C273" s="4" t="inlineStr">
+        <is>
+          <t>LogosCollab</t>
+        </is>
+      </c>
+      <c r="D273" s="14" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="274" ht="20" customHeight="1">
+      <c r="A274" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C274" s="4" t="inlineStr">
+        <is>
+          <t>CoberturasIconos</t>
+        </is>
+      </c>
+      <c r="D274" s="14" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="275" ht="20" customHeight="1">
+      <c r="A275" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C275" s="4" t="inlineStr">
+        <is>
+          <t>Scroll</t>
+        </is>
+      </c>
+      <c r="D275" s="14" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="276" ht="20" customHeight="1">
+      <c r="A276" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B276" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C276" s="4" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="D276" s="14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="277" ht="20" customHeight="1">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="inlineStr">
+        <is>
+          <t>menu</t>
+        </is>
+      </c>
+      <c r="D277" s="14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="278" ht="20" customHeight="1">
+      <c r="A278" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B278" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
+        <is>
+          <t>title_+_badges_download</t>
+        </is>
+      </c>
+      <c r="D278" s="14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="279" ht="20" customHeight="1">
+      <c r="A279" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C279" s="4" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="D181" s="14" t="n">
-        <v>2</v>
+      <c r="D279" s="14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="280" ht="20" customHeight="1">
+      <c r="A280" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="D280" s="14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="281" ht="20" customHeight="1">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr">
+        <is>
+          <t>youtube</t>
+        </is>
+      </c>
+      <c r="D281" s="14" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -5411,7 +7556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5473,19 +7618,19 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>64%</t>
         </is>
       </c>
       <c r="E2" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>645</v>
+        <v>825</v>
       </c>
       <c r="G2" s="6" t="n">
         <v>1294</v>
@@ -5544,13 +7689,13 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>450</v>
+        <v>1422</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>554</v>
+        <v>1759</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -5711,7 +7856,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Somos Corredores</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -5724,50 +7869,205 @@
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>79%</t>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>69%</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>3647</v>
+        <v>1508</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4614</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Somos Corredores</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>3647</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>4614</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>3684</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>4881</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2007</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>3273</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>2329</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>4071</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>3120</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>4451</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>Web Corporativa</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Q2 2026</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>82%</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>1842</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>2246</v>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>79%</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>10823</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>13705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-18 23:24 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -952,7 +952,7 @@
         <v>72</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>10823</v>
+        <v>10822</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>2882</v>
@@ -1005,7 +1005,7 @@
         <v>207</v>
       </c>
       <c r="E19" s="12" t="n">
-        <v>232064</v>
+        <v>232063</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>58961</v>
@@ -1821,13 +1821,13 @@
         <v>3</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>4389</v>
+        <v>4388</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>1477</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>5866</v>
+        <v>5865</v>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
@@ -8064,10 +8064,10 @@
         <v>72</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>10823</v>
+        <v>10822</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>13705</v>
+        <v>13704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-19 14:46 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -725,10 +725,10 @@
         <v>5</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>10368</v>
+        <v>10633</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2842</v>
+        <v>2951</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>34</v>
@@ -757,10 +757,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>13859</v>
+        <v>13997</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7467</v>
+        <v>7557</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -1457,10 +1457,10 @@
         <v>5</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10368</v>
+        <v>10633</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>2842</v>
+        <v>2951</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>34</v>
@@ -1559,17 +1559,17 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1801</v>
+        <v>1939</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>358</v>
+        <v>448</v>
       </c>
       <c r="G15" s="8" t="n">
         <v>27</v>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>81%</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E217" s="7" t="n">
-        <v>1495</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="218">
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="E219" s="7" t="n">
-        <v>1333</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="220">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="E220" s="7" t="n">
-        <v>1282</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="221">
@@ -7458,7 +7458,7 @@
         </is>
       </c>
       <c r="E221" s="7" t="n">
-        <v>774</v>
+        <v>804</v>
       </c>
     </row>
     <row r="222">
@@ -7483,7 +7483,7 @@
         </is>
       </c>
       <c r="E222" s="7" t="n">
-        <v>579</v>
+        <v>608</v>
       </c>
     </row>
     <row r="223">
@@ -7508,7 +7508,7 @@
         </is>
       </c>
       <c r="E223" s="7" t="n">
-        <v>431</v>
+        <v>441</v>
       </c>
     </row>
     <row r="224">
@@ -7533,7 +7533,7 @@
         </is>
       </c>
       <c r="E224" s="7" t="n">
-        <v>401</v>
+        <v>414</v>
       </c>
     </row>
     <row r="225">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="E225" s="7" t="n">
-        <v>306</v>
+        <v>316</v>
       </c>
     </row>
     <row r="226">
@@ -7604,11 +7604,11 @@
       </c>
       <c r="D227" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E227" s="7" t="n">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="228">
@@ -7633,7 +7633,7 @@
         </is>
       </c>
       <c r="E228" s="7" t="n">
-        <v>236</v>
+        <v>246</v>
       </c>
     </row>
     <row r="229">
@@ -7654,11 +7654,11 @@
       </c>
       <c r="D229" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E229" s="7" t="n">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="230">
@@ -7683,7 +7683,7 @@
         </is>
       </c>
       <c r="E230" s="7" t="n">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="231">
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="E231" s="7" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="232">
@@ -7808,7 +7808,7 @@
         </is>
       </c>
       <c r="E235" s="7" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="236">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E237" s="7" t="n">
@@ -7879,11 +7879,11 @@
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E238" s="7" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="239">
@@ -9583,7 +9583,7 @@
         </is>
       </c>
       <c r="E306" s="7" t="n">
-        <v>1216</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="307">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="E307" s="7" t="n">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="308">
@@ -9633,7 +9633,7 @@
         </is>
       </c>
       <c r="E308" s="7" t="n">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="309">
@@ -9658,7 +9658,7 @@
         </is>
       </c>
       <c r="E309" s="7" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="310">
@@ -9683,7 +9683,7 @@
         </is>
       </c>
       <c r="E310" s="7" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="311">
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="E312" s="7" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="313">
@@ -9754,11 +9754,11 @@
       </c>
       <c r="D313" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E313" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="314">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="D314" s="5" t="inlineStr">
         <is>
-          <t>Indicator Circle</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E314" s="7" t="n">
@@ -9804,11 +9804,11 @@
       </c>
       <c r="D315" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Indicator Circle</t>
         </is>
       </c>
       <c r="E315" s="7" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="316">
@@ -9833,7 +9833,7 @@
         </is>
       </c>
       <c r="E316" s="7" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="317">
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="E317" s="7" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="318">
@@ -9879,11 +9879,11 @@
       </c>
       <c r="D318" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E318" s="7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="319">
@@ -9904,11 +9904,11 @@
       </c>
       <c r="D319" s="5" t="inlineStr">
         <is>
-          <t>Main Search</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E319" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="320">
@@ -9929,11 +9929,11 @@
       </c>
       <c r="D320" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Main Search</t>
         </is>
       </c>
       <c r="E320" s="7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="321">
@@ -9954,7 +9954,7 @@
       </c>
       <c r="D321" s="5" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E321" s="7" t="n">
@@ -9979,11 +9979,11 @@
       </c>
       <c r="D322" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Pagination</t>
         </is>
       </c>
       <c r="E322" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="323">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="D323" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E323" s="7" t="n">
@@ -10029,11 +10029,11 @@
       </c>
       <c r="D324" s="5" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E324" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="325">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="D325" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="E325" s="7" t="n">
@@ -18060,7 +18060,7 @@
         </is>
       </c>
       <c r="D84" s="12" t="n">
-        <v>328</v>
+        <v>341</v>
       </c>
     </row>
     <row r="85">
@@ -18080,7 +18080,7 @@
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>268</v>
+        <v>275</v>
       </c>
     </row>
     <row r="86">
@@ -18100,7 +18100,7 @@
         </is>
       </c>
       <c r="D86" s="12" t="n">
-        <v>139</v>
+        <v>165</v>
       </c>
     </row>
     <row r="87">
@@ -18116,11 +18116,11 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Component 9</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="88">
@@ -18136,11 +18136,11 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Component 9</t>
         </is>
       </c>
       <c r="D88" s="12" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="89">
@@ -18160,7 +18160,7 @@
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="90">
@@ -18176,11 +18176,11 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>mail</t>
+          <t>Frame 1707479054</t>
         </is>
       </c>
       <c r="D90" s="12" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="91">
@@ -18196,11 +18196,11 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Frame 1707479054</t>
+          <t>mail</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="92">
@@ -18220,7 +18220,7 @@
         </is>
       </c>
       <c r="D92" s="12" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="93">
@@ -18256,11 +18256,11 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>informacion de poliza</t>
         </is>
       </c>
       <c r="D94" s="12" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="95">
@@ -18276,11 +18276,11 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>informacion de poliza</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="96">
@@ -18296,11 +18296,11 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Tooltip</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D96" s="12" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="97">
@@ -18316,7 +18316,7 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>dólares</t>
+          <t>Tooltip</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
@@ -18336,11 +18336,11 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>datos personales</t>
         </is>
       </c>
       <c r="D98" s="12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="99">
@@ -18356,11 +18356,11 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>directionLeft</t>
+          <t>dólares</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100">
@@ -18376,11 +18376,11 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>datos personales</t>
+          <t>directionLeft</t>
         </is>
       </c>
       <c r="D100" s="12" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="101">
@@ -18396,7 +18396,7 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>soles</t>
+          <t>24.timer</t>
         </is>
       </c>
       <c r="D101" s="12" t="n">
@@ -18576,11 +18576,11 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>DirectionUp</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="D110" s="12" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="111">
@@ -18596,7 +18596,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>DirectionUp</t>
         </is>
       </c>
       <c r="D111" s="12" t="n">
@@ -18620,7 +18620,7 @@
         </is>
       </c>
       <c r="D112" s="12" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="113">
@@ -18636,11 +18636,11 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>billetera</t>
         </is>
       </c>
       <c r="D113" s="12" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="114">
@@ -18656,11 +18656,11 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>billetera</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D114" s="12" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="115">
@@ -18676,7 +18676,7 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>create account</t>
         </is>
       </c>
       <c r="D115" s="12" t="n">
@@ -18696,11 +18696,11 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D116" s="12" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="117">
@@ -18716,11 +18716,11 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>create account</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D117" s="12" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="118">
@@ -18776,11 +18776,11 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>AGENDA</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D120" s="12" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="121">
@@ -18796,7 +18796,7 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>download</t>
+          <t>AGENDA</t>
         </is>
       </c>
       <c r="D121" s="12" t="n">
@@ -22243,10 +22243,10 @@
         <v>22</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>13859</v>
+        <v>13997</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>21326</v>
+        <v>21554</v>
       </c>
     </row>
     <row r="7">
@@ -22315,10 +22315,10 @@
         <v>5</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>10368</v>
+        <v>10633</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>13210</v>
+        <v>13584</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-19 17:32 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -693,10 +693,10 @@
         <v>44</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>172957</v>
+        <v>172968</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>11346</v>
+        <v>11352</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -725,10 +725,10 @@
         <v>5</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>10633</v>
+        <v>10716</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2951</v>
+        <v>3008</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>34</v>
@@ -757,10 +757,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>13997</v>
+        <v>14039</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7557</v>
+        <v>7579</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -1423,10 +1423,10 @@
         <v>37</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>157752</v>
+        <v>157763</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>10480</v>
+        <v>10486</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -1457,10 +1457,10 @@
         <v>5</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10633</v>
+        <v>10716</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>2951</v>
+        <v>3008</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>34</v>
@@ -1559,13 +1559,13 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1939</v>
+        <v>1981</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>448</v>
+        <v>470</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
@@ -1924,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E577"/>
+  <dimension ref="A1:E580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6408,7 +6408,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>7416</v>
+        <v>7421</v>
       </c>
     </row>
     <row r="180">
@@ -6433,7 +6433,7 @@
         </is>
       </c>
       <c r="E180" s="7" t="n">
-        <v>5248</v>
+        <v>5251</v>
       </c>
     </row>
     <row r="181">
@@ -6683,7 +6683,7 @@
         </is>
       </c>
       <c r="E190" s="7" t="n">
-        <v>1093</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="191">
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="E202" s="7" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="203">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E217" s="7" t="n">
-        <v>1532</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="218">
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="E219" s="7" t="n">
-        <v>1358</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="220">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="E220" s="7" t="n">
-        <v>1341</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="221">
@@ -7483,7 +7483,7 @@
         </is>
       </c>
       <c r="E222" s="7" t="n">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="223">
@@ -7504,11 +7504,11 @@
       </c>
       <c r="D223" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E223" s="7" t="n">
-        <v>441</v>
+        <v>454</v>
       </c>
     </row>
     <row r="224">
@@ -7529,11 +7529,11 @@
       </c>
       <c r="D224" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E224" s="7" t="n">
-        <v>414</v>
+        <v>445</v>
       </c>
     </row>
     <row r="225">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="E225" s="7" t="n">
-        <v>316</v>
+        <v>326</v>
       </c>
     </row>
     <row r="226">
@@ -7783,7 +7783,7 @@
         </is>
       </c>
       <c r="E234" s="7" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="235">
@@ -7833,7 +7833,7 @@
         </is>
       </c>
       <c r="E236" s="7" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="237">
@@ -7858,7 +7858,7 @@
         </is>
       </c>
       <c r="E237" s="7" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="238">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="E307" s="7" t="n">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="308">
@@ -9633,7 +9633,7 @@
         </is>
       </c>
       <c r="E308" s="7" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="309">
@@ -9658,7 +9658,7 @@
         </is>
       </c>
       <c r="E309" s="7" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="310">
@@ -9683,7 +9683,7 @@
         </is>
       </c>
       <c r="E310" s="7" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="311">
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="E312" s="7" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="313">
@@ -9758,7 +9758,7 @@
         </is>
       </c>
       <c r="E313" s="7" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="314">
@@ -9833,7 +9833,7 @@
         </is>
       </c>
       <c r="E316" s="7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="317">
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="E317" s="7" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="318">
@@ -10154,11 +10154,11 @@
       </c>
       <c r="D329" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E329" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="330">
@@ -10179,11 +10179,11 @@
       </c>
       <c r="D330" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E330" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="331">
@@ -10204,11 +10204,11 @@
       </c>
       <c r="D331" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E331" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="332">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="D332" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E332" s="7" t="n">
@@ -10239,76 +10239,76 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Vida Ley &amp; SCTR</t>
         </is>
       </c>
       <c r="D333" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E333" s="7" t="n">
-        <v>305</v>
+        <v>1</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Vida Ley &amp; SCTR</t>
         </is>
       </c>
       <c r="D334" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E334" s="7" t="n">
-        <v>243</v>
+        <v>1</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Vida Ley &amp; SCTR</t>
         </is>
       </c>
       <c r="D335" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E335" s="7" t="n">
-        <v>164</v>
+        <v>1</v>
       </c>
     </row>
     <row r="336">
@@ -10329,11 +10329,11 @@
       </c>
       <c r="D336" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E336" s="7" t="n">
-        <v>110</v>
+        <v>305</v>
       </c>
     </row>
     <row r="337">
@@ -10354,11 +10354,11 @@
       </c>
       <c r="D337" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E337" s="7" t="n">
-        <v>83</v>
+        <v>243</v>
       </c>
     </row>
     <row r="338">
@@ -10379,11 +10379,11 @@
       </c>
       <c r="D338" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E338" s="7" t="n">
-        <v>76</v>
+        <v>164</v>
       </c>
     </row>
     <row r="339">
@@ -10404,11 +10404,11 @@
       </c>
       <c r="D339" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E339" s="7" t="n">
-        <v>61</v>
+        <v>110</v>
       </c>
     </row>
     <row r="340">
@@ -10429,11 +10429,11 @@
       </c>
       <c r="D340" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E340" s="7" t="n">
-        <v>54</v>
+        <v>83</v>
       </c>
     </row>
     <row r="341">
@@ -10454,11 +10454,11 @@
       </c>
       <c r="D341" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E341" s="7" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
     </row>
     <row r="342">
@@ -10479,11 +10479,11 @@
       </c>
       <c r="D342" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E342" s="7" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="343">
@@ -10504,11 +10504,11 @@
       </c>
       <c r="D343" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E343" s="7" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="344">
@@ -10529,11 +10529,11 @@
       </c>
       <c r="D344" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E344" s="7" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="345">
@@ -10554,11 +10554,11 @@
       </c>
       <c r="D345" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E345" s="7" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="346">
@@ -10579,11 +10579,11 @@
       </c>
       <c r="D346" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E346" s="7" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
     </row>
     <row r="347">
@@ -10604,11 +10604,11 @@
       </c>
       <c r="D347" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E347" s="7" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
     </row>
     <row r="348">
@@ -10629,11 +10629,11 @@
       </c>
       <c r="D348" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E348" s="7" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
     </row>
     <row r="349">
@@ -10654,11 +10654,11 @@
       </c>
       <c r="D349" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E349" s="7" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="350">
@@ -10679,11 +10679,11 @@
       </c>
       <c r="D350" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E350" s="7" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="351">
@@ -10704,11 +10704,11 @@
       </c>
       <c r="D351" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E351" s="7" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="352">
@@ -10729,11 +10729,11 @@
       </c>
       <c r="D352" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E352" s="7" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="353">
@@ -10754,11 +10754,11 @@
       </c>
       <c r="D353" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E353" s="7" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="354">
@@ -10779,11 +10779,11 @@
       </c>
       <c r="D354" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E354" s="7" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="355">
@@ -10804,11 +10804,11 @@
       </c>
       <c r="D355" s="5" t="inlineStr">
         <is>
-          <t>Bottom Bar</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E355" s="7" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="356">
@@ -10829,11 +10829,11 @@
       </c>
       <c r="D356" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E356" s="7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="357">
@@ -10854,11 +10854,11 @@
       </c>
       <c r="D357" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E357" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="358">
@@ -10879,11 +10879,11 @@
       </c>
       <c r="D358" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="E358" s="7" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="359">
@@ -10904,11 +10904,11 @@
       </c>
       <c r="D359" s="5" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E359" s="7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="360">
@@ -10919,21 +10919,21 @@
       </c>
       <c r="B360" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C360" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="D360" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E360" s="7" t="n">
-        <v>433</v>
+        <v>2</v>
       </c>
     </row>
     <row r="361">
@@ -10944,21 +10944,21 @@
       </c>
       <c r="B361" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C361" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="D361" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E361" s="7" t="n">
-        <v>215</v>
+        <v>2</v>
       </c>
     </row>
     <row r="362">
@@ -10969,21 +10969,21 @@
       </c>
       <c r="B362" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C362" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="D362" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Links</t>
         </is>
       </c>
       <c r="E362" s="7" t="n">
-        <v>196</v>
+        <v>1</v>
       </c>
     </row>
     <row r="363">
@@ -11004,11 +11004,11 @@
       </c>
       <c r="D363" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E363" s="7" t="n">
-        <v>174</v>
+        <v>433</v>
       </c>
     </row>
     <row r="364">
@@ -11029,11 +11029,11 @@
       </c>
       <c r="D364" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E364" s="7" t="n">
-        <v>149</v>
+        <v>215</v>
       </c>
     </row>
     <row r="365">
@@ -11054,11 +11054,11 @@
       </c>
       <c r="D365" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E365" s="7" t="n">
-        <v>124</v>
+        <v>196</v>
       </c>
     </row>
     <row r="366">
@@ -11079,11 +11079,11 @@
       </c>
       <c r="D366" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E366" s="7" t="n">
-        <v>121</v>
+        <v>174</v>
       </c>
     </row>
     <row r="367">
@@ -11104,11 +11104,11 @@
       </c>
       <c r="D367" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E367" s="7" t="n">
-        <v>114</v>
+        <v>149</v>
       </c>
     </row>
     <row r="368">
@@ -11129,11 +11129,11 @@
       </c>
       <c r="D368" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E368" s="7" t="n">
-        <v>102</v>
+        <v>124</v>
       </c>
     </row>
     <row r="369">
@@ -11154,11 +11154,11 @@
       </c>
       <c r="D369" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E369" s="7" t="n">
-        <v>92</v>
+        <v>121</v>
       </c>
     </row>
     <row r="370">
@@ -11179,11 +11179,11 @@
       </c>
       <c r="D370" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E370" s="7" t="n">
-        <v>88</v>
+        <v>114</v>
       </c>
     </row>
     <row r="371">
@@ -11204,11 +11204,11 @@
       </c>
       <c r="D371" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E371" s="7" t="n">
-        <v>72</v>
+        <v>102</v>
       </c>
     </row>
     <row r="372">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="D372" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E372" s="7" t="n">
-        <v>64</v>
+        <v>92</v>
       </c>
     </row>
     <row r="373">
@@ -11254,11 +11254,11 @@
       </c>
       <c r="D373" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E373" s="7" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
     </row>
     <row r="374">
@@ -11279,11 +11279,11 @@
       </c>
       <c r="D374" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E374" s="7" t="n">
-        <v>49</v>
+        <v>72</v>
       </c>
     </row>
     <row r="375">
@@ -11304,11 +11304,11 @@
       </c>
       <c r="D375" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E375" s="7" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
     </row>
     <row r="376">
@@ -11329,11 +11329,11 @@
       </c>
       <c r="D376" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E376" s="7" t="n">
-        <v>41</v>
+        <v>62</v>
       </c>
     </row>
     <row r="377">
@@ -11354,11 +11354,11 @@
       </c>
       <c r="D377" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E377" s="7" t="n">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="378">
@@ -11379,11 +11379,11 @@
       </c>
       <c r="D378" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E378" s="7" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="379">
@@ -11404,11 +11404,11 @@
       </c>
       <c r="D379" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E379" s="7" t="n">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="380">
@@ -11429,11 +11429,11 @@
       </c>
       <c r="D380" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E380" s="7" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="381">
@@ -11454,11 +11454,11 @@
       </c>
       <c r="D381" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E381" s="7" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="382">
@@ -11479,11 +11479,11 @@
       </c>
       <c r="D382" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E382" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="383">
@@ -11504,11 +11504,11 @@
       </c>
       <c r="D383" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E383" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="384">
@@ -11529,11 +11529,11 @@
       </c>
       <c r="D384" s="5" t="inlineStr">
         <is>
-          <t>Bottom Bar</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E384" s="7" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="385">
@@ -11554,11 +11554,11 @@
       </c>
       <c r="D385" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E385" s="7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="386">
@@ -11579,11 +11579,11 @@
       </c>
       <c r="D386" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E386" s="7" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="387">
@@ -11604,11 +11604,11 @@
       </c>
       <c r="D387" s="5" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="E387" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="388">
@@ -11619,21 +11619,21 @@
       </c>
       <c r="B388" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C388" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="D388" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E388" s="7" t="n">
-        <v>160</v>
+        <v>9</v>
       </c>
     </row>
     <row r="389">
@@ -11644,21 +11644,21 @@
       </c>
       <c r="B389" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C389" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="D389" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E389" s="7" t="n">
-        <v>149</v>
+        <v>6</v>
       </c>
     </row>
     <row r="390">
@@ -11669,21 +11669,21 @@
       </c>
       <c r="B390" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C390" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="D390" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Links</t>
         </is>
       </c>
       <c r="E390" s="7" t="n">
-        <v>136</v>
+        <v>2</v>
       </c>
     </row>
     <row r="391">
@@ -11704,11 +11704,11 @@
       </c>
       <c r="D391" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E391" s="7" t="n">
-        <v>107</v>
+        <v>160</v>
       </c>
     </row>
     <row r="392">
@@ -11729,11 +11729,11 @@
       </c>
       <c r="D392" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E392" s="7" t="n">
-        <v>77</v>
+        <v>149</v>
       </c>
     </row>
     <row r="393">
@@ -11754,11 +11754,11 @@
       </c>
       <c r="D393" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E393" s="7" t="n">
-        <v>63</v>
+        <v>136</v>
       </c>
     </row>
     <row r="394">
@@ -11779,11 +11779,11 @@
       </c>
       <c r="D394" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E394" s="7" t="n">
-        <v>60</v>
+        <v>107</v>
       </c>
     </row>
     <row r="395">
@@ -11804,11 +11804,11 @@
       </c>
       <c r="D395" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E395" s="7" t="n">
-        <v>48</v>
+        <v>77</v>
       </c>
     </row>
     <row r="396">
@@ -11829,11 +11829,11 @@
       </c>
       <c r="D396" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E396" s="7" t="n">
-        <v>20</v>
+        <v>63</v>
       </c>
     </row>
     <row r="397">
@@ -11854,11 +11854,11 @@
       </c>
       <c r="D397" s="5" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E397" s="7" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="398">
@@ -11879,11 +11879,11 @@
       </c>
       <c r="D398" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E398" s="7" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
     </row>
     <row r="399">
@@ -11904,11 +11904,11 @@
       </c>
       <c r="D399" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E399" s="7" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="400">
@@ -11929,11 +11929,11 @@
       </c>
       <c r="D400" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="E400" s="7" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="401">
@@ -11954,11 +11954,11 @@
       </c>
       <c r="D401" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E401" s="7" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="402">
@@ -11979,11 +11979,11 @@
       </c>
       <c r="D402" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E402" s="7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="403">
@@ -12004,11 +12004,11 @@
       </c>
       <c r="D403" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E403" s="7" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="404">
@@ -12029,11 +12029,11 @@
       </c>
       <c r="D404" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E404" s="7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="405">
@@ -12054,11 +12054,11 @@
       </c>
       <c r="D405" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E405" s="7" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="406">
@@ -12079,11 +12079,11 @@
       </c>
       <c r="D406" s="5" t="inlineStr">
         <is>
-          <t>Infografia</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E406" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="407">
@@ -12104,11 +12104,11 @@
       </c>
       <c r="D407" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E407" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="408">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="D408" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E408" s="7" t="n">
@@ -12154,11 +12154,11 @@
       </c>
       <c r="D409" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Infografia</t>
         </is>
       </c>
       <c r="E409" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="410">
@@ -12179,11 +12179,11 @@
       </c>
       <c r="D410" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E410" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="411">
@@ -12204,11 +12204,11 @@
       </c>
       <c r="D411" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E411" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="412">
@@ -12229,11 +12229,11 @@
       </c>
       <c r="D412" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E412" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="413">
@@ -12244,21 +12244,21 @@
       </c>
       <c r="B413" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C413" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="D413" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E413" s="7" t="n">
-        <v>597</v>
+        <v>1</v>
       </c>
     </row>
     <row r="414">
@@ -12269,21 +12269,21 @@
       </c>
       <c r="B414" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C414" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="D414" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E414" s="7" t="n">
-        <v>331</v>
+        <v>1</v>
       </c>
     </row>
     <row r="415">
@@ -12294,21 +12294,21 @@
       </c>
       <c r="B415" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C415" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="D415" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E415" s="7" t="n">
-        <v>327</v>
+        <v>1</v>
       </c>
     </row>
     <row r="416">
@@ -12329,11 +12329,11 @@
       </c>
       <c r="D416" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E416" s="7" t="n">
-        <v>276</v>
+        <v>597</v>
       </c>
     </row>
     <row r="417">
@@ -12354,11 +12354,11 @@
       </c>
       <c r="D417" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E417" s="7" t="n">
-        <v>166</v>
+        <v>331</v>
       </c>
     </row>
     <row r="418">
@@ -12379,11 +12379,11 @@
       </c>
       <c r="D418" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E418" s="7" t="n">
-        <v>151</v>
+        <v>327</v>
       </c>
     </row>
     <row r="419">
@@ -12404,11 +12404,11 @@
       </c>
       <c r="D419" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E419" s="7" t="n">
-        <v>116</v>
+        <v>276</v>
       </c>
     </row>
     <row r="420">
@@ -12429,11 +12429,11 @@
       </c>
       <c r="D420" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E420" s="7" t="n">
-        <v>70</v>
+        <v>166</v>
       </c>
     </row>
     <row r="421">
@@ -12454,11 +12454,11 @@
       </c>
       <c r="D421" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E421" s="7" t="n">
-        <v>60</v>
+        <v>151</v>
       </c>
     </row>
     <row r="422">
@@ -12479,11 +12479,11 @@
       </c>
       <c r="D422" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E422" s="7" t="n">
-        <v>56</v>
+        <v>116</v>
       </c>
     </row>
     <row r="423">
@@ -12504,11 +12504,11 @@
       </c>
       <c r="D423" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E423" s="7" t="n">
-        <v>48</v>
+        <v>70</v>
       </c>
     </row>
     <row r="424">
@@ -12529,11 +12529,11 @@
       </c>
       <c r="D424" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E424" s="7" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="425">
@@ -12554,11 +12554,11 @@
       </c>
       <c r="D425" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E425" s="7" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="426">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="D426" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E426" s="7" t="n">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="D427" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E427" s="7" t="n">
@@ -12629,11 +12629,11 @@
       </c>
       <c r="D428" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E428" s="7" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="429">
@@ -12654,11 +12654,11 @@
       </c>
       <c r="D429" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E429" s="7" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
     </row>
     <row r="430">
@@ -12679,11 +12679,11 @@
       </c>
       <c r="D430" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E430" s="7" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
     </row>
     <row r="431">
@@ -12704,11 +12704,11 @@
       </c>
       <c r="D431" s="5" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E431" s="7" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
     </row>
     <row r="432">
@@ -12729,11 +12729,11 @@
       </c>
       <c r="D432" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E432" s="7" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
     </row>
     <row r="433">
@@ -12754,11 +12754,11 @@
       </c>
       <c r="D433" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E433" s="7" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="434">
@@ -12779,11 +12779,11 @@
       </c>
       <c r="D434" s="5" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>Links</t>
         </is>
       </c>
       <c r="E434" s="7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="435">
@@ -12804,11 +12804,11 @@
       </c>
       <c r="D435" s="5" t="inlineStr">
         <is>
-          <t>Bottom Bar</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E435" s="7" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="436">
@@ -12829,11 +12829,11 @@
       </c>
       <c r="D436" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E436" s="7" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="437">
@@ -12854,11 +12854,11 @@
       </c>
       <c r="D437" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="E437" s="7" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="438">
@@ -12879,11 +12879,11 @@
       </c>
       <c r="D438" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="E438" s="7" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="439">
@@ -12904,11 +12904,11 @@
       </c>
       <c r="D439" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E439" s="7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="440">
@@ -12929,11 +12929,11 @@
       </c>
       <c r="D440" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E440" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="441">
@@ -12954,11 +12954,11 @@
       </c>
       <c r="D441" s="5" t="inlineStr">
         <is>
-          <t>Comparador</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E441" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="442">
@@ -12969,21 +12969,21 @@
       </c>
       <c r="B442" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="C442" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="D442" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E442" s="7" t="n">
-        <v>1536</v>
+        <v>8</v>
       </c>
     </row>
     <row r="443">
@@ -12994,21 +12994,21 @@
       </c>
       <c r="B443" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="C443" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="D443" s="5" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E443" s="7" t="n">
-        <v>340</v>
+        <v>2</v>
       </c>
     </row>
     <row r="444">
@@ -13019,21 +13019,21 @@
       </c>
       <c r="B444" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="C444" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="D444" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Comparador</t>
         </is>
       </c>
       <c r="E444" s="7" t="n">
-        <v>256</v>
+        <v>2</v>
       </c>
     </row>
     <row r="445">
@@ -13054,11 +13054,11 @@
       </c>
       <c r="D445" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E445" s="7" t="n">
-        <v>251</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="446">
@@ -13079,11 +13079,11 @@
       </c>
       <c r="D446" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Menu Item</t>
         </is>
       </c>
       <c r="E446" s="7" t="n">
-        <v>160</v>
+        <v>340</v>
       </c>
     </row>
     <row r="447">
@@ -13104,11 +13104,11 @@
       </c>
       <c r="D447" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E447" s="7" t="n">
-        <v>155</v>
+        <v>256</v>
       </c>
     </row>
     <row r="448">
@@ -13129,11 +13129,11 @@
       </c>
       <c r="D448" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E448" s="7" t="n">
-        <v>131</v>
+        <v>251</v>
       </c>
     </row>
     <row r="449">
@@ -13154,11 +13154,11 @@
       </c>
       <c r="D449" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E449" s="7" t="n">
-        <v>128</v>
+        <v>160</v>
       </c>
     </row>
     <row r="450">
@@ -13179,11 +13179,11 @@
       </c>
       <c r="D450" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E450" s="7" t="n">
-        <v>87</v>
+        <v>155</v>
       </c>
     </row>
     <row r="451">
@@ -13204,11 +13204,11 @@
       </c>
       <c r="D451" s="5" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E451" s="7" t="n">
-        <v>85</v>
+        <v>131</v>
       </c>
     </row>
     <row r="452">
@@ -13229,11 +13229,11 @@
       </c>
       <c r="D452" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E452" s="7" t="n">
-        <v>64</v>
+        <v>128</v>
       </c>
     </row>
     <row r="453">
@@ -13254,11 +13254,11 @@
       </c>
       <c r="D453" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E453" s="7" t="n">
-        <v>54</v>
+        <v>87</v>
       </c>
     </row>
     <row r="454">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="D454" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="E454" s="7" t="n">
-        <v>48</v>
+        <v>85</v>
       </c>
     </row>
     <row r="455">
@@ -13304,11 +13304,11 @@
       </c>
       <c r="D455" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E455" s="7" t="n">
-        <v>39</v>
+        <v>64</v>
       </c>
     </row>
     <row r="456">
@@ -13329,11 +13329,11 @@
       </c>
       <c r="D456" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E456" s="7" t="n">
-        <v>32</v>
+        <v>54</v>
       </c>
     </row>
     <row r="457">
@@ -13354,11 +13354,11 @@
       </c>
       <c r="D457" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E457" s="7" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
     </row>
     <row r="458">
@@ -13379,11 +13379,11 @@
       </c>
       <c r="D458" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E458" s="7" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="459">
@@ -13404,11 +13404,11 @@
       </c>
       <c r="D459" s="5" t="inlineStr">
         <is>
-          <t>Topbar</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E459" s="7" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="460">
@@ -13429,11 +13429,11 @@
       </c>
       <c r="D460" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E460" s="7" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="461">
@@ -13454,11 +13454,11 @@
       </c>
       <c r="D461" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E461" s="7" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="462">
@@ -13479,11 +13479,11 @@
       </c>
       <c r="D462" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Topbar</t>
         </is>
       </c>
       <c r="E462" s="7" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="463">
@@ -13504,11 +13504,11 @@
       </c>
       <c r="D463" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E463" s="7" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="464">
@@ -13529,11 +13529,11 @@
       </c>
       <c r="D464" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E464" s="7" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="465">
@@ -13554,11 +13554,11 @@
       </c>
       <c r="D465" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E465" s="7" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="466">
@@ -13579,11 +13579,11 @@
       </c>
       <c r="D466" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E466" s="7" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="467">
@@ -13604,11 +13604,11 @@
       </c>
       <c r="D467" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E467" s="7" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="468">
@@ -13629,11 +13629,11 @@
       </c>
       <c r="D468" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E468" s="7" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="469">
@@ -13654,11 +13654,11 @@
       </c>
       <c r="D469" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E469" s="7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="470">
@@ -13679,11 +13679,11 @@
       </c>
       <c r="D470" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E470" s="7" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="471">
@@ -13694,21 +13694,21 @@
       </c>
       <c r="B471" s="4" t="inlineStr">
         <is>
-          <t>VDT</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="C471" s="4" t="inlineStr">
         <is>
-          <t>VDT — Perfilador Productos Vida</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="D471" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E471" s="7" t="n">
-        <v>1152</v>
+        <v>10</v>
       </c>
     </row>
     <row r="472">
@@ -13719,21 +13719,21 @@
       </c>
       <c r="B472" s="4" t="inlineStr">
         <is>
-          <t>VDT</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="C472" s="4" t="inlineStr">
         <is>
-          <t>VDT — Perfilador Productos Vida</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="D472" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E472" s="7" t="n">
-        <v>618</v>
+        <v>9</v>
       </c>
     </row>
     <row r="473">
@@ -13744,21 +13744,21 @@
       </c>
       <c r="B473" s="4" t="inlineStr">
         <is>
-          <t>VDT</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="C473" s="4" t="inlineStr">
         <is>
-          <t>VDT — Perfilador Productos Vida</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="D473" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E473" s="7" t="n">
-        <v>440</v>
+        <v>6</v>
       </c>
     </row>
     <row r="474">
@@ -13779,11 +13779,11 @@
       </c>
       <c r="D474" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E474" s="7" t="n">
-        <v>375</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="475">
@@ -13804,11 +13804,11 @@
       </c>
       <c r="D475" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E475" s="7" t="n">
-        <v>192</v>
+        <v>618</v>
       </c>
     </row>
     <row r="476">
@@ -13829,11 +13829,11 @@
       </c>
       <c r="D476" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E476" s="7" t="n">
-        <v>120</v>
+        <v>440</v>
       </c>
     </row>
     <row r="477">
@@ -13854,11 +13854,11 @@
       </c>
       <c r="D477" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E477" s="7" t="n">
-        <v>104</v>
+        <v>375</v>
       </c>
     </row>
     <row r="478">
@@ -13879,11 +13879,11 @@
       </c>
       <c r="D478" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E478" s="7" t="n">
-        <v>96</v>
+        <v>192</v>
       </c>
     </row>
     <row r="479">
@@ -13904,11 +13904,11 @@
       </c>
       <c r="D479" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E479" s="7" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
     </row>
     <row r="480">
@@ -13929,11 +13929,11 @@
       </c>
       <c r="D480" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E480" s="7" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
     </row>
     <row r="481">
@@ -13954,11 +13954,11 @@
       </c>
       <c r="D481" s="5" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E481" s="7" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
     </row>
     <row r="482">
@@ -13979,11 +13979,11 @@
       </c>
       <c r="D482" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E482" s="7" t="n">
-        <v>71</v>
+        <v>93</v>
       </c>
     </row>
     <row r="483">
@@ -14004,11 +14004,11 @@
       </c>
       <c r="D483" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E483" s="7" t="n">
-        <v>68</v>
+        <v>90</v>
       </c>
     </row>
     <row r="484">
@@ -14029,11 +14029,11 @@
       </c>
       <c r="D484" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Menu Item</t>
         </is>
       </c>
       <c r="E484" s="7" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
     </row>
     <row r="485">
@@ -14054,11 +14054,11 @@
       </c>
       <c r="D485" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E485" s="7" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
     </row>
     <row r="486">
@@ -14079,11 +14079,11 @@
       </c>
       <c r="D486" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E486" s="7" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
     </row>
     <row r="487">
@@ -14104,11 +14104,11 @@
       </c>
       <c r="D487" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E487" s="7" t="n">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="488">
@@ -14129,11 +14129,11 @@
       </c>
       <c r="D488" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E488" s="7" t="n">
-        <v>34</v>
+        <v>57</v>
       </c>
     </row>
     <row r="489">
@@ -14154,11 +14154,11 @@
       </c>
       <c r="D489" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E489" s="7" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="490">
@@ -14179,11 +14179,11 @@
       </c>
       <c r="D490" s="5" t="inlineStr">
         <is>
-          <t>Chip Deleteable</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E490" s="7" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="491">
@@ -14204,11 +14204,11 @@
       </c>
       <c r="D491" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E491" s="7" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="492">
@@ -14229,11 +14229,11 @@
       </c>
       <c r="D492" s="5" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E492" s="7" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="493">
@@ -14254,11 +14254,11 @@
       </c>
       <c r="D493" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Chip Deleteable</t>
         </is>
       </c>
       <c r="E493" s="7" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="494">
@@ -14279,11 +14279,11 @@
       </c>
       <c r="D494" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E494" s="7" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="495">
@@ -14304,11 +14304,11 @@
       </c>
       <c r="D495" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="E495" s="7" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="496">
@@ -14329,11 +14329,11 @@
       </c>
       <c r="D496" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E496" s="7" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="497">
@@ -14354,11 +14354,11 @@
       </c>
       <c r="D497" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E497" s="7" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="498">
@@ -14379,11 +14379,11 @@
       </c>
       <c r="D498" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E498" s="7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="499">
@@ -14404,86 +14404,86 @@
       </c>
       <c r="D499" s="5" t="inlineStr">
         <is>
-          <t>Topbar</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E499" s="7" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B500" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="C500" s="4" t="inlineStr">
         <is>
-          <t>Productos Vida</t>
+          <t>VDT — Perfilador Productos Vida</t>
         </is>
       </c>
       <c r="D500" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E500" s="7" t="n">
-        <v>950</v>
+        <v>7</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B501" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="C501" s="4" t="inlineStr">
         <is>
-          <t>Productos Vida</t>
+          <t>VDT — Perfilador Productos Vida</t>
         </is>
       </c>
       <c r="D501" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E501" s="7" t="n">
-        <v>909</v>
+        <v>6</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B502" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="C502" s="4" t="inlineStr">
         <is>
-          <t>Productos Vida</t>
+          <t>VDT — Perfilador Productos Vida</t>
         </is>
       </c>
       <c r="D502" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Topbar</t>
         </is>
       </c>
       <c r="E502" s="7" t="n">
-        <v>819</v>
+        <v>4</v>
       </c>
     </row>
     <row r="503">
@@ -14504,11 +14504,11 @@
       </c>
       <c r="D503" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E503" s="7" t="n">
-        <v>678</v>
+        <v>950</v>
       </c>
     </row>
     <row r="504">
@@ -14529,11 +14529,11 @@
       </c>
       <c r="D504" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E504" s="7" t="n">
-        <v>484</v>
+        <v>909</v>
       </c>
     </row>
     <row r="505">
@@ -14554,11 +14554,11 @@
       </c>
       <c r="D505" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E505" s="7" t="n">
-        <v>404</v>
+        <v>819</v>
       </c>
     </row>
     <row r="506">
@@ -14579,11 +14579,11 @@
       </c>
       <c r="D506" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E506" s="7" t="n">
-        <v>214</v>
+        <v>678</v>
       </c>
     </row>
     <row r="507">
@@ -14604,11 +14604,11 @@
       </c>
       <c r="D507" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E507" s="7" t="n">
-        <v>150</v>
+        <v>484</v>
       </c>
     </row>
     <row r="508">
@@ -14629,11 +14629,11 @@
       </c>
       <c r="D508" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E508" s="7" t="n">
-        <v>100</v>
+        <v>404</v>
       </c>
     </row>
     <row r="509">
@@ -14654,11 +14654,11 @@
       </c>
       <c r="D509" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E509" s="7" t="n">
-        <v>86</v>
+        <v>214</v>
       </c>
     </row>
     <row r="510">
@@ -14679,11 +14679,11 @@
       </c>
       <c r="D510" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E510" s="7" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="511">
@@ -14704,11 +14704,11 @@
       </c>
       <c r="D511" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E511" s="7" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="512">
@@ -14729,11 +14729,11 @@
       </c>
       <c r="D512" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E512" s="7" t="n">
-        <v>30</v>
+        <v>86</v>
       </c>
     </row>
     <row r="513">
@@ -14754,11 +14754,11 @@
       </c>
       <c r="D513" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E513" s="7" t="n">
-        <v>26</v>
+        <v>86</v>
       </c>
     </row>
     <row r="514">
@@ -14779,11 +14779,11 @@
       </c>
       <c r="D514" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E514" s="7" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="515">
@@ -14804,11 +14804,11 @@
       </c>
       <c r="D515" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E515" s="7" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
     </row>
     <row r="516">
@@ -14829,11 +14829,11 @@
       </c>
       <c r="D516" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E516" s="7" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="517">
@@ -14854,11 +14854,11 @@
       </c>
       <c r="D517" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E517" s="7" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="518">
@@ -14879,11 +14879,11 @@
       </c>
       <c r="D518" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E518" s="7" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="519">
@@ -14904,11 +14904,11 @@
       </c>
       <c r="D519" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E519" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="520">
@@ -14929,11 +14929,11 @@
       </c>
       <c r="D520" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E520" s="7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="521">
@@ -14949,16 +14949,16 @@
       </c>
       <c r="C521" s="4" t="inlineStr">
         <is>
-          <t>Menú / Home</t>
+          <t>Productos Vida</t>
         </is>
       </c>
       <c r="D521" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E521" s="7" t="n">
-        <v>1995</v>
+        <v>9</v>
       </c>
     </row>
     <row r="522">
@@ -14974,16 +14974,16 @@
       </c>
       <c r="C522" s="4" t="inlineStr">
         <is>
-          <t>Menú / Home</t>
+          <t>Productos Vida</t>
         </is>
       </c>
       <c r="D522" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E522" s="7" t="n">
-        <v>350</v>
+        <v>9</v>
       </c>
     </row>
     <row r="523">
@@ -14999,16 +14999,16 @@
       </c>
       <c r="C523" s="4" t="inlineStr">
         <is>
-          <t>Menú / Home</t>
+          <t>Productos Vida</t>
         </is>
       </c>
       <c r="D523" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E523" s="7" t="n">
-        <v>331</v>
+        <v>2</v>
       </c>
     </row>
     <row r="524">
@@ -15029,11 +15029,11 @@
       </c>
       <c r="D524" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E524" s="7" t="n">
-        <v>315</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="525">
@@ -15054,11 +15054,11 @@
       </c>
       <c r="D525" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E525" s="7" t="n">
-        <v>302</v>
+        <v>350</v>
       </c>
     </row>
     <row r="526">
@@ -15079,11 +15079,11 @@
       </c>
       <c r="D526" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E526" s="7" t="n">
-        <v>272</v>
+        <v>331</v>
       </c>
     </row>
     <row r="527">
@@ -15104,11 +15104,11 @@
       </c>
       <c r="D527" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E527" s="7" t="n">
-        <v>200</v>
+        <v>315</v>
       </c>
     </row>
     <row r="528">
@@ -15129,11 +15129,11 @@
       </c>
       <c r="D528" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E528" s="7" t="n">
-        <v>168</v>
+        <v>302</v>
       </c>
     </row>
     <row r="529">
@@ -15154,11 +15154,11 @@
       </c>
       <c r="D529" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E529" s="7" t="n">
-        <v>155</v>
+        <v>272</v>
       </c>
     </row>
     <row r="530">
@@ -15179,11 +15179,11 @@
       </c>
       <c r="D530" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E530" s="7" t="n">
-        <v>152</v>
+        <v>200</v>
       </c>
     </row>
     <row r="531">
@@ -15204,11 +15204,11 @@
       </c>
       <c r="D531" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E531" s="7" t="n">
-        <v>146</v>
+        <v>168</v>
       </c>
     </row>
     <row r="532">
@@ -15229,11 +15229,11 @@
       </c>
       <c r="D532" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E532" s="7" t="n">
-        <v>71</v>
+        <v>155</v>
       </c>
     </row>
     <row r="533">
@@ -15254,11 +15254,11 @@
       </c>
       <c r="D533" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E533" s="7" t="n">
-        <v>63</v>
+        <v>152</v>
       </c>
     </row>
     <row r="534">
@@ -15279,11 +15279,11 @@
       </c>
       <c r="D534" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E534" s="7" t="n">
-        <v>40</v>
+        <v>146</v>
       </c>
     </row>
     <row r="535">
@@ -15304,11 +15304,11 @@
       </c>
       <c r="D535" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E535" s="7" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
     </row>
     <row r="536">
@@ -15329,11 +15329,11 @@
       </c>
       <c r="D536" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E536" s="7" t="n">
-        <v>21</v>
+        <v>63</v>
       </c>
     </row>
     <row r="537">
@@ -15354,11 +15354,11 @@
       </c>
       <c r="D537" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E537" s="7" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="538">
@@ -15374,16 +15374,16 @@
       </c>
       <c r="C538" s="4" t="inlineStr">
         <is>
-          <t>Productos Líneas Personales</t>
+          <t>Menú / Home</t>
         </is>
       </c>
       <c r="D538" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E538" s="7" t="n">
-        <v>285</v>
+        <v>21</v>
       </c>
     </row>
     <row r="539">
@@ -15399,16 +15399,16 @@
       </c>
       <c r="C539" s="4" t="inlineStr">
         <is>
-          <t>Productos Líneas Personales</t>
+          <t>Menú / Home</t>
         </is>
       </c>
       <c r="D539" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E539" s="7" t="n">
-        <v>282</v>
+        <v>21</v>
       </c>
     </row>
     <row r="540">
@@ -15424,16 +15424,16 @@
       </c>
       <c r="C540" s="4" t="inlineStr">
         <is>
-          <t>Productos Líneas Personales</t>
+          <t>Menú / Home</t>
         </is>
       </c>
       <c r="D540" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E540" s="7" t="n">
-        <v>266</v>
+        <v>3</v>
       </c>
     </row>
     <row r="541">
@@ -15454,11 +15454,11 @@
       </c>
       <c r="D541" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E541" s="7" t="n">
-        <v>132</v>
+        <v>285</v>
       </c>
     </row>
     <row r="542">
@@ -15479,11 +15479,11 @@
       </c>
       <c r="D542" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E542" s="7" t="n">
-        <v>132</v>
+        <v>282</v>
       </c>
     </row>
     <row r="543">
@@ -15504,11 +15504,11 @@
       </c>
       <c r="D543" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E543" s="7" t="n">
-        <v>107</v>
+        <v>266</v>
       </c>
     </row>
     <row r="544">
@@ -15529,11 +15529,11 @@
       </c>
       <c r="D544" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E544" s="7" t="n">
-        <v>48</v>
+        <v>132</v>
       </c>
     </row>
     <row r="545">
@@ -15554,11 +15554,11 @@
       </c>
       <c r="D545" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E545" s="7" t="n">
-        <v>45</v>
+        <v>132</v>
       </c>
     </row>
     <row r="546">
@@ -15579,11 +15579,11 @@
       </c>
       <c r="D546" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E546" s="7" t="n">
-        <v>24</v>
+        <v>107</v>
       </c>
     </row>
     <row r="547">
@@ -15604,11 +15604,11 @@
       </c>
       <c r="D547" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E547" s="7" t="n">
-        <v>19</v>
+        <v>48</v>
       </c>
     </row>
     <row r="548">
@@ -15629,11 +15629,11 @@
       </c>
       <c r="D548" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E548" s="7" t="n">
-        <v>19</v>
+        <v>45</v>
       </c>
     </row>
     <row r="549">
@@ -15654,11 +15654,11 @@
       </c>
       <c r="D549" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E549" s="7" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="550">
@@ -15679,11 +15679,11 @@
       </c>
       <c r="D550" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E550" s="7" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="551">
@@ -15704,11 +15704,11 @@
       </c>
       <c r="D551" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E551" s="7" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="552">
@@ -15729,11 +15729,11 @@
       </c>
       <c r="D552" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E552" s="7" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="553">
@@ -15754,11 +15754,11 @@
       </c>
       <c r="D553" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E553" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="554">
@@ -15779,11 +15779,11 @@
       </c>
       <c r="D554" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E554" s="7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="555">
@@ -15804,11 +15804,11 @@
       </c>
       <c r="D555" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E555" s="7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="556">
@@ -15829,11 +15829,11 @@
       </c>
       <c r="D556" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E556" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="557">
@@ -15854,11 +15854,11 @@
       </c>
       <c r="D557" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E557" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="558">
@@ -15879,86 +15879,86 @@
       </c>
       <c r="D558" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E558" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="B559" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="C559" s="4" t="inlineStr">
         <is>
-          <t>Landing Alianzas</t>
+          <t>Productos Líneas Personales</t>
         </is>
       </c>
       <c r="D559" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E559" s="7" t="n">
-        <v>570</v>
+        <v>3</v>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="B560" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="C560" s="4" t="inlineStr">
         <is>
-          <t>Landing Alianzas</t>
+          <t>Productos Líneas Personales</t>
         </is>
       </c>
       <c r="D560" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E560" s="7" t="n">
-        <v>188</v>
+        <v>2</v>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="B561" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="C561" s="4" t="inlineStr">
         <is>
-          <t>Landing Alianzas</t>
+          <t>Productos Líneas Personales</t>
         </is>
       </c>
       <c r="D561" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E561" s="7" t="n">
-        <v>128</v>
+        <v>2</v>
       </c>
     </row>
     <row r="562">
@@ -15979,11 +15979,11 @@
       </c>
       <c r="D562" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E562" s="7" t="n">
-        <v>100</v>
+        <v>570</v>
       </c>
     </row>
     <row r="563">
@@ -16004,11 +16004,11 @@
       </c>
       <c r="D563" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E563" s="7" t="n">
-        <v>90</v>
+        <v>188</v>
       </c>
     </row>
     <row r="564">
@@ -16029,11 +16029,11 @@
       </c>
       <c r="D564" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E564" s="7" t="n">
-        <v>81</v>
+        <v>128</v>
       </c>
     </row>
     <row r="565">
@@ -16054,11 +16054,11 @@
       </c>
       <c r="D565" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E565" s="7" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
     </row>
     <row r="566">
@@ -16079,11 +16079,11 @@
       </c>
       <c r="D566" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E566" s="7" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="567">
@@ -16104,11 +16104,11 @@
       </c>
       <c r="D567" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E567" s="7" t="n">
-        <v>48</v>
+        <v>81</v>
       </c>
     </row>
     <row r="568">
@@ -16129,11 +16129,11 @@
       </c>
       <c r="D568" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E568" s="7" t="n">
-        <v>18</v>
+        <v>81</v>
       </c>
     </row>
     <row r="569">
@@ -16154,11 +16154,11 @@
       </c>
       <c r="D569" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E569" s="7" t="n">
-        <v>16</v>
+        <v>60</v>
       </c>
     </row>
     <row r="570">
@@ -16179,11 +16179,11 @@
       </c>
       <c r="D570" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E570" s="7" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
     </row>
     <row r="571">
@@ -16204,11 +16204,11 @@
       </c>
       <c r="D571" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E571" s="7" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="572">
@@ -16229,11 +16229,11 @@
       </c>
       <c r="D572" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E572" s="7" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="573">
@@ -16254,11 +16254,11 @@
       </c>
       <c r="D573" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E573" s="7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="574">
@@ -16279,11 +16279,11 @@
       </c>
       <c r="D574" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E574" s="7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="575">
@@ -16304,11 +16304,11 @@
       </c>
       <c r="D575" s="5" t="inlineStr">
         <is>
-          <t>Logo Horizontal</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E575" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="576">
@@ -16329,11 +16329,11 @@
       </c>
       <c r="D576" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E576" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="577">
@@ -16354,10 +16354,85 @@
       </c>
       <c r="D577" s="5" t="inlineStr">
         <is>
+          <t>title_+_social media</t>
+        </is>
+      </c>
+      <c r="E577" s="7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B578" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C578" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D578" s="5" t="inlineStr">
+        <is>
+          <t>Logo Horizontal</t>
+        </is>
+      </c>
+      <c r="E578" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B579" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C579" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D579" s="5" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="E579" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B580" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C580" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D580" s="5" t="inlineStr">
+        <is>
           <t>Calendar</t>
         </is>
       </c>
-      <c r="E577" s="7" t="n">
+      <c r="E580" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -17680,7 +17755,7 @@
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="66">
@@ -18000,7 +18075,7 @@
         </is>
       </c>
       <c r="D81" s="12" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="82">
@@ -18020,7 +18095,7 @@
         </is>
       </c>
       <c r="D82" s="12" t="n">
-        <v>484</v>
+        <v>499</v>
       </c>
     </row>
     <row r="83">
@@ -18040,7 +18115,7 @@
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>439</v>
+        <v>454</v>
       </c>
     </row>
     <row r="84">
@@ -18060,7 +18135,7 @@
         </is>
       </c>
       <c r="D84" s="12" t="n">
-        <v>341</v>
+        <v>348</v>
       </c>
     </row>
     <row r="85">
@@ -18080,7 +18155,7 @@
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="86">
@@ -18256,11 +18331,11 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>informacion de poliza</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D94" s="12" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="95">
@@ -18276,7 +18351,7 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>informacion de poliza</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
@@ -18316,11 +18391,11 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Tooltip</t>
+          <t>datos personales</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="98">
@@ -18336,11 +18411,11 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>datos personales</t>
+          <t>dólares</t>
         </is>
       </c>
       <c r="D98" s="12" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="99">
@@ -18356,7 +18431,7 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>dólares</t>
+          <t>directionLeft</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
@@ -18376,11 +18451,11 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>directionLeft</t>
+          <t>Tooltip</t>
         </is>
       </c>
       <c r="D100" s="12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="101">
@@ -22243,10 +22318,10 @@
         <v>22</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>13997</v>
+        <v>14039</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>21554</v>
+        <v>21618</v>
       </c>
     </row>
     <row r="7">
@@ -22279,10 +22354,10 @@
         <v>44</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>172957</v>
+        <v>172968</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>184303</v>
+        <v>184320</v>
       </c>
     </row>
     <row r="8">
@@ -22315,10 +22390,10 @@
         <v>5</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>10633</v>
+        <v>10716</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>13584</v>
+        <v>13724</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-19 22:22 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -757,10 +757,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>14039</v>
+        <v>14009</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7579</v>
+        <v>7570</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -1559,10 +1559,10 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1981</v>
+        <v>1951</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>470</v>
+        <v>461</v>
       </c>
       <c r="G15" s="8" t="n">
         <v>30</v>
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="E307" s="7" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="308">
@@ -9633,7 +9633,7 @@
         </is>
       </c>
       <c r="E308" s="7" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="309">
@@ -9658,7 +9658,7 @@
         </is>
       </c>
       <c r="E309" s="7" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="310">
@@ -9683,7 +9683,7 @@
         </is>
       </c>
       <c r="E310" s="7" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="311">
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="E312" s="7" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="313">
@@ -9758,7 +9758,7 @@
         </is>
       </c>
       <c r="E313" s="7" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="314">
@@ -9833,7 +9833,7 @@
         </is>
       </c>
       <c r="E316" s="7" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="317">
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="E317" s="7" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="318">
@@ -22318,10 +22318,10 @@
         <v>22</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>14039</v>
+        <v>14009</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>21618</v>
+        <v>21579</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-22 19:06 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -533,7 +533,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  2026-06-19</t>
+          <t>Quarter: Q2 2026  |  2026-06-22</t>
         </is>
       </c>
     </row>
@@ -693,10 +693,10 @@
         <v>44</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>172968</v>
+        <v>172970</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>11352</v>
+        <v>11356</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -978,16 +978,16 @@
         <v>3</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>11118</v>
+        <v>11472</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>2066</v>
+        <v>2122</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
@@ -1423,10 +1423,10 @@
         <v>37</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>157763</v>
+        <v>157765</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>10486</v>
+        <v>10490</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -1794,16 +1794,16 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>5094</v>
+        <v>5448</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>731</v>
+        <v>787</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
@@ -1924,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E580"/>
+  <dimension ref="A1:E581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6408,7 +6408,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>7421</v>
+        <v>7423</v>
       </c>
     </row>
     <row r="180">
@@ -14508,7 +14508,7 @@
         </is>
       </c>
       <c r="E503" s="7" t="n">
-        <v>950</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="504">
@@ -14533,7 +14533,7 @@
         </is>
       </c>
       <c r="E504" s="7" t="n">
-        <v>909</v>
+        <v>959</v>
       </c>
     </row>
     <row r="505">
@@ -14558,7 +14558,7 @@
         </is>
       </c>
       <c r="E505" s="7" t="n">
-        <v>819</v>
+        <v>870</v>
       </c>
     </row>
     <row r="506">
@@ -14583,7 +14583,7 @@
         </is>
       </c>
       <c r="E506" s="7" t="n">
-        <v>678</v>
+        <v>699</v>
       </c>
     </row>
     <row r="507">
@@ -14608,7 +14608,7 @@
         </is>
       </c>
       <c r="E507" s="7" t="n">
-        <v>484</v>
+        <v>506</v>
       </c>
     </row>
     <row r="508">
@@ -14633,7 +14633,7 @@
         </is>
       </c>
       <c r="E508" s="7" t="n">
-        <v>404</v>
+        <v>444</v>
       </c>
     </row>
     <row r="509">
@@ -14658,7 +14658,7 @@
         </is>
       </c>
       <c r="E509" s="7" t="n">
-        <v>214</v>
+        <v>230</v>
       </c>
     </row>
     <row r="510">
@@ -14683,7 +14683,7 @@
         </is>
       </c>
       <c r="E510" s="7" t="n">
-        <v>150</v>
+        <v>165</v>
       </c>
     </row>
     <row r="511">
@@ -14708,7 +14708,7 @@
         </is>
       </c>
       <c r="E511" s="7" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="512">
@@ -14733,7 +14733,7 @@
         </is>
       </c>
       <c r="E512" s="7" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
     </row>
     <row r="513">
@@ -14758,7 +14758,7 @@
         </is>
       </c>
       <c r="E513" s="7" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="514">
@@ -14783,7 +14783,7 @@
         </is>
       </c>
       <c r="E514" s="7" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="515">
@@ -14808,7 +14808,7 @@
         </is>
       </c>
       <c r="E515" s="7" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="516">
@@ -14833,7 +14833,7 @@
         </is>
       </c>
       <c r="E516" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="517">
@@ -14858,7 +14858,7 @@
         </is>
       </c>
       <c r="E517" s="7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="518">
@@ -14908,7 +14908,7 @@
         </is>
       </c>
       <c r="E519" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="520">
@@ -14933,7 +14933,7 @@
         </is>
       </c>
       <c r="E520" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="521">
@@ -14958,7 +14958,7 @@
         </is>
       </c>
       <c r="E521" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="522">
@@ -15004,11 +15004,11 @@
       </c>
       <c r="D523" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E523" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="524">
@@ -15024,16 +15024,16 @@
       </c>
       <c r="C524" s="4" t="inlineStr">
         <is>
-          <t>Menú / Home</t>
+          <t>Productos Vida</t>
         </is>
       </c>
       <c r="D524" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E524" s="7" t="n">
-        <v>1995</v>
+        <v>2</v>
       </c>
     </row>
     <row r="525">
@@ -15054,11 +15054,11 @@
       </c>
       <c r="D525" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E525" s="7" t="n">
-        <v>350</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="526">
@@ -15079,11 +15079,11 @@
       </c>
       <c r="D526" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E526" s="7" t="n">
-        <v>331</v>
+        <v>350</v>
       </c>
     </row>
     <row r="527">
@@ -15104,11 +15104,11 @@
       </c>
       <c r="D527" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E527" s="7" t="n">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="528">
@@ -15129,11 +15129,11 @@
       </c>
       <c r="D528" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E528" s="7" t="n">
-        <v>302</v>
+        <v>315</v>
       </c>
     </row>
     <row r="529">
@@ -15154,11 +15154,11 @@
       </c>
       <c r="D529" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E529" s="7" t="n">
-        <v>272</v>
+        <v>302</v>
       </c>
     </row>
     <row r="530">
@@ -15179,11 +15179,11 @@
       </c>
       <c r="D530" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E530" s="7" t="n">
-        <v>200</v>
+        <v>272</v>
       </c>
     </row>
     <row r="531">
@@ -15204,11 +15204,11 @@
       </c>
       <c r="D531" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E531" s="7" t="n">
-        <v>168</v>
+        <v>200</v>
       </c>
     </row>
     <row r="532">
@@ -15229,11 +15229,11 @@
       </c>
       <c r="D532" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E532" s="7" t="n">
-        <v>155</v>
+        <v>168</v>
       </c>
     </row>
     <row r="533">
@@ -15254,11 +15254,11 @@
       </c>
       <c r="D533" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E533" s="7" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="534">
@@ -15279,11 +15279,11 @@
       </c>
       <c r="D534" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E534" s="7" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="535">
@@ -15304,11 +15304,11 @@
       </c>
       <c r="D535" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E535" s="7" t="n">
-        <v>71</v>
+        <v>146</v>
       </c>
     </row>
     <row r="536">
@@ -15329,11 +15329,11 @@
       </c>
       <c r="D536" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E536" s="7" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
     </row>
     <row r="537">
@@ -15354,11 +15354,11 @@
       </c>
       <c r="D537" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E537" s="7" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
     </row>
     <row r="538">
@@ -15379,11 +15379,11 @@
       </c>
       <c r="D538" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E538" s="7" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="539">
@@ -15404,7 +15404,7 @@
       </c>
       <c r="D539" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E539" s="7" t="n">
@@ -15429,11 +15429,11 @@
       </c>
       <c r="D540" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E540" s="7" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="541">
@@ -15449,16 +15449,16 @@
       </c>
       <c r="C541" s="4" t="inlineStr">
         <is>
-          <t>Productos Líneas Personales</t>
+          <t>Menú / Home</t>
         </is>
       </c>
       <c r="D541" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E541" s="7" t="n">
-        <v>285</v>
+        <v>3</v>
       </c>
     </row>
     <row r="542">
@@ -15479,11 +15479,11 @@
       </c>
       <c r="D542" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E542" s="7" t="n">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="543">
@@ -15504,11 +15504,11 @@
       </c>
       <c r="D543" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E543" s="7" t="n">
-        <v>266</v>
+        <v>282</v>
       </c>
     </row>
     <row r="544">
@@ -15529,11 +15529,11 @@
       </c>
       <c r="D544" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E544" s="7" t="n">
-        <v>132</v>
+        <v>266</v>
       </c>
     </row>
     <row r="545">
@@ -15554,7 +15554,7 @@
       </c>
       <c r="D545" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E545" s="7" t="n">
@@ -15579,11 +15579,11 @@
       </c>
       <c r="D546" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E546" s="7" t="n">
-        <v>107</v>
+        <v>132</v>
       </c>
     </row>
     <row r="547">
@@ -15604,11 +15604,11 @@
       </c>
       <c r="D547" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E547" s="7" t="n">
-        <v>48</v>
+        <v>107</v>
       </c>
     </row>
     <row r="548">
@@ -15629,11 +15629,11 @@
       </c>
       <c r="D548" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E548" s="7" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="549">
@@ -15654,11 +15654,11 @@
       </c>
       <c r="D549" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E549" s="7" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
     </row>
     <row r="550">
@@ -15679,11 +15679,11 @@
       </c>
       <c r="D550" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E550" s="7" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="551">
@@ -15704,7 +15704,7 @@
       </c>
       <c r="D551" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E551" s="7" t="n">
@@ -15729,11 +15729,11 @@
       </c>
       <c r="D552" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E552" s="7" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="553">
@@ -15754,11 +15754,11 @@
       </c>
       <c r="D553" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E553" s="7" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="554">
@@ -15779,11 +15779,11 @@
       </c>
       <c r="D554" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E554" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="555">
@@ -15804,11 +15804,11 @@
       </c>
       <c r="D555" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E555" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="556">
@@ -15829,11 +15829,11 @@
       </c>
       <c r="D556" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E556" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="557">
@@ -15854,11 +15854,11 @@
       </c>
       <c r="D557" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E557" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="558">
@@ -15879,11 +15879,11 @@
       </c>
       <c r="D558" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E558" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="559">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="D559" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E559" s="7" t="n">
@@ -15929,11 +15929,11 @@
       </c>
       <c r="D560" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E560" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="561">
@@ -15954,7 +15954,7 @@
       </c>
       <c r="D561" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E561" s="7" t="n">
@@ -15964,26 +15964,26 @@
     <row r="562">
       <c r="A562" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="B562" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="C562" s="4" t="inlineStr">
         <is>
-          <t>Landing Alianzas</t>
+          <t>Productos Líneas Personales</t>
         </is>
       </c>
       <c r="D562" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E562" s="7" t="n">
-        <v>570</v>
+        <v>2</v>
       </c>
     </row>
     <row r="563">
@@ -16004,11 +16004,11 @@
       </c>
       <c r="D563" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E563" s="7" t="n">
-        <v>188</v>
+        <v>570</v>
       </c>
     </row>
     <row r="564">
@@ -16029,11 +16029,11 @@
       </c>
       <c r="D564" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E564" s="7" t="n">
-        <v>128</v>
+        <v>188</v>
       </c>
     </row>
     <row r="565">
@@ -16054,11 +16054,11 @@
       </c>
       <c r="D565" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E565" s="7" t="n">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="566">
@@ -16079,11 +16079,11 @@
       </c>
       <c r="D566" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E566" s="7" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="567">
@@ -16104,11 +16104,11 @@
       </c>
       <c r="D567" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E567" s="7" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="568">
@@ -16129,7 +16129,7 @@
       </c>
       <c r="D568" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E568" s="7" t="n">
@@ -16154,11 +16154,11 @@
       </c>
       <c r="D569" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E569" s="7" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="570">
@@ -16179,11 +16179,11 @@
       </c>
       <c r="D570" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E570" s="7" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="571">
@@ -16204,11 +16204,11 @@
       </c>
       <c r="D571" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E571" s="7" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="572">
@@ -16229,11 +16229,11 @@
       </c>
       <c r="D572" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E572" s="7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="573">
@@ -16254,11 +16254,11 @@
       </c>
       <c r="D573" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E573" s="7" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="574">
@@ -16279,11 +16279,11 @@
       </c>
       <c r="D574" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E574" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="575">
@@ -16304,11 +16304,11 @@
       </c>
       <c r="D575" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E575" s="7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="576">
@@ -16329,7 +16329,7 @@
       </c>
       <c r="D576" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E576" s="7" t="n">
@@ -16354,7 +16354,7 @@
       </c>
       <c r="D577" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E577" s="7" t="n">
@@ -16379,11 +16379,11 @@
       </c>
       <c r="D578" s="5" t="inlineStr">
         <is>
-          <t>Logo Horizontal</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E578" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="579">
@@ -16404,11 +16404,11 @@
       </c>
       <c r="D579" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Logo Horizontal</t>
         </is>
       </c>
       <c r="E579" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="580">
@@ -16429,10 +16429,35 @@
       </c>
       <c r="D580" s="5" t="inlineStr">
         <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="E580" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B581" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C581" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D581" s="5" t="inlineStr">
+        <is>
           <t>Calendar</t>
         </is>
       </c>
-      <c r="E580" s="7" t="n">
+      <c r="E581" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21335,7 +21360,7 @@
         </is>
       </c>
       <c r="D244" s="12" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="245">
@@ -21355,7 +21380,7 @@
         </is>
       </c>
       <c r="D245" s="12" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="246">
@@ -21375,7 +21400,7 @@
         </is>
       </c>
       <c r="D246" s="12" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="247">
@@ -21395,7 +21420,7 @@
         </is>
       </c>
       <c r="D247" s="12" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="248">
@@ -21455,7 +21480,7 @@
         </is>
       </c>
       <c r="D250" s="12" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="251">
@@ -21475,7 +21500,7 @@
         </is>
       </c>
       <c r="D251" s="12" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="252">
@@ -21535,7 +21560,7 @@
         </is>
       </c>
       <c r="D254" s="12" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="255">
@@ -21555,7 +21580,7 @@
         </is>
       </c>
       <c r="D255" s="12" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="256">
@@ -21571,7 +21596,7 @@
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>Car</t>
+          <t>submenu</t>
         </is>
       </c>
       <c r="D256" s="12" t="n">
@@ -21591,11 +21616,11 @@
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Car</t>
         </is>
       </c>
       <c r="D257" s="12" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="258">
@@ -21611,7 +21636,7 @@
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>MedicalService</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="D258" s="12" t="n">
@@ -21631,11 +21656,11 @@
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>submenu</t>
+          <t>MedicalService</t>
         </is>
       </c>
       <c r="D259" s="12" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="260">
@@ -21655,7 +21680,7 @@
         </is>
       </c>
       <c r="D260" s="12" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="261">
@@ -21675,7 +21700,7 @@
         </is>
       </c>
       <c r="D261" s="12" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="262">
@@ -22162,7 +22187,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
@@ -22234,7 +22259,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -22270,7 +22295,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -22306,7 +22331,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -22342,7 +22367,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -22354,10 +22379,10 @@
         <v>44</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>172968</v>
+        <v>172970</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>184320</v>
+        <v>184326</v>
       </c>
     </row>
     <row r="8">
@@ -22378,7 +22403,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -22414,7 +22439,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -22450,7 +22475,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -22486,7 +22511,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -22522,7 +22547,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -22558,7 +22583,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -22594,7 +22619,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -22630,7 +22655,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -22666,7 +22691,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -22675,13 +22700,13 @@
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>11118</v>
+        <v>11472</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>13184</v>
+        <v>13594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-23 17:37 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -533,7 +533,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  2026-06-22</t>
+          <t>Quarter: Q2 2026  |  2026-06-23</t>
         </is>
       </c>
     </row>
@@ -725,17 +725,17 @@
         <v>5</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>10716</v>
+        <v>8539</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>3008</v>
+        <v>1687</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>84%</t>
         </is>
       </c>
     </row>
@@ -757,10 +757,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>14009</v>
+        <v>14010</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7570</v>
+        <v>7576</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -917,10 +917,10 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>3596</v>
+        <v>3566</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>599</v>
+        <v>593</v>
       </c>
       <c r="G15" s="8" t="n">
         <v>29</v>
@@ -1457,17 +1457,17 @@
         <v>5</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10716</v>
+        <v>8539</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>3008</v>
+        <v>1687</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>84%</t>
         </is>
       </c>
     </row>
@@ -1559,13 +1559,13 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1951</v>
+        <v>1952</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
@@ -1729,10 +1729,10 @@
         <v>8</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>3596</v>
+        <v>3566</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>599</v>
+        <v>593</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>29</v>
@@ -7354,11 +7354,11 @@
       </c>
       <c r="D217" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E217" s="7" t="n">
-        <v>1543</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="218">
@@ -7379,11 +7379,11 @@
       </c>
       <c r="D218" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E218" s="7" t="n">
-        <v>1440</v>
+        <v>998</v>
       </c>
     </row>
     <row r="219">
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="E219" s="7" t="n">
-        <v>1363</v>
+        <v>993</v>
       </c>
     </row>
     <row r="220">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="E220" s="7" t="n">
-        <v>1346</v>
+        <v>976</v>
       </c>
     </row>
     <row r="221">
@@ -7458,7 +7458,7 @@
         </is>
       </c>
       <c r="E221" s="7" t="n">
-        <v>804</v>
+        <v>756</v>
       </c>
     </row>
     <row r="222">
@@ -7479,11 +7479,11 @@
       </c>
       <c r="D222" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E222" s="7" t="n">
-        <v>610</v>
+        <v>390</v>
       </c>
     </row>
     <row r="223">
@@ -7504,11 +7504,11 @@
       </c>
       <c r="D223" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E223" s="7" t="n">
-        <v>454</v>
+        <v>390</v>
       </c>
     </row>
     <row r="224">
@@ -7533,7 +7533,7 @@
         </is>
       </c>
       <c r="E224" s="7" t="n">
-        <v>445</v>
+        <v>289</v>
       </c>
     </row>
     <row r="225">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="E225" s="7" t="n">
-        <v>326</v>
+        <v>266</v>
       </c>
     </row>
     <row r="226">
@@ -7579,11 +7579,11 @@
       </c>
       <c r="D226" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E226" s="7" t="n">
-        <v>273</v>
+        <v>240</v>
       </c>
     </row>
     <row r="227">
@@ -7604,11 +7604,11 @@
       </c>
       <c r="D227" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E227" s="7" t="n">
-        <v>249</v>
+        <v>229</v>
       </c>
     </row>
     <row r="228">
@@ -7629,11 +7629,11 @@
       </c>
       <c r="D228" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E228" s="7" t="n">
-        <v>246</v>
+        <v>229</v>
       </c>
     </row>
     <row r="229">
@@ -7654,11 +7654,11 @@
       </c>
       <c r="D229" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E229" s="7" t="n">
-        <v>240</v>
+        <v>204</v>
       </c>
     </row>
     <row r="230">
@@ -7683,7 +7683,7 @@
         </is>
       </c>
       <c r="E230" s="7" t="n">
-        <v>209</v>
+        <v>199</v>
       </c>
     </row>
     <row r="231">
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="E231" s="7" t="n">
-        <v>200</v>
+        <v>152</v>
       </c>
     </row>
     <row r="232">
@@ -7779,11 +7779,11 @@
       </c>
       <c r="D234" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E234" s="7" t="n">
-        <v>108</v>
+        <v>60</v>
       </c>
     </row>
     <row r="235">
@@ -7804,11 +7804,11 @@
       </c>
       <c r="D235" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>Card Dashboard</t>
         </is>
       </c>
       <c r="E235" s="7" t="n">
-        <v>79</v>
+        <v>56</v>
       </c>
     </row>
     <row r="236">
@@ -7829,11 +7829,11 @@
       </c>
       <c r="D236" s="5" t="inlineStr">
         <is>
-          <t>Logo Horizontal</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E236" s="7" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
     </row>
     <row r="237">
@@ -7854,11 +7854,11 @@
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E237" s="7" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="238">
@@ -7879,11 +7879,11 @@
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E238" s="7" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="239">
@@ -7904,11 +7904,11 @@
       </c>
       <c r="D239" s="5" t="inlineStr">
         <is>
-          <t>Card Dashboard</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E239" s="7" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
     </row>
     <row r="240">
@@ -7929,11 +7929,11 @@
       </c>
       <c r="D240" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E240" s="7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="241">
@@ -7954,11 +7954,11 @@
       </c>
       <c r="D241" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Indicator Circle</t>
         </is>
       </c>
       <c r="E241" s="7" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="242">
@@ -7979,7 +7979,7 @@
       </c>
       <c r="D242" s="5" t="inlineStr">
         <is>
-          <t>Indicator Circle</t>
+          <t>Indicator number</t>
         </is>
       </c>
       <c r="E242" s="7" t="n">
@@ -8004,11 +8004,11 @@
       </c>
       <c r="D243" s="5" t="inlineStr">
         <is>
-          <t>Indicator number</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E243" s="7" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="244">
@@ -8029,11 +8029,11 @@
       </c>
       <c r="D244" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E244" s="7" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="245">
@@ -8054,11 +8054,11 @@
       </c>
       <c r="D245" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E245" s="7" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="246">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="D246" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E246" s="7" t="n">
@@ -8104,11 +8104,11 @@
       </c>
       <c r="D247" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E247" s="7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="248">
@@ -8129,11 +8129,11 @@
       </c>
       <c r="D248" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E248" s="7" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="249">
@@ -8154,36 +8154,36 @@
       </c>
       <c r="D249" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="E249" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día 2026</t>
         </is>
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Sidebar</t>
         </is>
       </c>
       <c r="E250" s="7" t="n">
-        <v>4</v>
+        <v>2929</v>
       </c>
     </row>
     <row r="251">
@@ -8204,11 +8204,11 @@
       </c>
       <c r="D251" s="5" t="inlineStr">
         <is>
-          <t>Sidebar</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E251" s="7" t="n">
-        <v>2929</v>
+        <v>685</v>
       </c>
     </row>
     <row r="252">
@@ -8229,11 +8229,11 @@
       </c>
       <c r="D252" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E252" s="7" t="n">
-        <v>685</v>
+        <v>653</v>
       </c>
     </row>
     <row r="253">
@@ -8254,11 +8254,11 @@
       </c>
       <c r="D253" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E253" s="7" t="n">
-        <v>653</v>
+        <v>553</v>
       </c>
     </row>
     <row r="254">
@@ -8279,11 +8279,11 @@
       </c>
       <c r="D254" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E254" s="7" t="n">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="255">
@@ -8304,11 +8304,11 @@
       </c>
       <c r="D255" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E255" s="7" t="n">
-        <v>551</v>
+        <v>512</v>
       </c>
     </row>
     <row r="256">
@@ -8329,11 +8329,11 @@
       </c>
       <c r="D256" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E256" s="7" t="n">
-        <v>512</v>
+        <v>347</v>
       </c>
     </row>
     <row r="257">
@@ -8354,11 +8354,11 @@
       </c>
       <c r="D257" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E257" s="7" t="n">
-        <v>347</v>
+        <v>335</v>
       </c>
     </row>
     <row r="258">
@@ -8379,11 +8379,11 @@
       </c>
       <c r="D258" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E258" s="7" t="n">
-        <v>335</v>
+        <v>187</v>
       </c>
     </row>
     <row r="259">
@@ -8404,11 +8404,11 @@
       </c>
       <c r="D259" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E259" s="7" t="n">
-        <v>187</v>
+        <v>145</v>
       </c>
     </row>
     <row r="260">
@@ -8429,11 +8429,11 @@
       </c>
       <c r="D260" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E260" s="7" t="n">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="261">
@@ -8454,11 +8454,11 @@
       </c>
       <c r="D261" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E261" s="7" t="n">
-        <v>139</v>
+        <v>120</v>
       </c>
     </row>
     <row r="262">
@@ -8479,11 +8479,11 @@
       </c>
       <c r="D262" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Indicator Circle</t>
         </is>
       </c>
       <c r="E262" s="7" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="263">
@@ -8504,11 +8504,11 @@
       </c>
       <c r="D263" s="5" t="inlineStr">
         <is>
-          <t>Indicator Circle</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E263" s="7" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="264">
@@ -8529,11 +8529,11 @@
       </c>
       <c r="D264" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E264" s="7" t="n">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="265">
@@ -8554,11 +8554,11 @@
       </c>
       <c r="D265" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Indicator number</t>
         </is>
       </c>
       <c r="E265" s="7" t="n">
-        <v>94</v>
+        <v>80</v>
       </c>
     </row>
     <row r="266">
@@ -8579,11 +8579,11 @@
       </c>
       <c r="D266" s="5" t="inlineStr">
         <is>
-          <t>Indicator number</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E266" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="267">
@@ -8604,11 +8604,11 @@
       </c>
       <c r="D267" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E267" s="7" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
     </row>
     <row r="268">
@@ -8629,11 +8629,11 @@
       </c>
       <c r="D268" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E268" s="7" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
     </row>
     <row r="269">
@@ -8654,11 +8654,11 @@
       </c>
       <c r="D269" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E269" s="7" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="270">
@@ -8679,11 +8679,11 @@
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E270" s="7" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="271">
@@ -8704,11 +8704,11 @@
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E271" s="7" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="272">
@@ -8729,11 +8729,11 @@
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="E272" s="7" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="273">
@@ -8754,11 +8754,11 @@
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E273" s="7" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="274">
@@ -8779,11 +8779,11 @@
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E274" s="7" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="275">
@@ -8804,11 +8804,11 @@
       </c>
       <c r="D275" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E275" s="7" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="276">
@@ -8829,7 +8829,7 @@
       </c>
       <c r="D276" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E276" s="7" t="n">
@@ -8854,11 +8854,11 @@
       </c>
       <c r="D277" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="E277" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="278">
@@ -8879,11 +8879,11 @@
       </c>
       <c r="D278" s="5" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="E278" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="279">
@@ -8904,7 +8904,7 @@
       </c>
       <c r="D279" s="5" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>Toggle</t>
         </is>
       </c>
       <c r="E279" s="7" t="n">
@@ -8929,11 +8929,11 @@
       </c>
       <c r="D280" s="5" t="inlineStr">
         <is>
-          <t>Toggle</t>
+          <t>Pagination</t>
         </is>
       </c>
       <c r="E280" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="281">
@@ -8954,11 +8954,11 @@
       </c>
       <c r="D281" s="5" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E281" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="282">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="D282" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Main Search</t>
         </is>
       </c>
       <c r="E282" s="7" t="n">
@@ -9004,11 +9004,11 @@
       </c>
       <c r="D283" s="5" t="inlineStr">
         <is>
-          <t>Main Search</t>
+          <t>File uploader</t>
         </is>
       </c>
       <c r="E283" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="284">
@@ -9024,16 +9024,16 @@
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>Modelo Día 2026</t>
+          <t>Portal de Suscripción &amp; Emisión</t>
         </is>
       </c>
       <c r="D284" s="5" t="inlineStr">
         <is>
-          <t>File uploader</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E284" s="7" t="n">
-        <v>2</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="285">
@@ -9054,11 +9054,11 @@
       </c>
       <c r="D285" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="E285" s="7" t="n">
-        <v>1316</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="286">
@@ -9079,11 +9079,11 @@
       </c>
       <c r="D286" s="5" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E286" s="7" t="n">
-        <v>1258</v>
+        <v>531</v>
       </c>
     </row>
     <row r="287">
@@ -9104,11 +9104,11 @@
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E287" s="7" t="n">
-        <v>531</v>
+        <v>184</v>
       </c>
     </row>
     <row r="288">
@@ -9129,11 +9129,11 @@
       </c>
       <c r="D288" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E288" s="7" t="n">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="289">
@@ -9154,11 +9154,11 @@
       </c>
       <c r="D289" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E289" s="7" t="n">
-        <v>178</v>
+        <v>161</v>
       </c>
     </row>
     <row r="290">
@@ -9179,11 +9179,11 @@
       </c>
       <c r="D290" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E290" s="7" t="n">
-        <v>161</v>
+        <v>126</v>
       </c>
     </row>
     <row r="291">
@@ -9204,11 +9204,11 @@
       </c>
       <c r="D291" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E291" s="7" t="n">
-        <v>126</v>
+        <v>107</v>
       </c>
     </row>
     <row r="292">
@@ -9229,11 +9229,11 @@
       </c>
       <c r="D292" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E292" s="7" t="n">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="293">
@@ -9254,11 +9254,11 @@
       </c>
       <c r="D293" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Pagination</t>
         </is>
       </c>
       <c r="E293" s="7" t="n">
-        <v>83</v>
+        <v>68</v>
       </c>
     </row>
     <row r="294">
@@ -9279,11 +9279,11 @@
       </c>
       <c r="D294" s="5" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E294" s="7" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="295">
@@ -9304,11 +9304,11 @@
       </c>
       <c r="D295" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E295" s="7" t="n">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="296">
@@ -9329,11 +9329,11 @@
       </c>
       <c r="D296" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E296" s="7" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="297">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D297" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E297" s="7" t="n">
@@ -9379,11 +9379,11 @@
       </c>
       <c r="D298" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E298" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="299">
@@ -9404,11 +9404,11 @@
       </c>
       <c r="D299" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E299" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="300">
@@ -9429,11 +9429,11 @@
       </c>
       <c r="D300" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E300" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="301">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="D301" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E301" s="7" t="n">
@@ -9479,7 +9479,7 @@
       </c>
       <c r="D302" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E302" s="7" t="n">
@@ -9504,7 +9504,7 @@
       </c>
       <c r="D303" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Chip Deleteable</t>
         </is>
       </c>
       <c r="E303" s="7" t="n">
@@ -9529,11 +9529,11 @@
       </c>
       <c r="D304" s="5" t="inlineStr">
         <is>
-          <t>Chip Deleteable</t>
+          <t>File uploader</t>
         </is>
       </c>
       <c r="E304" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="305">
@@ -9549,16 +9549,16 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Portal de Suscripción &amp; Emisión</t>
+          <t>Vida Ley &amp; SCTR</t>
         </is>
       </c>
       <c r="D305" s="5" t="inlineStr">
         <is>
-          <t>File uploader</t>
+          <t>Sidebar</t>
         </is>
       </c>
       <c r="E305" s="7" t="n">
-        <v>2</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="306">
@@ -9579,11 +9579,11 @@
       </c>
       <c r="D306" s="5" t="inlineStr">
         <is>
-          <t>Sidebar</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E306" s="7" t="n">
-        <v>1292</v>
+        <v>144</v>
       </c>
     </row>
     <row r="307">
@@ -9604,11 +9604,11 @@
       </c>
       <c r="D307" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E307" s="7" t="n">
-        <v>144</v>
+        <v>90</v>
       </c>
     </row>
     <row r="308">
@@ -9629,11 +9629,11 @@
       </c>
       <c r="D308" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E308" s="7" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
     </row>
     <row r="309">
@@ -9654,11 +9654,11 @@
       </c>
       <c r="D309" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E309" s="7" t="n">
-        <v>74</v>
+        <v>52</v>
       </c>
     </row>
     <row r="310">
@@ -9679,11 +9679,11 @@
       </c>
       <c r="D310" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E310" s="7" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="311">
@@ -9704,11 +9704,11 @@
       </c>
       <c r="D311" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E311" s="7" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="312">
@@ -9729,11 +9729,11 @@
       </c>
       <c r="D312" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E312" s="7" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="313">
@@ -9754,11 +9754,11 @@
       </c>
       <c r="D313" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E313" s="7" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="314">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="D314" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Indicator Circle</t>
         </is>
       </c>
       <c r="E314" s="7" t="n">
@@ -9804,11 +9804,11 @@
       </c>
       <c r="D315" s="5" t="inlineStr">
         <is>
-          <t>Indicator Circle</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E315" s="7" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="316">
@@ -9829,11 +9829,11 @@
       </c>
       <c r="D316" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E316" s="7" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="317">
@@ -9854,11 +9854,11 @@
       </c>
       <c r="D317" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E317" s="7" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="318">
@@ -9879,11 +9879,11 @@
       </c>
       <c r="D318" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E318" s="7" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="319">
@@ -9904,11 +9904,11 @@
       </c>
       <c r="D319" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Main Search</t>
         </is>
       </c>
       <c r="E319" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="320">
@@ -9929,11 +9929,11 @@
       </c>
       <c r="D320" s="5" t="inlineStr">
         <is>
-          <t>Main Search</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E320" s="7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="321">
@@ -9954,7 +9954,7 @@
       </c>
       <c r="D321" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Pagination</t>
         </is>
       </c>
       <c r="E321" s="7" t="n">
@@ -9979,11 +9979,11 @@
       </c>
       <c r="D322" s="5" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E322" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="323">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="D323" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E323" s="7" t="n">
@@ -10029,11 +10029,11 @@
       </c>
       <c r="D324" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="E324" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="325">
@@ -10054,11 +10054,11 @@
       </c>
       <c r="D325" s="5" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E325" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="326">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="D326" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="E326" s="7" t="n">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="D327" s="5" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="E327" s="7" t="n">
@@ -10129,11 +10129,11 @@
       </c>
       <c r="D328" s="5" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E328" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="329">
@@ -10154,11 +10154,11 @@
       </c>
       <c r="D329" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E329" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="330">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="D330" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E330" s="7" t="n">
@@ -10204,11 +10204,11 @@
       </c>
       <c r="D331" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E331" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="332">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="D332" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E332" s="7" t="n">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="D333" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E333" s="7" t="n">
@@ -10279,7 +10279,7 @@
       </c>
       <c r="D334" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E334" s="7" t="n">
@@ -10304,7 +10304,7 @@
       </c>
       <c r="D335" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E335" s="7" t="n">
@@ -13183,7 +13183,7 @@
         </is>
       </c>
       <c r="E450" s="7" t="n">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="451">
@@ -13204,11 +13204,11 @@
       </c>
       <c r="D451" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E451" s="7" t="n">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="452">
@@ -13229,11 +13229,11 @@
       </c>
       <c r="D452" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E452" s="7" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="453">
@@ -13254,11 +13254,11 @@
       </c>
       <c r="D453" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="E453" s="7" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="454">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="D454" s="5" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E454" s="7" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="455">
@@ -13358,7 +13358,7 @@
         </is>
       </c>
       <c r="E457" s="7" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="458">
@@ -18116,11 +18116,11 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Pegar Icon</t>
+          <t>DirectionDown</t>
         </is>
       </c>
       <c r="D82" s="12" t="n">
-        <v>499</v>
+        <v>233</v>
       </c>
     </row>
     <row r="83">
@@ -18136,11 +18136,11 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>copy</t>
+          <t>DirectionRight</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>454</v>
+        <v>198</v>
       </c>
     </row>
     <row r="84">
@@ -18156,11 +18156,11 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>DirectionDown</t>
+          <t>Option</t>
         </is>
       </c>
       <c r="D84" s="12" t="n">
-        <v>348</v>
+        <v>165</v>
       </c>
     </row>
     <row r="85">
@@ -18176,11 +18176,11 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>DirectionRight</t>
+          <t>Pegar Icon</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>281</v>
+        <v>102</v>
       </c>
     </row>
     <row r="86">
@@ -18196,11 +18196,11 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Component 9</t>
         </is>
       </c>
       <c r="D86" s="12" t="n">
-        <v>165</v>
+        <v>90</v>
       </c>
     </row>
     <row r="87">
@@ -18216,11 +18216,11 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>copy</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>95</v>
+        <v>57</v>
       </c>
     </row>
     <row r="88">
@@ -18236,11 +18236,11 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Component 9</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D88" s="12" t="n">
-        <v>94</v>
+        <v>37</v>
       </c>
     </row>
     <row r="89">
@@ -18256,11 +18256,11 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
     </row>
     <row r="90">
@@ -18276,11 +18276,11 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Frame 1707479054</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="D90" s="12" t="n">
-        <v>51</v>
+        <v>29</v>
       </c>
     </row>
     <row r="91">
@@ -18296,11 +18296,11 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>mail</t>
+          <t>Tooltip</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92">
@@ -18316,11 +18316,11 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Frame 1707479133</t>
+          <t>mail</t>
         </is>
       </c>
       <c r="D92" s="12" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="93">
@@ -18336,11 +18336,11 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>download</t>
+          <t>informacion de poliza</t>
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="94">
@@ -18356,11 +18356,11 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>datos personales</t>
         </is>
       </c>
       <c r="D94" s="12" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="95">
@@ -18376,11 +18376,11 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>informacion de poliza</t>
+          <t>soles</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="96">
@@ -18396,11 +18396,11 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>directionLeft</t>
         </is>
       </c>
       <c r="D96" s="12" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="97">
@@ -18416,11 +18416,11 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>datos personales</t>
+          <t>24.timer</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="98">
@@ -18436,11 +18436,11 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>dólares</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D98" s="12" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="99">
@@ -18456,11 +18456,11 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>directionLeft</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="100">
@@ -18476,11 +18476,11 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Tooltip</t>
+          <t>circle</t>
         </is>
       </c>
       <c r="D100" s="12" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="101">
@@ -18496,11 +18496,11 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>24.timer</t>
+          <t>Cargador circular</t>
         </is>
       </c>
       <c r="D101" s="12" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="102">
@@ -20676,11 +20676,11 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>mail</t>
+          <t>A.white</t>
         </is>
       </c>
       <c r="D210" s="12" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="211">
@@ -20696,7 +20696,7 @@
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>A.white</t>
+          <t>mail</t>
         </is>
       </c>
       <c r="D211" s="12" t="n">
@@ -20896,11 +20896,11 @@
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Seguridad_72x72</t>
+          <t>Emergencias</t>
         </is>
       </c>
       <c r="D221" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="222">
@@ -22187,7 +22187,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
@@ -22259,7 +22259,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -22295,7 +22295,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -22331,7 +22331,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -22343,10 +22343,10 @@
         <v>22</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>14009</v>
+        <v>14010</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>21579</v>
+        <v>21586</v>
       </c>
     </row>
     <row r="7">
@@ -22367,7 +22367,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -22403,22 +22403,22 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>84%</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>10716</v>
+        <v>8539</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>13724</v>
+        <v>10226</v>
       </c>
     </row>
     <row r="9">
@@ -22439,7 +22439,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -22475,7 +22475,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -22511,7 +22511,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -22547,7 +22547,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -22583,7 +22583,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -22619,7 +22619,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -22655,7 +22655,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -22667,10 +22667,10 @@
         <v>8</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3596</v>
+        <v>3566</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>4195</v>
+        <v>4159</v>
       </c>
     </row>
     <row r="16">
@@ -22691,7 +22691,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-23 22:31 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -821,10 +821,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2296</v>
+        <v>2301</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>28</v>
@@ -1627,10 +1627,10 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>2296</v>
+        <v>2301</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="G17" s="8" t="n">
         <v>28</v>
@@ -11033,7 +11033,7 @@
         </is>
       </c>
       <c r="E364" s="7" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="365">
@@ -11083,7 +11083,7 @@
         </is>
       </c>
       <c r="E366" s="7" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="367">
@@ -11158,7 +11158,7 @@
         </is>
       </c>
       <c r="E369" s="7" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="370">
@@ -22595,10 +22595,10 @@
         <v>1</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>2296</v>
+        <v>2301</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>3143</v>
+        <v>3147</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-24 17:26 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -533,7 +533,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  2026-06-23</t>
+          <t>Quarter: Q2 2026  |  2026-06-24</t>
         </is>
       </c>
     </row>
@@ -22187,7 +22187,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
@@ -22259,7 +22259,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -22295,7 +22295,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -22331,7 +22331,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -22367,7 +22367,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -22403,7 +22403,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -22439,7 +22439,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -22475,7 +22475,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -22511,7 +22511,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -22547,7 +22547,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -22583,7 +22583,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -22619,7 +22619,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -22655,7 +22655,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -22691,7 +22691,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-24 22:33 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -757,10 +757,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>14010</v>
+        <v>14454</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7576</v>
+        <v>7650</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -920,14 +920,14 @@
         <v>3566</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>593</v>
+        <v>638</v>
       </c>
       <c r="G15" s="8" t="n">
         <v>29</v>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>85%</t>
         </is>
       </c>
     </row>
@@ -1559,17 +1559,17 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1952</v>
+        <v>2396</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>467</v>
+        <v>541</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -1732,14 +1732,14 @@
         <v>3566</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>593</v>
+        <v>638</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>29</v>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>85%</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E581"/>
+  <dimension ref="A1:E580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9558,7 +9558,7 @@
         </is>
       </c>
       <c r="E305" s="7" t="n">
-        <v>1292</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="306">
@@ -9583,7 +9583,7 @@
         </is>
       </c>
       <c r="E306" s="7" t="n">
-        <v>144</v>
+        <v>191</v>
       </c>
     </row>
     <row r="307">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="E307" s="7" t="n">
-        <v>90</v>
+        <v>119</v>
       </c>
     </row>
     <row r="308">
@@ -9633,7 +9633,7 @@
         </is>
       </c>
       <c r="E308" s="7" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="309">
@@ -9654,11 +9654,11 @@
       </c>
       <c r="D309" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E309" s="7" t="n">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="310">
@@ -9679,11 +9679,11 @@
       </c>
       <c r="D310" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E310" s="7" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="311">
@@ -9708,7 +9708,7 @@
         </is>
       </c>
       <c r="E311" s="7" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="312">
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="E312" s="7" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="313">
@@ -9754,11 +9754,11 @@
       </c>
       <c r="D313" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E313" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="314">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="D314" s="5" t="inlineStr">
         <is>
-          <t>Indicator Circle</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E314" s="7" t="n">
@@ -9804,11 +9804,11 @@
       </c>
       <c r="D315" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Indicator Circle</t>
         </is>
       </c>
       <c r="E315" s="7" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="316">
@@ -9833,7 +9833,7 @@
         </is>
       </c>
       <c r="E316" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="317">
@@ -9879,7 +9879,7 @@
       </c>
       <c r="D318" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E318" s="7" t="n">
@@ -9904,11 +9904,11 @@
       </c>
       <c r="D319" s="5" t="inlineStr">
         <is>
-          <t>Main Search</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E319" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="320">
@@ -9929,11 +9929,11 @@
       </c>
       <c r="D320" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Main Search</t>
         </is>
       </c>
       <c r="E320" s="7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="321">
@@ -9979,11 +9979,11 @@
       </c>
       <c r="D322" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E322" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="323">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="D323" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E323" s="7" t="n">
@@ -10289,26 +10289,26 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>Modelo Día</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>Modelo Día</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Vida Ley &amp; SCTR</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="D335" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E335" s="7" t="n">
-        <v>1</v>
+        <v>305</v>
       </c>
     </row>
     <row r="336">
@@ -10329,11 +10329,11 @@
       </c>
       <c r="D336" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E336" s="7" t="n">
-        <v>305</v>
+        <v>243</v>
       </c>
     </row>
     <row r="337">
@@ -10354,11 +10354,11 @@
       </c>
       <c r="D337" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E337" s="7" t="n">
-        <v>243</v>
+        <v>164</v>
       </c>
     </row>
     <row r="338">
@@ -10379,11 +10379,11 @@
       </c>
       <c r="D338" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E338" s="7" t="n">
-        <v>164</v>
+        <v>110</v>
       </c>
     </row>
     <row r="339">
@@ -10404,11 +10404,11 @@
       </c>
       <c r="D339" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E339" s="7" t="n">
-        <v>110</v>
+        <v>83</v>
       </c>
     </row>
     <row r="340">
@@ -10429,11 +10429,11 @@
       </c>
       <c r="D340" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E340" s="7" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="341">
@@ -10454,11 +10454,11 @@
       </c>
       <c r="D341" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E341" s="7" t="n">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="342">
@@ -10479,11 +10479,11 @@
       </c>
       <c r="D342" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E342" s="7" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="343">
@@ -10504,11 +10504,11 @@
       </c>
       <c r="D343" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E343" s="7" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="344">
@@ -10529,7 +10529,7 @@
       </c>
       <c r="D344" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E344" s="7" t="n">
@@ -10554,11 +10554,11 @@
       </c>
       <c r="D345" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E345" s="7" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="346">
@@ -10579,11 +10579,11 @@
       </c>
       <c r="D346" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E346" s="7" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="347">
@@ -10604,11 +10604,11 @@
       </c>
       <c r="D347" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E347" s="7" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="348">
@@ -10629,11 +10629,11 @@
       </c>
       <c r="D348" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E348" s="7" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="349">
@@ -10654,11 +10654,11 @@
       </c>
       <c r="D349" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E349" s="7" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="350">
@@ -10679,11 +10679,11 @@
       </c>
       <c r="D350" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E350" s="7" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="351">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="D351" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E351" s="7" t="n">
@@ -10729,7 +10729,7 @@
       </c>
       <c r="D352" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E352" s="7" t="n">
@@ -10754,11 +10754,11 @@
       </c>
       <c r="D353" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E353" s="7" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="354">
@@ -10779,11 +10779,11 @@
       </c>
       <c r="D354" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E354" s="7" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="355">
@@ -10804,11 +10804,11 @@
       </c>
       <c r="D355" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E355" s="7" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="356">
@@ -10829,11 +10829,11 @@
       </c>
       <c r="D356" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E356" s="7" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="357">
@@ -10854,11 +10854,11 @@
       </c>
       <c r="D357" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="E357" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="358">
@@ -10879,11 +10879,11 @@
       </c>
       <c r="D358" s="5" t="inlineStr">
         <is>
-          <t>Bottom Bar</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E358" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="359">
@@ -10904,11 +10904,11 @@
       </c>
       <c r="D359" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E359" s="7" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="360">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="D360" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E360" s="7" t="n">
@@ -10954,11 +10954,11 @@
       </c>
       <c r="D361" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Links</t>
         </is>
       </c>
       <c r="E361" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="362">
@@ -10969,21 +10969,21 @@
       </c>
       <c r="B362" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="C362" s="4" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Vehicular</t>
         </is>
       </c>
       <c r="D362" s="5" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E362" s="7" t="n">
-        <v>1</v>
+        <v>433</v>
       </c>
     </row>
     <row r="363">
@@ -11004,11 +11004,11 @@
       </c>
       <c r="D363" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E363" s="7" t="n">
-        <v>433</v>
+        <v>217</v>
       </c>
     </row>
     <row r="364">
@@ -11029,11 +11029,11 @@
       </c>
       <c r="D364" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E364" s="7" t="n">
-        <v>217</v>
+        <v>196</v>
       </c>
     </row>
     <row r="365">
@@ -11054,11 +11054,11 @@
       </c>
       <c r="D365" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E365" s="7" t="n">
-        <v>196</v>
+        <v>176</v>
       </c>
     </row>
     <row r="366">
@@ -11079,11 +11079,11 @@
       </c>
       <c r="D366" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E366" s="7" t="n">
-        <v>176</v>
+        <v>149</v>
       </c>
     </row>
     <row r="367">
@@ -11104,11 +11104,11 @@
       </c>
       <c r="D367" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E367" s="7" t="n">
-        <v>149</v>
+        <v>124</v>
       </c>
     </row>
     <row r="368">
@@ -11129,11 +11129,11 @@
       </c>
       <c r="D368" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E368" s="7" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="369">
@@ -11154,11 +11154,11 @@
       </c>
       <c r="D369" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E369" s="7" t="n">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="370">
@@ -11179,11 +11179,11 @@
       </c>
       <c r="D370" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E370" s="7" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
     </row>
     <row r="371">
@@ -11204,11 +11204,11 @@
       </c>
       <c r="D371" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E371" s="7" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="372">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="D372" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E372" s="7" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="373">
@@ -11254,11 +11254,11 @@
       </c>
       <c r="D373" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E373" s="7" t="n">
-        <v>88</v>
+        <v>72</v>
       </c>
     </row>
     <row r="374">
@@ -11279,11 +11279,11 @@
       </c>
       <c r="D374" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E374" s="7" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="375">
@@ -11304,11 +11304,11 @@
       </c>
       <c r="D375" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E375" s="7" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="376">
@@ -11329,11 +11329,11 @@
       </c>
       <c r="D376" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E376" s="7" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="377">
@@ -11354,11 +11354,11 @@
       </c>
       <c r="D377" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E377" s="7" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="378">
@@ -11379,11 +11379,11 @@
       </c>
       <c r="D378" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E378" s="7" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="379">
@@ -11404,11 +11404,11 @@
       </c>
       <c r="D379" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E379" s="7" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="380">
@@ -11429,11 +11429,11 @@
       </c>
       <c r="D380" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E380" s="7" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="381">
@@ -11454,11 +11454,11 @@
       </c>
       <c r="D381" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E381" s="7" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="382">
@@ -11479,7 +11479,7 @@
       </c>
       <c r="D382" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E382" s="7" t="n">
@@ -11504,11 +11504,11 @@
       </c>
       <c r="D383" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E383" s="7" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="384">
@@ -11529,11 +11529,11 @@
       </c>
       <c r="D384" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E384" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="385">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="D385" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E385" s="7" t="n">
@@ -11579,11 +11579,11 @@
       </c>
       <c r="D386" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="E386" s="7" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="387">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="D387" s="5" t="inlineStr">
         <is>
-          <t>Bottom Bar</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E387" s="7" t="n">
@@ -11629,11 +11629,11 @@
       </c>
       <c r="D388" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E388" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="389">
@@ -11654,11 +11654,11 @@
       </c>
       <c r="D389" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Links</t>
         </is>
       </c>
       <c r="E389" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="390">
@@ -11669,21 +11669,21 @@
       </c>
       <c r="B390" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="C390" s="4" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>Auto Efectivo</t>
         </is>
       </c>
       <c r="D390" s="5" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E390" s="7" t="n">
-        <v>2</v>
+        <v>160</v>
       </c>
     </row>
     <row r="391">
@@ -11704,11 +11704,11 @@
       </c>
       <c r="D391" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E391" s="7" t="n">
-        <v>160</v>
+        <v>149</v>
       </c>
     </row>
     <row r="392">
@@ -11729,11 +11729,11 @@
       </c>
       <c r="D392" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E392" s="7" t="n">
-        <v>149</v>
+        <v>136</v>
       </c>
     </row>
     <row r="393">
@@ -11754,11 +11754,11 @@
       </c>
       <c r="D393" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E393" s="7" t="n">
-        <v>136</v>
+        <v>107</v>
       </c>
     </row>
     <row r="394">
@@ -11779,11 +11779,11 @@
       </c>
       <c r="D394" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E394" s="7" t="n">
-        <v>107</v>
+        <v>77</v>
       </c>
     </row>
     <row r="395">
@@ -11804,11 +11804,11 @@
       </c>
       <c r="D395" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E395" s="7" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
     </row>
     <row r="396">
@@ -11829,11 +11829,11 @@
       </c>
       <c r="D396" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E396" s="7" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="397">
@@ -11854,11 +11854,11 @@
       </c>
       <c r="D397" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E397" s="7" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="398">
@@ -11879,11 +11879,11 @@
       </c>
       <c r="D398" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E398" s="7" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="399">
@@ -11904,11 +11904,11 @@
       </c>
       <c r="D399" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="E399" s="7" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="400">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="D400" s="5" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E400" s="7" t="n">
@@ -11954,11 +11954,11 @@
       </c>
       <c r="D401" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E401" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="402">
@@ -11979,11 +11979,11 @@
       </c>
       <c r="D402" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E402" s="7" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="403">
@@ -12004,11 +12004,11 @@
       </c>
       <c r="D403" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E403" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="404">
@@ -12029,11 +12029,11 @@
       </c>
       <c r="D404" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E404" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="405">
@@ -12054,11 +12054,11 @@
       </c>
       <c r="D405" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E405" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="406">
@@ -12079,11 +12079,11 @@
       </c>
       <c r="D406" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E406" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="407">
@@ -12104,11 +12104,11 @@
       </c>
       <c r="D407" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E407" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="408">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="D408" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Infografia</t>
         </is>
       </c>
       <c r="E408" s="7" t="n">
@@ -12154,7 +12154,7 @@
       </c>
       <c r="D409" s="5" t="inlineStr">
         <is>
-          <t>Infografia</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E409" s="7" t="n">
@@ -12179,7 +12179,7 @@
       </c>
       <c r="D410" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E410" s="7" t="n">
@@ -12204,11 +12204,11 @@
       </c>
       <c r="D411" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E411" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="412">
@@ -12229,11 +12229,11 @@
       </c>
       <c r="D412" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E412" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="413">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D413" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E413" s="7" t="n">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="D414" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E414" s="7" t="n">
@@ -12294,21 +12294,21 @@
       </c>
       <c r="B415" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="C415" s="4" t="inlineStr">
         <is>
-          <t>Auto Efectivo</t>
+          <t>Vehicular Todo Riesgo</t>
         </is>
       </c>
       <c r="D415" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E415" s="7" t="n">
-        <v>1</v>
+        <v>597</v>
       </c>
     </row>
     <row r="416">
@@ -12329,11 +12329,11 @@
       </c>
       <c r="D416" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E416" s="7" t="n">
-        <v>597</v>
+        <v>331</v>
       </c>
     </row>
     <row r="417">
@@ -12354,11 +12354,11 @@
       </c>
       <c r="D417" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E417" s="7" t="n">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="418">
@@ -12379,11 +12379,11 @@
       </c>
       <c r="D418" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E418" s="7" t="n">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="419">
@@ -12404,11 +12404,11 @@
       </c>
       <c r="D419" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E419" s="7" t="n">
-        <v>276</v>
+        <v>166</v>
       </c>
     </row>
     <row r="420">
@@ -12429,11 +12429,11 @@
       </c>
       <c r="D420" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E420" s="7" t="n">
-        <v>166</v>
+        <v>151</v>
       </c>
     </row>
     <row r="421">
@@ -12454,11 +12454,11 @@
       </c>
       <c r="D421" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E421" s="7" t="n">
-        <v>151</v>
+        <v>116</v>
       </c>
     </row>
     <row r="422">
@@ -12479,11 +12479,11 @@
       </c>
       <c r="D422" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E422" s="7" t="n">
-        <v>116</v>
+        <v>70</v>
       </c>
     </row>
     <row r="423">
@@ -12504,11 +12504,11 @@
       </c>
       <c r="D423" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E423" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="424">
@@ -12529,11 +12529,11 @@
       </c>
       <c r="D424" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E424" s="7" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="425">
@@ -12554,11 +12554,11 @@
       </c>
       <c r="D425" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="E425" s="7" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="426">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="D426" s="5" t="inlineStr">
         <is>
-          <t>Cards</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E426" s="7" t="n">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="D427" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Left Label</t>
         </is>
       </c>
       <c r="E427" s="7" t="n">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="D428" s="5" t="inlineStr">
         <is>
-          <t>Left Label</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E428" s="7" t="n">
@@ -12654,7 +12654,7 @@
       </c>
       <c r="D429" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E429" s="7" t="n">
@@ -12679,11 +12679,11 @@
       </c>
       <c r="D430" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E430" s="7" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="431">
@@ -12704,11 +12704,11 @@
       </c>
       <c r="D431" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E431" s="7" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="432">
@@ -12729,11 +12729,11 @@
       </c>
       <c r="D432" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E432" s="7" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="433">
@@ -12754,11 +12754,11 @@
       </c>
       <c r="D433" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Links</t>
         </is>
       </c>
       <c r="E433" s="7" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="434">
@@ -12779,7 +12779,7 @@
       </c>
       <c r="D434" s="5" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E434" s="7" t="n">
@@ -12804,11 +12804,11 @@
       </c>
       <c r="D435" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E435" s="7" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="436">
@@ -12829,7 +12829,7 @@
       </c>
       <c r="D436" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Commercial Chips</t>
         </is>
       </c>
       <c r="E436" s="7" t="n">
@@ -12854,11 +12854,11 @@
       </c>
       <c r="D437" s="5" t="inlineStr">
         <is>
-          <t>Commercial Chips</t>
+          <t>Bottom Bar</t>
         </is>
       </c>
       <c r="E437" s="7" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="438">
@@ -12879,11 +12879,11 @@
       </c>
       <c r="D438" s="5" t="inlineStr">
         <is>
-          <t>Bottom Bar</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E438" s="7" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="439">
@@ -12904,11 +12904,11 @@
       </c>
       <c r="D439" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E439" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="440">
@@ -12929,7 +12929,7 @@
       </c>
       <c r="D440" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E440" s="7" t="n">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="D441" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E441" s="7" t="n">
@@ -12979,11 +12979,11 @@
       </c>
       <c r="D442" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E442" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="443">
@@ -13004,7 +13004,7 @@
       </c>
       <c r="D443" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Comparador</t>
         </is>
       </c>
       <c r="E443" s="7" t="n">
@@ -13019,21 +13019,21 @@
       </c>
       <c r="B444" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="C444" s="4" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="D444" s="5" t="inlineStr">
         <is>
-          <t>Comparador</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E444" s="7" t="n">
-        <v>2</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="445">
@@ -13054,11 +13054,11 @@
       </c>
       <c r="D445" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Menu Item</t>
         </is>
       </c>
       <c r="E445" s="7" t="n">
-        <v>1536</v>
+        <v>340</v>
       </c>
     </row>
     <row r="446">
@@ -13079,11 +13079,11 @@
       </c>
       <c r="D446" s="5" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E446" s="7" t="n">
-        <v>340</v>
+        <v>256</v>
       </c>
     </row>
     <row r="447">
@@ -13104,11 +13104,11 @@
       </c>
       <c r="D447" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E447" s="7" t="n">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="448">
@@ -13129,11 +13129,11 @@
       </c>
       <c r="D448" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E448" s="7" t="n">
-        <v>251</v>
+        <v>160</v>
       </c>
     </row>
     <row r="449">
@@ -13154,11 +13154,11 @@
       </c>
       <c r="D449" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E449" s="7" t="n">
-        <v>160</v>
+        <v>149</v>
       </c>
     </row>
     <row r="450">
@@ -13179,11 +13179,11 @@
       </c>
       <c r="D450" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E450" s="7" t="n">
-        <v>149</v>
+        <v>128</v>
       </c>
     </row>
     <row r="451">
@@ -13204,11 +13204,11 @@
       </c>
       <c r="D451" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E451" s="7" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="452">
@@ -13229,11 +13229,11 @@
       </c>
       <c r="D452" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="E452" s="7" t="n">
-        <v>122</v>
+        <v>85</v>
       </c>
     </row>
     <row r="453">
@@ -13254,11 +13254,11 @@
       </c>
       <c r="D453" s="5" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E453" s="7" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="454">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="D454" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E454" s="7" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
     </row>
     <row r="455">
@@ -13304,11 +13304,11 @@
       </c>
       <c r="D455" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E455" s="7" t="n">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="456">
@@ -13329,11 +13329,11 @@
       </c>
       <c r="D456" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E456" s="7" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="457">
@@ -13354,11 +13354,11 @@
       </c>
       <c r="D457" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E457" s="7" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="458">
@@ -13379,11 +13379,11 @@
       </c>
       <c r="D458" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E458" s="7" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="459">
@@ -13404,11 +13404,11 @@
       </c>
       <c r="D459" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Stepper</t>
         </is>
       </c>
       <c r="E459" s="7" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="460">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="D460" s="5" t="inlineStr">
         <is>
-          <t>Stepper</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E460" s="7" t="n">
@@ -13454,11 +13454,11 @@
       </c>
       <c r="D461" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Topbar</t>
         </is>
       </c>
       <c r="E461" s="7" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="462">
@@ -13479,7 +13479,7 @@
       </c>
       <c r="D462" s="5" t="inlineStr">
         <is>
-          <t>Topbar</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E462" s="7" t="n">
@@ -13504,11 +13504,11 @@
       </c>
       <c r="D463" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E463" s="7" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="464">
@@ -13529,11 +13529,11 @@
       </c>
       <c r="D464" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E464" s="7" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="465">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="D465" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E465" s="7" t="n">
@@ -13579,11 +13579,11 @@
       </c>
       <c r="D466" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E466" s="7" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="467">
@@ -13604,7 +13604,7 @@
       </c>
       <c r="D467" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E467" s="7" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="D468" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Bar Progress</t>
         </is>
       </c>
       <c r="E468" s="7" t="n">
@@ -13654,11 +13654,11 @@
       </c>
       <c r="D469" s="5" t="inlineStr">
         <is>
-          <t>Bar Progress</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E469" s="7" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="470">
@@ -13679,11 +13679,11 @@
       </c>
       <c r="D470" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E470" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="471">
@@ -13704,11 +13704,11 @@
       </c>
       <c r="D471" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E471" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="472">
@@ -13729,11 +13729,11 @@
       </c>
       <c r="D472" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E472" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="473">
@@ -13744,21 +13744,21 @@
       </c>
       <c r="B473" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="C473" s="4" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>VDT — Perfilador Productos Vida</t>
         </is>
       </c>
       <c r="D473" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E473" s="7" t="n">
-        <v>6</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="474">
@@ -13779,11 +13779,11 @@
       </c>
       <c r="D474" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E474" s="7" t="n">
-        <v>1152</v>
+        <v>618</v>
       </c>
     </row>
     <row r="475">
@@ -13804,11 +13804,11 @@
       </c>
       <c r="D475" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E475" s="7" t="n">
-        <v>618</v>
+        <v>440</v>
       </c>
     </row>
     <row r="476">
@@ -13829,11 +13829,11 @@
       </c>
       <c r="D476" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E476" s="7" t="n">
-        <v>440</v>
+        <v>375</v>
       </c>
     </row>
     <row r="477">
@@ -13854,11 +13854,11 @@
       </c>
       <c r="D477" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E477" s="7" t="n">
-        <v>375</v>
+        <v>192</v>
       </c>
     </row>
     <row r="478">
@@ -13879,11 +13879,11 @@
       </c>
       <c r="D478" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E478" s="7" t="n">
-        <v>192</v>
+        <v>120</v>
       </c>
     </row>
     <row r="479">
@@ -13904,11 +13904,11 @@
       </c>
       <c r="D479" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="E479" s="7" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="480">
@@ -13929,11 +13929,11 @@
       </c>
       <c r="D480" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E480" s="7" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="481">
@@ -13954,11 +13954,11 @@
       </c>
       <c r="D481" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E481" s="7" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="482">
@@ -13979,11 +13979,11 @@
       </c>
       <c r="D482" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E482" s="7" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="483">
@@ -14004,11 +14004,11 @@
       </c>
       <c r="D483" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Menu Item</t>
         </is>
       </c>
       <c r="E483" s="7" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="484">
@@ -14029,11 +14029,11 @@
       </c>
       <c r="D484" s="5" t="inlineStr">
         <is>
-          <t>Menu Item</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E484" s="7" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
     </row>
     <row r="485">
@@ -14054,11 +14054,11 @@
       </c>
       <c r="D485" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E485" s="7" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="486">
@@ -14079,11 +14079,11 @@
       </c>
       <c r="D486" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Label in</t>
         </is>
       </c>
       <c r="E486" s="7" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
     </row>
     <row r="487">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="D487" s="5" t="inlineStr">
         <is>
-          <t>Label in</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E487" s="7" t="n">
@@ -14129,11 +14129,11 @@
       </c>
       <c r="D488" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E488" s="7" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="489">
@@ -14154,11 +14154,11 @@
       </c>
       <c r="D489" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E489" s="7" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="490">
@@ -14179,11 +14179,11 @@
       </c>
       <c r="D490" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E490" s="7" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="491">
@@ -14204,11 +14204,11 @@
       </c>
       <c r="D491" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E491" s="7" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="492">
@@ -14229,11 +14229,11 @@
       </c>
       <c r="D492" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Chip Deleteable</t>
         </is>
       </c>
       <c r="E492" s="7" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="493">
@@ -14254,11 +14254,11 @@
       </c>
       <c r="D493" s="5" t="inlineStr">
         <is>
-          <t>Chip Deleteable</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E493" s="7" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="494">
@@ -14279,11 +14279,11 @@
       </c>
       <c r="D494" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="E494" s="7" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="495">
@@ -14304,11 +14304,11 @@
       </c>
       <c r="D495" s="5" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E495" s="7" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="496">
@@ -14329,11 +14329,11 @@
       </c>
       <c r="D496" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E496" s="7" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="497">
@@ -14354,7 +14354,7 @@
       </c>
       <c r="D497" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E497" s="7" t="n">
@@ -14379,7 +14379,7 @@
       </c>
       <c r="D498" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E498" s="7" t="n">
@@ -14404,11 +14404,11 @@
       </c>
       <c r="D499" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E499" s="7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="500">
@@ -14429,11 +14429,11 @@
       </c>
       <c r="D500" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Progress bar</t>
         </is>
       </c>
       <c r="E500" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="501">
@@ -14454,36 +14454,36 @@
       </c>
       <c r="D501" s="5" t="inlineStr">
         <is>
-          <t>Progress bar</t>
+          <t>Topbar</t>
         </is>
       </c>
       <c r="E501" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="B502" s="4" t="inlineStr">
         <is>
-          <t>VDT</t>
+          <t>Web Corporativa</t>
         </is>
       </c>
       <c r="C502" s="4" t="inlineStr">
         <is>
-          <t>VDT — Perfilador Productos Vida</t>
+          <t>Productos Vida</t>
         </is>
       </c>
       <c r="D502" s="5" t="inlineStr">
         <is>
-          <t>Topbar</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E502" s="7" t="n">
-        <v>4</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="503">
@@ -14504,11 +14504,11 @@
       </c>
       <c r="D503" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E503" s="7" t="n">
-        <v>1045</v>
+        <v>959</v>
       </c>
     </row>
     <row r="504">
@@ -14529,11 +14529,11 @@
       </c>
       <c r="D504" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E504" s="7" t="n">
-        <v>959</v>
+        <v>870</v>
       </c>
     </row>
     <row r="505">
@@ -14554,11 +14554,11 @@
       </c>
       <c r="D505" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E505" s="7" t="n">
-        <v>870</v>
+        <v>699</v>
       </c>
     </row>
     <row r="506">
@@ -14579,11 +14579,11 @@
       </c>
       <c r="D506" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E506" s="7" t="n">
-        <v>699</v>
+        <v>506</v>
       </c>
     </row>
     <row r="507">
@@ -14604,11 +14604,11 @@
       </c>
       <c r="D507" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E507" s="7" t="n">
-        <v>506</v>
+        <v>444</v>
       </c>
     </row>
     <row r="508">
@@ -14629,11 +14629,11 @@
       </c>
       <c r="D508" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E508" s="7" t="n">
-        <v>444</v>
+        <v>230</v>
       </c>
     </row>
     <row r="509">
@@ -14654,11 +14654,11 @@
       </c>
       <c r="D509" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E509" s="7" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
     </row>
     <row r="510">
@@ -14679,11 +14679,11 @@
       </c>
       <c r="D510" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E510" s="7" t="n">
-        <v>165</v>
+        <v>110</v>
       </c>
     </row>
     <row r="511">
@@ -14704,11 +14704,11 @@
       </c>
       <c r="D511" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E511" s="7" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="512">
@@ -14729,11 +14729,11 @@
       </c>
       <c r="D512" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E512" s="7" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="513">
@@ -14754,11 +14754,11 @@
       </c>
       <c r="D513" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E513" s="7" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="514">
@@ -14779,11 +14779,11 @@
       </c>
       <c r="D514" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E514" s="7" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
     </row>
     <row r="515">
@@ -14804,11 +14804,11 @@
       </c>
       <c r="D515" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E515" s="7" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="516">
@@ -14829,11 +14829,11 @@
       </c>
       <c r="D516" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E516" s="7" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="517">
@@ -14854,11 +14854,11 @@
       </c>
       <c r="D517" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E517" s="7" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="518">
@@ -14879,11 +14879,11 @@
       </c>
       <c r="D518" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E518" s="7" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="519">
@@ -14904,7 +14904,7 @@
       </c>
       <c r="D519" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E519" s="7" t="n">
@@ -14929,11 +14929,11 @@
       </c>
       <c r="D520" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E520" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="521">
@@ -14954,11 +14954,11 @@
       </c>
       <c r="D521" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E521" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="522">
@@ -14979,11 +14979,11 @@
       </c>
       <c r="D522" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E522" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="523">
@@ -15004,11 +15004,11 @@
       </c>
       <c r="D523" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E523" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="524">
@@ -15024,16 +15024,16 @@
       </c>
       <c r="C524" s="4" t="inlineStr">
         <is>
-          <t>Productos Vida</t>
+          <t>Menú / Home</t>
         </is>
       </c>
       <c r="D524" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E524" s="7" t="n">
-        <v>2</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="525">
@@ -15054,11 +15054,11 @@
       </c>
       <c r="D525" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E525" s="7" t="n">
-        <v>1995</v>
+        <v>350</v>
       </c>
     </row>
     <row r="526">
@@ -15079,11 +15079,11 @@
       </c>
       <c r="D526" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E526" s="7" t="n">
-        <v>350</v>
+        <v>331</v>
       </c>
     </row>
     <row r="527">
@@ -15104,11 +15104,11 @@
       </c>
       <c r="D527" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E527" s="7" t="n">
-        <v>331</v>
+        <v>315</v>
       </c>
     </row>
     <row r="528">
@@ -15129,11 +15129,11 @@
       </c>
       <c r="D528" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E528" s="7" t="n">
-        <v>315</v>
+        <v>302</v>
       </c>
     </row>
     <row r="529">
@@ -15154,11 +15154,11 @@
       </c>
       <c r="D529" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E529" s="7" t="n">
-        <v>302</v>
+        <v>272</v>
       </c>
     </row>
     <row r="530">
@@ -15179,11 +15179,11 @@
       </c>
       <c r="D530" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E530" s="7" t="n">
-        <v>272</v>
+        <v>200</v>
       </c>
     </row>
     <row r="531">
@@ -15204,11 +15204,11 @@
       </c>
       <c r="D531" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E531" s="7" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="532">
@@ -15229,11 +15229,11 @@
       </c>
       <c r="D532" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E532" s="7" t="n">
-        <v>168</v>
+        <v>155</v>
       </c>
     </row>
     <row r="533">
@@ -15254,11 +15254,11 @@
       </c>
       <c r="D533" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E533" s="7" t="n">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="534">
@@ -15279,11 +15279,11 @@
       </c>
       <c r="D534" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E534" s="7" t="n">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="535">
@@ -15304,11 +15304,11 @@
       </c>
       <c r="D535" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E535" s="7" t="n">
-        <v>146</v>
+        <v>71</v>
       </c>
     </row>
     <row r="536">
@@ -15329,11 +15329,11 @@
       </c>
       <c r="D536" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E536" s="7" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="537">
@@ -15354,11 +15354,11 @@
       </c>
       <c r="D537" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E537" s="7" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
     </row>
     <row r="538">
@@ -15379,11 +15379,11 @@
       </c>
       <c r="D538" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E538" s="7" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="539">
@@ -15404,7 +15404,7 @@
       </c>
       <c r="D539" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E539" s="7" t="n">
@@ -15429,11 +15429,11 @@
       </c>
       <c r="D540" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E540" s="7" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="541">
@@ -15449,16 +15449,16 @@
       </c>
       <c r="C541" s="4" t="inlineStr">
         <is>
-          <t>Menú / Home</t>
+          <t>Productos Líneas Personales</t>
         </is>
       </c>
       <c r="D541" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E541" s="7" t="n">
-        <v>3</v>
+        <v>285</v>
       </c>
     </row>
     <row r="542">
@@ -15479,11 +15479,11 @@
       </c>
       <c r="D542" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E542" s="7" t="n">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="543">
@@ -15504,11 +15504,11 @@
       </c>
       <c r="D543" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E543" s="7" t="n">
-        <v>282</v>
+        <v>266</v>
       </c>
     </row>
     <row r="544">
@@ -15529,11 +15529,11 @@
       </c>
       <c r="D544" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E544" s="7" t="n">
-        <v>266</v>
+        <v>132</v>
       </c>
     </row>
     <row r="545">
@@ -15554,7 +15554,7 @@
       </c>
       <c r="D545" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E545" s="7" t="n">
@@ -15579,11 +15579,11 @@
       </c>
       <c r="D546" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E546" s="7" t="n">
-        <v>132</v>
+        <v>107</v>
       </c>
     </row>
     <row r="547">
@@ -15604,11 +15604,11 @@
       </c>
       <c r="D547" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E547" s="7" t="n">
-        <v>107</v>
+        <v>48</v>
       </c>
     </row>
     <row r="548">
@@ -15629,11 +15629,11 @@
       </c>
       <c r="D548" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E548" s="7" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="549">
@@ -15654,11 +15654,11 @@
       </c>
       <c r="D549" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E549" s="7" t="n">
-        <v>45</v>
+        <v>24</v>
       </c>
     </row>
     <row r="550">
@@ -15679,11 +15679,11 @@
       </c>
       <c r="D550" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E550" s="7" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="551">
@@ -15704,7 +15704,7 @@
       </c>
       <c r="D551" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E551" s="7" t="n">
@@ -15729,11 +15729,11 @@
       </c>
       <c r="D552" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E552" s="7" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="553">
@@ -15754,11 +15754,11 @@
       </c>
       <c r="D553" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E553" s="7" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="554">
@@ -15779,11 +15779,11 @@
       </c>
       <c r="D554" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E554" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="555">
@@ -15804,11 +15804,11 @@
       </c>
       <c r="D555" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E555" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="556">
@@ -15829,11 +15829,11 @@
       </c>
       <c r="D556" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E556" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="557">
@@ -15854,11 +15854,11 @@
       </c>
       <c r="D557" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E557" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="558">
@@ -15879,11 +15879,11 @@
       </c>
       <c r="D558" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E558" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="559">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="D559" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E559" s="7" t="n">
@@ -15929,11 +15929,11 @@
       </c>
       <c r="D560" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E560" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="561">
@@ -15954,7 +15954,7 @@
       </c>
       <c r="D561" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E561" s="7" t="n">
@@ -15964,26 +15964,26 @@
     <row r="562">
       <c r="A562" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Embebidos</t>
         </is>
       </c>
       <c r="B562" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Embebidos</t>
         </is>
       </c>
       <c r="C562" s="4" t="inlineStr">
         <is>
-          <t>Productos Líneas Personales</t>
+          <t>Landing Alianzas</t>
         </is>
       </c>
       <c r="D562" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>type_option</t>
         </is>
       </c>
       <c r="E562" s="7" t="n">
-        <v>2</v>
+        <v>570</v>
       </c>
     </row>
     <row r="563">
@@ -16004,11 +16004,11 @@
       </c>
       <c r="D563" s="5" t="inlineStr">
         <is>
-          <t>type_option</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E563" s="7" t="n">
-        <v>570</v>
+        <v>188</v>
       </c>
     </row>
     <row r="564">
@@ -16029,11 +16029,11 @@
       </c>
       <c r="D564" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E564" s="7" t="n">
-        <v>188</v>
+        <v>128</v>
       </c>
     </row>
     <row r="565">
@@ -16054,11 +16054,11 @@
       </c>
       <c r="D565" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E565" s="7" t="n">
-        <v>128</v>
+        <v>100</v>
       </c>
     </row>
     <row r="566">
@@ -16079,11 +16079,11 @@
       </c>
       <c r="D566" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E566" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="567">
@@ -16104,11 +16104,11 @@
       </c>
       <c r="D567" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="E567" s="7" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
     <row r="568">
@@ -16129,7 +16129,7 @@
       </c>
       <c r="D568" s="5" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E568" s="7" t="n">
@@ -16154,11 +16154,11 @@
       </c>
       <c r="D569" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E569" s="7" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
     </row>
     <row r="570">
@@ -16179,11 +16179,11 @@
       </c>
       <c r="D570" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E570" s="7" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="571">
@@ -16204,11 +16204,11 @@
       </c>
       <c r="D571" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E571" s="7" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="572">
@@ -16229,11 +16229,11 @@
       </c>
       <c r="D572" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E572" s="7" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="573">
@@ -16254,11 +16254,11 @@
       </c>
       <c r="D573" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>src_option_stores_download</t>
         </is>
       </c>
       <c r="E573" s="7" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="574">
@@ -16279,11 +16279,11 @@
       </c>
       <c r="D574" s="5" t="inlineStr">
         <is>
-          <t>src_option_stores_download</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E574" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="575">
@@ -16304,11 +16304,11 @@
       </c>
       <c r="D575" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E575" s="7" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="576">
@@ -16329,7 +16329,7 @@
       </c>
       <c r="D576" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E576" s="7" t="n">
@@ -16354,7 +16354,7 @@
       </c>
       <c r="D577" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E577" s="7" t="n">
@@ -16379,11 +16379,11 @@
       </c>
       <c r="D578" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Logo Horizontal</t>
         </is>
       </c>
       <c r="E578" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="579">
@@ -16404,11 +16404,11 @@
       </c>
       <c r="D579" s="5" t="inlineStr">
         <is>
-          <t>Logo Horizontal</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E579" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="580">
@@ -16429,35 +16429,10 @@
       </c>
       <c r="D580" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E580" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="581">
-      <c r="A581" s="4" t="inlineStr">
-        <is>
-          <t>Embebidos</t>
-        </is>
-      </c>
-      <c r="B581" s="4" t="inlineStr">
-        <is>
-          <t>Embebidos</t>
-        </is>
-      </c>
-      <c r="C581" s="4" t="inlineStr">
-        <is>
-          <t>Landing Alianzas</t>
-        </is>
-      </c>
-      <c r="D581" s="5" t="inlineStr">
-        <is>
-          <t>Calendar</t>
-        </is>
-      </c>
-      <c r="E581" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -18676,11 +18651,11 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>barras</t>
         </is>
       </c>
       <c r="D110" s="12" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="111">
@@ -18696,11 +18671,11 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>DirectionUp</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="D111" s="12" t="n">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="112">
@@ -18716,11 +18691,11 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>barras</t>
+          <t>billetera</t>
         </is>
       </c>
       <c r="D112" s="12" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="113">
@@ -18736,11 +18711,11 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>billetera</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D113" s="12" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="114">
@@ -18756,11 +18731,11 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>create account</t>
         </is>
       </c>
       <c r="D114" s="12" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="115">
@@ -18776,11 +18751,11 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>create account</t>
+          <t>DirectionUp</t>
         </is>
       </c>
       <c r="D115" s="12" t="n">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="116">
@@ -18816,11 +18791,11 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>ArrowLeft</t>
         </is>
       </c>
       <c r="D117" s="12" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="118">
@@ -18836,11 +18811,11 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>ArrowLeft</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D118" s="12" t="n">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="119">
@@ -18856,11 +18831,11 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>directionLeft</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D119" s="12" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="120">
@@ -18876,11 +18851,11 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>download</t>
+          <t>directionLeft</t>
         </is>
       </c>
       <c r="D120" s="12" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="121">
@@ -20596,11 +20571,11 @@
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Indicator Mobile</t>
+          <t>DirectionDown</t>
         </is>
       </c>
       <c r="D206" s="12" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="207">
@@ -20616,7 +20591,7 @@
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Step 01</t>
+          <t>Indicator Mobile</t>
         </is>
       </c>
       <c r="D207" s="12" t="n">
@@ -20636,7 +20611,7 @@
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Step 02</t>
+          <t>Step 01</t>
         </is>
       </c>
       <c r="D208" s="12" t="n">
@@ -20656,7 +20631,7 @@
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>torito</t>
+          <t>Step 02</t>
         </is>
       </c>
       <c r="D209" s="12" t="n">
@@ -20676,11 +20651,11 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>A.white</t>
+          <t>torito</t>
         </is>
       </c>
       <c r="D210" s="12" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="211">
@@ -20696,7 +20671,7 @@
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>mail</t>
+          <t>A.white</t>
         </is>
       </c>
       <c r="D211" s="12" t="n">
@@ -20716,11 +20691,11 @@
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Viajeros</t>
+          <t>mail</t>
         </is>
       </c>
       <c r="D212" s="12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="213">
@@ -20736,11 +20711,11 @@
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>advertencia</t>
+          <t>iaSpark</t>
         </is>
       </c>
       <c r="D213" s="12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="214">
@@ -20756,11 +20731,11 @@
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>hiking</t>
+          <t>DirectionRight</t>
         </is>
       </c>
       <c r="D214" s="12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="215">
@@ -20776,11 +20751,11 @@
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Viajeros Mobile</t>
+          <t>Viajeros</t>
         </is>
       </c>
       <c r="D215" s="12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="216">
@@ -20796,11 +20771,11 @@
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Cancel Icon</t>
+          <t>advertencia</t>
         </is>
       </c>
       <c r="D216" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="217">
@@ -20816,11 +20791,11 @@
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Pasajeros</t>
+          <t>hiking</t>
         </is>
       </c>
       <c r="D217" s="12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="218">
@@ -20836,11 +20811,11 @@
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Spinner mesagge</t>
+          <t>Viajeros Mobile</t>
         </is>
       </c>
       <c r="D218" s="12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="219">
@@ -20856,11 +20831,11 @@
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Spinner</t>
+          <t>Cancel Icon</t>
         </is>
       </c>
       <c r="D219" s="12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="220">
@@ -20876,11 +20851,11 @@
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>DirectionUp</t>
+          <t>Pasajeros</t>
         </is>
       </c>
       <c r="D220" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221">
@@ -20896,11 +20871,11 @@
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Emergencias</t>
+          <t>Spinner mesagge</t>
         </is>
       </c>
       <c r="D221" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="222">
@@ -22343,10 +22318,10 @@
         <v>22</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>14010</v>
+        <v>14454</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>21586</v>
+        <v>22104</v>
       </c>
     </row>
     <row r="7">
@@ -22660,7 +22635,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="F15" s="6" t="n">
@@ -22670,7 +22645,7 @@
         <v>3566</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>4159</v>
+        <v>4204</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-26 22:27 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -661,17 +661,17 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>8343</v>
+        <v>7739</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>845</v>
+        <v>821</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>38</v>
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>90%</t>
         </is>
       </c>
     </row>
@@ -1353,17 +1353,17 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>1308</v>
+        <v>704</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>211</v>
+        <v>187</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>20</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>79%</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
         </is>
       </c>
       <c r="E88" s="7" t="n">
-        <v>576</v>
+        <v>192</v>
       </c>
     </row>
     <row r="89">
@@ -4224,7 +4224,7 @@
         </is>
       </c>
       <c r="E89" s="7" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
     </row>
     <row r="90">
@@ -4245,11 +4245,11 @@
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>section_footer</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
-        <v>96</v>
+        <v>73</v>
       </c>
     </row>
     <row r="91">
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="92">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
-        <v>85</v>
+        <v>48</v>
       </c>
     </row>
     <row r="93">
@@ -4320,11 +4320,11 @@
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="94">
@@ -4345,11 +4345,11 @@
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>reemplazar slot</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="95">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Slider Controls</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="96">
@@ -4395,11 +4395,11 @@
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>section_footer</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="97">
@@ -4420,11 +4420,11 @@
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>reemplazar slot</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
     </row>
     <row r="98">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>src_option_redes</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="99">
@@ -4470,11 +4470,11 @@
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Slider Controls</t>
+          <t>src_option_redes</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="100">
@@ -4495,11 +4495,11 @@
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>title_+_options</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="101">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>title_+_options</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="102">
@@ -4545,11 +4545,11 @@
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="103">
@@ -4570,11 +4570,11 @@
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Status Control</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="105">
@@ -4620,11 +4620,11 @@
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="106">
@@ -4645,11 +4645,11 @@
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>Status Control</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
@@ -17631,7 +17631,7 @@
         </is>
       </c>
       <c r="D43" s="12" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44">
@@ -17707,11 +17707,11 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>NorthEast</t>
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48">
@@ -17727,11 +17727,11 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>NorthEast</t>
+          <t>Menú_Desktop</t>
         </is>
       </c>
       <c r="D48" s="12" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49">
@@ -17747,11 +17747,11 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Menú_Desktop</t>
+          <t>Line Tracking Vertical</t>
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50">
@@ -17767,11 +17767,11 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Line Tracking Vertical</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="D50" s="12" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="51">
@@ -22735,17 +22735,17 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="F9" s="6" t="n">
         <v>8</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>8343</v>
+        <v>7739</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>9188</v>
+        <v>8560</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-29 17:56 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -533,7 +533,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  2026-06-26</t>
+          <t>Quarter: Q2 2026  |  2026-06-29</t>
         </is>
       </c>
     </row>
@@ -22478,7 +22478,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -22550,7 +22550,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -22586,7 +22586,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -22622,7 +22622,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -22658,7 +22658,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -22694,7 +22694,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -22730,7 +22730,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -22766,7 +22766,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -22802,7 +22802,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -22874,7 +22874,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -22910,7 +22910,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -22946,7 +22946,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -22982,7 +22982,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -23018,7 +23018,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-06-30 16:11 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Por archivo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Familias DS usadas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Internos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Historial" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Detach rate" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Familias DS usadas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Internos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Historial" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,8 +86,26 @@
       <color rgb="FFD94F3D"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF212529"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF6C757D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF8C8880"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1A7FA8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBA7517"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -142,7 +166,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -510,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -521,6 +553,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -533,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q2 2026  |  2026-06-29</t>
+          <t>Quarter: Q2 2026  |  2026-06-30</t>
         </is>
       </c>
     </row>
@@ -578,6 +611,11 @@
           <t>Adopción %</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Detach %</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -610,6 +648,11 @@
           <t>51%</t>
         </is>
       </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -642,6 +685,11 @@
           <t>87%</t>
         </is>
       </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -674,6 +722,11 @@
           <t>90%</t>
         </is>
       </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -706,6 +759,11 @@
           <t>94%</t>
         </is>
       </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -738,6 +796,11 @@
           <t>84%</t>
         </is>
       </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -757,10 +820,10 @@
         <v>22</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>14386</v>
+        <v>14419</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7654</v>
+        <v>7680</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -770,6 +833,11 @@
           <t>65%</t>
         </is>
       </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -802,6 +870,11 @@
           <t>75%</t>
         </is>
       </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -834,6 +907,11 @@
           <t>73%</t>
         </is>
       </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -866,6 +944,11 @@
           <t>0%</t>
         </is>
       </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -898,6 +981,11 @@
           <t>69%</t>
         </is>
       </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -930,6 +1018,11 @@
           <t>85%</t>
         </is>
       </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -962,6 +1055,11 @@
           <t>85%</t>
         </is>
       </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -981,7 +1079,7 @@
         <v>2</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>11371</v>
+        <v>11370</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>706</v>
@@ -994,6 +1092,11 @@
           <t>94%</t>
         </is>
       </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -1026,6 +1129,11 @@
           <t>84%</t>
         </is>
       </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1058,11 +1166,16 @@
           <t>88%</t>
         </is>
       </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1591,10 +1704,10 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2328</v>
+        <v>2361</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>545</v>
+        <v>571</v>
       </c>
       <c r="G15" s="8" t="n">
         <v>30</v>
@@ -1829,7 +1942,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>11371</v>
+        <v>11370</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>706</v>
@@ -1985,6 +2098,261 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Detach rate por categoría — Library Analytics API</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Fuente: Figma Library Analytics (Enterprise). Fórmula: detachments / (detachments + insertions) del quarter actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Detachments</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Insertions</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Total acciones</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Detach %</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>17415</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>17437</v>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Somos Corredores</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>31512</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>31599</v>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Protege 365</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>317</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>6526</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>6843</v>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Nueva Web Empresas</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>69191</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>69208</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Portal Digital de Siniestros</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>6637</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>6638</v>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Modelo Día</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>4334</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>4339</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>615</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>27625</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>28240</v>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>19514</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>19541</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>10670</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>10704</v>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9649,7 +10017,7 @@
         </is>
       </c>
       <c r="E306" s="7" t="n">
-        <v>188</v>
+        <v>209</v>
       </c>
     </row>
     <row r="307">
@@ -9699,7 +10067,7 @@
         </is>
       </c>
       <c r="E308" s="7" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="309">
@@ -9799,7 +10167,7 @@
         </is>
       </c>
       <c r="E312" s="7" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="313">
@@ -14549,7 +14917,7 @@
         </is>
       </c>
       <c r="E502" s="7" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="503">
@@ -16757,7 +17125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16810,7 +17178,7 @@
           <t>menú</t>
         </is>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="15" t="n">
         <v>1761</v>
       </c>
     </row>
@@ -16830,7 +17198,7 @@
           <t>card_accion</t>
         </is>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="15" t="n">
         <v>217</v>
       </c>
     </row>
@@ -16850,7 +17218,7 @@
           <t>card_atajo_home</t>
         </is>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="15" t="n">
         <v>212</v>
       </c>
     </row>
@@ -16870,7 +17238,7 @@
           <t>documento simple</t>
         </is>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="15" t="n">
         <v>100</v>
       </c>
     </row>
@@ -16890,7 +17258,7 @@
           <t>Seguros card</t>
         </is>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="15" t="n">
         <v>45</v>
       </c>
     </row>
@@ -16910,7 +17278,7 @@
           <t>Card_ beneficios</t>
         </is>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="15" t="n">
         <v>37</v>
       </c>
     </row>
@@ -16930,7 +17298,7 @@
           <t>beneficios vehiculares</t>
         </is>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="15" t="n">
         <v>36</v>
       </c>
     </row>
@@ -16950,7 +17318,7 @@
           <t>informacion de poliza</t>
         </is>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="15" t="n">
         <v>34</v>
       </c>
     </row>
@@ -16970,7 +17338,7 @@
           <t>carro</t>
         </is>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="15" t="n">
         <v>26</v>
       </c>
     </row>
@@ -16990,7 +17358,7 @@
           <t>buscar clínicas</t>
         </is>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="15" t="n">
         <v>26</v>
       </c>
     </row>
@@ -17010,7 +17378,7 @@
           <t>hogar</t>
         </is>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="15" t="n">
         <v>26</v>
       </c>
     </row>
@@ -17030,7 +17398,7 @@
           <t>drag</t>
         </is>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="15" t="n">
         <v>26</v>
       </c>
     </row>
@@ -17050,7 +17418,7 @@
           <t>Infotip</t>
         </is>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="15" t="n">
         <v>25</v>
       </c>
     </row>
@@ -17070,7 +17438,7 @@
           <t>error duda</t>
         </is>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -17090,7 +17458,7 @@
           <t>logo beneficios</t>
         </is>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -17110,7 +17478,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -17130,7 +17498,7 @@
           <t>Line Tracking Vertical</t>
         </is>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17150,7 +17518,7 @@
           <t>Bottom Navigation</t>
         </is>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -17170,7 +17538,7 @@
           <t>billetera</t>
         </is>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="15" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17190,7 +17558,7 @@
           <t>card_atajo</t>
         </is>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17210,7 +17578,7 @@
           <t>Suggested search (Deprecated)</t>
         </is>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="15" t="n">
         <v>65</v>
       </c>
     </row>
@@ -17230,7 +17598,7 @@
           <t>Step 01</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="15" t="n">
         <v>59</v>
       </c>
     </row>
@@ -17250,7 +17618,7 @@
           <t>Step 02</t>
         </is>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="D24" s="15" t="n">
         <v>59</v>
       </c>
     </row>
@@ -17270,7 +17638,7 @@
           <t>Step 03</t>
         </is>
       </c>
-      <c r="D25" s="12" t="n">
+      <c r="D25" s="15" t="n">
         <v>59</v>
       </c>
     </row>
@@ -17290,7 +17658,7 @@
           <t>celda L</t>
         </is>
       </c>
-      <c r="D26" s="12" t="n">
+      <c r="D26" s="15" t="n">
         <v>49</v>
       </c>
     </row>
@@ -17310,7 +17678,7 @@
           <t>Step 04</t>
         </is>
       </c>
-      <c r="D27" s="12" t="n">
+      <c r="D27" s="15" t="n">
         <v>39</v>
       </c>
     </row>
@@ -17330,7 +17698,7 @@
           <t>Step 05</t>
         </is>
       </c>
-      <c r="D28" s="12" t="n">
+      <c r="D28" s="15" t="n">
         <v>39</v>
       </c>
     </row>
@@ -17350,7 +17718,7 @@
           <t>Upload icon</t>
         </is>
       </c>
-      <c r="D29" s="12" t="n">
+      <c r="D29" s="15" t="n">
         <v>31</v>
       </c>
     </row>
@@ -17370,7 +17738,7 @@
           <t>Userflow</t>
         </is>
       </c>
-      <c r="D30" s="12" t="n">
+      <c r="D30" s="15" t="n">
         <v>27</v>
       </c>
     </row>
@@ -17390,7 +17758,7 @@
           <t>ArrowLeft</t>
         </is>
       </c>
-      <c r="D31" s="12" t="n">
+      <c r="D31" s="15" t="n">
         <v>21</v>
       </c>
     </row>
@@ -17410,7 +17778,7 @@
           <t>celda S</t>
         </is>
       </c>
-      <c r="D32" s="12" t="n">
+      <c r="D32" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17430,7 +17798,7 @@
           <t>File</t>
         </is>
       </c>
-      <c r="D33" s="12" t="n">
+      <c r="D33" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17450,7 +17818,7 @@
           <t>titulo-fila</t>
         </is>
       </c>
-      <c r="D34" s="12" t="n">
+      <c r="D34" s="15" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17470,7 +17838,7 @@
           <t>Respuesta</t>
         </is>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D35" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -17490,7 +17858,7 @@
           <t>Infotip</t>
         </is>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D36" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -17510,7 +17878,7 @@
           <t>audifonos</t>
         </is>
       </c>
-      <c r="D37" s="12" t="n">
+      <c r="D37" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -17530,7 +17898,7 @@
           <t>Container Drag and Drop</t>
         </is>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D38" s="15" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17550,7 +17918,7 @@
           <t>Option</t>
         </is>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D39" s="15" t="n">
         <v>6</v>
       </c>
     </row>
@@ -17570,7 +17938,7 @@
           <t>Page</t>
         </is>
       </c>
-      <c r="D40" s="12" t="n">
+      <c r="D40" s="15" t="n">
         <v>6</v>
       </c>
     </row>
@@ -17590,7 +17958,7 @@
           <t>DirectionUp</t>
         </is>
       </c>
-      <c r="D41" s="12" t="n">
+      <c r="D41" s="15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -17610,7 +17978,7 @@
           <t>HealthAndSafe</t>
         </is>
       </c>
-      <c r="D42" s="12" t="n">
+      <c r="D42" s="15" t="n">
         <v>96</v>
       </c>
     </row>
@@ -17630,7 +17998,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D43" s="12" t="n">
+      <c r="D43" s="15" t="n">
         <v>54</v>
       </c>
     </row>
@@ -17650,7 +18018,7 @@
           <t>Slider</t>
         </is>
       </c>
-      <c r="D44" s="12" t="n">
+      <c r="D44" s="15" t="n">
         <v>44</v>
       </c>
     </row>
@@ -17670,7 +18038,7 @@
           <t>Atajos | Beneficios (new)</t>
         </is>
       </c>
-      <c r="D45" s="12" t="n">
+      <c r="D45" s="15" t="n">
         <v>35</v>
       </c>
     </row>
@@ -17690,7 +18058,7 @@
           <t>Menu_Mobile</t>
         </is>
       </c>
-      <c r="D46" s="12" t="n">
+      <c r="D46" s="15" t="n">
         <v>34</v>
       </c>
     </row>
@@ -17710,7 +18078,7 @@
           <t>NorthEast</t>
         </is>
       </c>
-      <c r="D47" s="12" t="n">
+      <c r="D47" s="15" t="n">
         <v>32</v>
       </c>
     </row>
@@ -17730,7 +18098,7 @@
           <t>Menú_Desktop</t>
         </is>
       </c>
-      <c r="D48" s="12" t="n">
+      <c r="D48" s="15" t="n">
         <v>31</v>
       </c>
     </row>
@@ -17750,7 +18118,7 @@
           <t>Line Tracking Vertical</t>
         </is>
       </c>
-      <c r="D49" s="12" t="n">
+      <c r="D49" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -17770,7 +18138,7 @@
           <t>whatsapp</t>
         </is>
       </c>
-      <c r="D50" s="12" t="n">
+      <c r="D50" s="15" t="n">
         <v>29</v>
       </c>
     </row>
@@ -17790,7 +18158,7 @@
           <t>datos personales</t>
         </is>
       </c>
-      <c r="D51" s="12" t="n">
+      <c r="D51" s="15" t="n">
         <v>28</v>
       </c>
     </row>
@@ -17810,7 +18178,7 @@
           <t>beneficios reconocerte</t>
         </is>
       </c>
-      <c r="D52" s="12" t="n">
+      <c r="D52" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17830,7 +18198,7 @@
           <t>advertencia</t>
         </is>
       </c>
-      <c r="D53" s="12" t="n">
+      <c r="D53" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17850,7 +18218,7 @@
           <t>filter</t>
         </is>
       </c>
-      <c r="D54" s="12" t="n">
+      <c r="D54" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17870,7 +18238,7 @@
           <t>title_+_badges_download</t>
         </is>
       </c>
-      <c r="D55" s="12" t="n">
+      <c r="D55" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17890,7 +18258,7 @@
           <t>Feed</t>
         </is>
       </c>
-      <c r="D56" s="12" t="n">
+      <c r="D56" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17910,7 +18278,7 @@
           <t>Infotip</t>
         </is>
       </c>
-      <c r="D57" s="12" t="n">
+      <c r="D57" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -17930,7 +18298,7 @@
           <t>trofeo</t>
         </is>
       </c>
-      <c r="D58" s="12" t="n">
+      <c r="D58" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -17950,7 +18318,7 @@
           <t>vida ley</t>
         </is>
       </c>
-      <c r="D59" s="12" t="n">
+      <c r="D59" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -17970,7 +18338,7 @@
           <t>tratamiento</t>
         </is>
       </c>
-      <c r="D60" s="12" t="n">
+      <c r="D60" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -17990,7 +18358,7 @@
           <t>Right Label</t>
         </is>
       </c>
-      <c r="D61" s="12" t="n">
+      <c r="D61" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -18010,7 +18378,7 @@
           <t>celda S</t>
         </is>
       </c>
-      <c r="D62" s="12" t="n">
+      <c r="D62" s="15" t="n">
         <v>2366</v>
       </c>
     </row>
@@ -18030,7 +18398,7 @@
           <t>Icon</t>
         </is>
       </c>
-      <c r="D63" s="12" t="n">
+      <c r="D63" s="15" t="n">
         <v>699</v>
       </c>
     </row>
@@ -18050,7 +18418,7 @@
           <t>title_+_badges_download</t>
         </is>
       </c>
-      <c r="D64" s="12" t="n">
+      <c r="D64" s="15" t="n">
         <v>550</v>
       </c>
     </row>
@@ -18070,7 +18438,7 @@
           <t>Home_Header</t>
         </is>
       </c>
-      <c r="D65" s="12" t="n">
+      <c r="D65" s="15" t="n">
         <v>512</v>
       </c>
     </row>
@@ -18090,7 +18458,7 @@
           <t>Action 1</t>
         </is>
       </c>
-      <c r="D66" s="12" t="n">
+      <c r="D66" s="15" t="n">
         <v>496</v>
       </c>
     </row>
@@ -18110,7 +18478,7 @@
           <t>Action 2</t>
         </is>
       </c>
-      <c r="D67" s="12" t="n">
+      <c r="D67" s="15" t="n">
         <v>496</v>
       </c>
     </row>
@@ -18130,7 +18498,7 @@
           <t>Menu_Mobile</t>
         </is>
       </c>
-      <c r="D68" s="12" t="n">
+      <c r="D68" s="15" t="n">
         <v>482</v>
       </c>
     </row>
@@ -18150,7 +18518,7 @@
           <t>titulo-fila</t>
         </is>
       </c>
-      <c r="D69" s="12" t="n">
+      <c r="D69" s="15" t="n">
         <v>433</v>
       </c>
     </row>
@@ -18170,7 +18538,7 @@
           <t>Step 01</t>
         </is>
       </c>
-      <c r="D70" s="12" t="n">
+      <c r="D70" s="15" t="n">
         <v>398</v>
       </c>
     </row>
@@ -18190,7 +18558,7 @@
           <t>Step 02</t>
         </is>
       </c>
-      <c r="D71" s="12" t="n">
+      <c r="D71" s="15" t="n">
         <v>398</v>
       </c>
     </row>
@@ -18210,7 +18578,7 @@
           <t>Indicator Mobile</t>
         </is>
       </c>
-      <c r="D72" s="12" t="n">
+      <c r="D72" s="15" t="n">
         <v>390</v>
       </c>
     </row>
@@ -18230,7 +18598,7 @@
           <t>Step 03</t>
         </is>
       </c>
-      <c r="D73" s="12" t="n">
+      <c r="D73" s="15" t="n">
         <v>382</v>
       </c>
     </row>
@@ -18250,7 +18618,7 @@
           <t>save</t>
         </is>
       </c>
-      <c r="D74" s="12" t="n">
+      <c r="D74" s="15" t="n">
         <v>328</v>
       </c>
     </row>
@@ -18270,7 +18638,7 @@
           <t>Page</t>
         </is>
       </c>
-      <c r="D75" s="12" t="n">
+      <c r="D75" s="15" t="n">
         <v>324</v>
       </c>
     </row>
@@ -18290,7 +18658,7 @@
           <t>Control</t>
         </is>
       </c>
-      <c r="D76" s="12" t="n">
+      <c r="D76" s="15" t="n">
         <v>312</v>
       </c>
     </row>
@@ -18310,7 +18678,7 @@
           <t>Line Tracking Vertical</t>
         </is>
       </c>
-      <c r="D77" s="12" t="n">
+      <c r="D77" s="15" t="n">
         <v>295</v>
       </c>
     </row>
@@ -18330,7 +18698,7 @@
           <t>medios de pago</t>
         </is>
       </c>
-      <c r="D78" s="12" t="n">
+      <c r="D78" s="15" t="n">
         <v>280</v>
       </c>
     </row>
@@ -18350,7 +18718,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D79" s="12" t="n">
+      <c r="D79" s="15" t="n">
         <v>116</v>
       </c>
     </row>
@@ -18370,7 +18738,7 @@
           <t>add</t>
         </is>
       </c>
-      <c r="D80" s="12" t="n">
+      <c r="D80" s="15" t="n">
         <v>104</v>
       </c>
     </row>
@@ -18390,7 +18758,7 @@
           <t>width fixed pagination</t>
         </is>
       </c>
-      <c r="D81" s="12" t="n">
+      <c r="D81" s="15" t="n">
         <v>104</v>
       </c>
     </row>
@@ -18410,7 +18778,7 @@
           <t>DirectionDown</t>
         </is>
       </c>
-      <c r="D82" s="12" t="n">
+      <c r="D82" s="15" t="n">
         <v>233</v>
       </c>
     </row>
@@ -18430,7 +18798,7 @@
           <t>DirectionRight</t>
         </is>
       </c>
-      <c r="D83" s="12" t="n">
+      <c r="D83" s="15" t="n">
         <v>198</v>
       </c>
     </row>
@@ -18450,7 +18818,7 @@
           <t>Option</t>
         </is>
       </c>
-      <c r="D84" s="12" t="n">
+      <c r="D84" s="15" t="n">
         <v>165</v>
       </c>
     </row>
@@ -18470,7 +18838,7 @@
           <t>Pegar Icon</t>
         </is>
       </c>
-      <c r="D85" s="12" t="n">
+      <c r="D85" s="15" t="n">
         <v>102</v>
       </c>
     </row>
@@ -18490,7 +18858,7 @@
           <t>Component 9</t>
         </is>
       </c>
-      <c r="D86" s="12" t="n">
+      <c r="D86" s="15" t="n">
         <v>90</v>
       </c>
     </row>
@@ -18510,7 +18878,7 @@
           <t>copy</t>
         </is>
       </c>
-      <c r="D87" s="12" t="n">
+      <c r="D87" s="15" t="n">
         <v>57</v>
       </c>
     </row>
@@ -18530,7 +18898,7 @@
           <t>Icon</t>
         </is>
       </c>
-      <c r="D88" s="12" t="n">
+      <c r="D88" s="15" t="n">
         <v>37</v>
       </c>
     </row>
@@ -18550,7 +18918,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D89" s="12" t="n">
+      <c r="D89" s="15" t="n">
         <v>32</v>
       </c>
     </row>
@@ -18570,7 +18938,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="D90" s="12" t="n">
+      <c r="D90" s="15" t="n">
         <v>29</v>
       </c>
     </row>
@@ -18590,7 +18958,7 @@
           <t>Tooltip</t>
         </is>
       </c>
-      <c r="D91" s="12" t="n">
+      <c r="D91" s="15" t="n">
         <v>25</v>
       </c>
     </row>
@@ -18610,7 +18978,7 @@
           <t>mail</t>
         </is>
       </c>
-      <c r="D92" s="12" t="n">
+      <c r="D92" s="15" t="n">
         <v>25</v>
       </c>
     </row>
@@ -18630,7 +18998,7 @@
           <t>informacion de poliza</t>
         </is>
       </c>
-      <c r="D93" s="12" t="n">
+      <c r="D93" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -18650,7 +19018,7 @@
           <t>datos personales</t>
         </is>
       </c>
-      <c r="D94" s="12" t="n">
+      <c r="D94" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -18670,7 +19038,7 @@
           <t>soles</t>
         </is>
       </c>
-      <c r="D95" s="12" t="n">
+      <c r="D95" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -18690,7 +19058,7 @@
           <t>directionLeft</t>
         </is>
       </c>
-      <c r="D96" s="12" t="n">
+      <c r="D96" s="15" t="n">
         <v>22</v>
       </c>
     </row>
@@ -18710,7 +19078,7 @@
           <t>24.timer</t>
         </is>
       </c>
-      <c r="D97" s="12" t="n">
+      <c r="D97" s="15" t="n">
         <v>22</v>
       </c>
     </row>
@@ -18730,7 +19098,7 @@
           <t>File</t>
         </is>
       </c>
-      <c r="D98" s="12" t="n">
+      <c r="D98" s="15" t="n">
         <v>22</v>
       </c>
     </row>
@@ -18750,7 +19118,7 @@
           <t>Action</t>
         </is>
       </c>
-      <c r="D99" s="12" t="n">
+      <c r="D99" s="15" t="n">
         <v>19</v>
       </c>
     </row>
@@ -18770,7 +19138,7 @@
           <t>circle</t>
         </is>
       </c>
-      <c r="D100" s="12" t="n">
+      <c r="D100" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -18790,7 +19158,7 @@
           <t>Cargador circular</t>
         </is>
       </c>
-      <c r="D101" s="12" t="n">
+      <c r="D101" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -18810,7 +19178,7 @@
           <t>desk Table cell</t>
         </is>
       </c>
-      <c r="D102" s="12" t="n">
+      <c r="D102" s="15" t="n">
         <v>2624</v>
       </c>
     </row>
@@ -18830,8 +19198,8 @@
           <t>Control</t>
         </is>
       </c>
-      <c r="D103" s="12" t="n">
-        <v>643</v>
+      <c r="D103" s="15" t="n">
+        <v>636</v>
       </c>
     </row>
     <row r="104">
@@ -18850,7 +19218,7 @@
           <t>DirectionDown</t>
         </is>
       </c>
-      <c r="D104" s="12" t="n">
+      <c r="D104" s="15" t="n">
         <v>311</v>
       </c>
     </row>
@@ -18870,8 +19238,8 @@
           <t>Component 16</t>
         </is>
       </c>
-      <c r="D105" s="12" t="n">
-        <v>282</v>
+      <c r="D105" s="15" t="n">
+        <v>297</v>
       </c>
     </row>
     <row r="106">
@@ -18890,8 +19258,8 @@
           <t>Botón Primario</t>
         </is>
       </c>
-      <c r="D106" s="12" t="n">
-        <v>188</v>
+      <c r="D106" s="15" t="n">
+        <v>198</v>
       </c>
     </row>
     <row r="107">
@@ -18910,7 +19278,7 @@
           <t>Dropdown filter page</t>
         </is>
       </c>
-      <c r="D107" s="12" t="n">
+      <c r="D107" s="15" t="n">
         <v>159</v>
       </c>
     </row>
@@ -18930,7 +19298,7 @@
           <t>width fixed pagination</t>
         </is>
       </c>
-      <c r="D108" s="12" t="n">
+      <c r="D108" s="15" t="n">
         <v>159</v>
       </c>
     </row>
@@ -18950,7 +19318,7 @@
           <t>Line Tracking Vertical</t>
         </is>
       </c>
-      <c r="D109" s="12" t="n">
+      <c r="D109" s="15" t="n">
         <v>135</v>
       </c>
     </row>
@@ -18970,7 +19338,7 @@
           <t>barras</t>
         </is>
       </c>
-      <c r="D110" s="12" t="n">
+      <c r="D110" s="15" t="n">
         <v>127</v>
       </c>
     </row>
@@ -18990,7 +19358,7 @@
           <t>Article</t>
         </is>
       </c>
-      <c r="D111" s="12" t="n">
+      <c r="D111" s="15" t="n">
         <v>125</v>
       </c>
     </row>
@@ -19010,7 +19378,7 @@
           <t>billetera</t>
         </is>
       </c>
-      <c r="D112" s="12" t="n">
+      <c r="D112" s="15" t="n">
         <v>118</v>
       </c>
     </row>
@@ -19030,7 +19398,7 @@
           <t>description</t>
         </is>
       </c>
-      <c r="D113" s="12" t="n">
+      <c r="D113" s="15" t="n">
         <v>117</v>
       </c>
     </row>
@@ -19050,7 +19418,7 @@
           <t>DirectionUp</t>
         </is>
       </c>
-      <c r="D114" s="12" t="n">
+      <c r="D114" s="15" t="n">
         <v>116</v>
       </c>
     </row>
@@ -19070,7 +19438,7 @@
           <t>create account</t>
         </is>
       </c>
-      <c r="D115" s="12" t="n">
+      <c r="D115" s="15" t="n">
         <v>116</v>
       </c>
     </row>
@@ -19090,7 +19458,7 @@
           <t>ArrowLeft</t>
         </is>
       </c>
-      <c r="D116" s="12" t="n">
+      <c r="D116" s="15" t="n">
         <v>104</v>
       </c>
     </row>
@@ -19110,7 +19478,7 @@
           <t>Icon</t>
         </is>
       </c>
-      <c r="D117" s="12" t="n">
+      <c r="D117" s="15" t="n">
         <v>103</v>
       </c>
     </row>
@@ -19130,7 +19498,7 @@
           <t>Page</t>
         </is>
       </c>
-      <c r="D118" s="12" t="n">
+      <c r="D118" s="15" t="n">
         <v>102</v>
       </c>
     </row>
@@ -19150,8 +19518,8 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D119" s="12" t="n">
-        <v>98</v>
+      <c r="D119" s="15" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="120">
@@ -19167,11 +19535,11 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>directionLeft</t>
-        </is>
-      </c>
-      <c r="D120" s="12" t="n">
-        <v>96</v>
+          <t>BtnBackNext</t>
+        </is>
+      </c>
+      <c r="D120" s="15" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="121">
@@ -19187,11 +19555,11 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>AGENDA</t>
-        </is>
-      </c>
-      <c r="D121" s="12" t="n">
-        <v>92</v>
+          <t>directionLeft</t>
+        </is>
+      </c>
+      <c r="D121" s="15" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="122">
@@ -19210,7 +19578,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="D122" s="12" t="n">
+      <c r="D122" s="15" t="n">
         <v>41</v>
       </c>
     </row>
@@ -19230,7 +19598,7 @@
           <t>Indicator Mobile</t>
         </is>
       </c>
-      <c r="D123" s="12" t="n">
+      <c r="D123" s="15" t="n">
         <v>31</v>
       </c>
     </row>
@@ -19250,7 +19618,7 @@
           <t>torito</t>
         </is>
       </c>
-      <c r="D124" s="12" t="n">
+      <c r="D124" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -19270,7 +19638,7 @@
           <t>Infotip</t>
         </is>
       </c>
-      <c r="D125" s="12" t="n">
+      <c r="D125" s="15" t="n">
         <v>29</v>
       </c>
     </row>
@@ -19290,7 +19658,7 @@
           <t>number_deskop</t>
         </is>
       </c>
-      <c r="D126" s="12" t="n">
+      <c r="D126" s="15" t="n">
         <v>24</v>
       </c>
     </row>
@@ -19310,7 +19678,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="D127" s="12" t="n">
+      <c r="D127" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -19330,7 +19698,7 @@
           <t>eye_open</t>
         </is>
       </c>
-      <c r="D128" s="12" t="n">
+      <c r="D128" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -19350,7 +19718,7 @@
           <t>Step 01</t>
         </is>
       </c>
-      <c r="D129" s="12" t="n">
+      <c r="D129" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19370,7 +19738,7 @@
           <t>Step 02</t>
         </is>
       </c>
-      <c r="D130" s="12" t="n">
+      <c r="D130" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19390,7 +19758,7 @@
           <t>Step 03</t>
         </is>
       </c>
-      <c r="D131" s="12" t="n">
+      <c r="D131" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19410,7 +19778,7 @@
           <t>tarjeta de crédito</t>
         </is>
       </c>
-      <c r="D132" s="12" t="n">
+      <c r="D132" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19430,7 +19798,7 @@
           <t>Póliza Salud</t>
         </is>
       </c>
-      <c r="D133" s="12" t="n">
+      <c r="D133" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19450,7 +19818,7 @@
           <t>whatsapp</t>
         </is>
       </c>
-      <c r="D134" s="12" t="n">
+      <c r="D134" s="15" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19470,7 +19838,7 @@
           <t>Toast</t>
         </is>
       </c>
-      <c r="D135" s="12" t="n">
+      <c r="D135" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -19490,7 +19858,7 @@
           <t>face</t>
         </is>
       </c>
-      <c r="D136" s="12" t="n">
+      <c r="D136" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -19510,7 +19878,7 @@
           <t>soat</t>
         </is>
       </c>
-      <c r="D137" s="12" t="n">
+      <c r="D137" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -19530,7 +19898,7 @@
           <t>01_card selector</t>
         </is>
       </c>
-      <c r="D138" s="12" t="n">
+      <c r="D138" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -19550,7 +19918,7 @@
           <t>vehiculares</t>
         </is>
       </c>
-      <c r="D139" s="12" t="n">
+      <c r="D139" s="15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -19570,7 +19938,7 @@
           <t>Card_Cross_RT_Deskop_Cob</t>
         </is>
       </c>
-      <c r="D140" s="12" t="n">
+      <c r="D140" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -19590,7 +19958,7 @@
           <t>AddCard</t>
         </is>
       </c>
-      <c r="D141" s="12" t="n">
+      <c r="D141" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -19610,7 +19978,7 @@
           <t>02</t>
         </is>
       </c>
-      <c r="D142" s="12" t="n">
+      <c r="D142" s="15" t="n">
         <v>105</v>
       </c>
     </row>
@@ -19630,7 +19998,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="D143" s="12" t="n">
+      <c r="D143" s="15" t="n">
         <v>58</v>
       </c>
     </row>
@@ -19650,7 +20018,7 @@
           <t>add</t>
         </is>
       </c>
-      <c r="D144" s="12" t="n">
+      <c r="D144" s="15" t="n">
         <v>50</v>
       </c>
     </row>
@@ -19670,7 +20038,7 @@
           <t>whatsapp</t>
         </is>
       </c>
-      <c r="D145" s="12" t="n">
+      <c r="D145" s="15" t="n">
         <v>38</v>
       </c>
     </row>
@@ -19690,7 +20058,7 @@
           <t>Toast</t>
         </is>
       </c>
-      <c r="D146" s="12" t="n">
+      <c r="D146" s="15" t="n">
         <v>34</v>
       </c>
     </row>
@@ -19710,7 +20078,7 @@
           <t>Infotip</t>
         </is>
       </c>
-      <c r="D147" s="12" t="n">
+      <c r="D147" s="15" t="n">
         <v>28</v>
       </c>
     </row>
@@ -19730,7 +20098,7 @@
           <t>Smile</t>
         </is>
       </c>
-      <c r="D148" s="12" t="n">
+      <c r="D148" s="15" t="n">
         <v>25</v>
       </c>
     </row>
@@ -19750,7 +20118,7 @@
           <t>Image</t>
         </is>
       </c>
-      <c r="D149" s="12" t="n">
+      <c r="D149" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -19770,7 +20138,7 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="D150" s="12" t="n">
+      <c r="D150" s="15" t="n">
         <v>22</v>
       </c>
     </row>
@@ -19790,7 +20158,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="D151" s="12" t="n">
+      <c r="D151" s="15" t="n">
         <v>22</v>
       </c>
     </row>
@@ -19810,7 +20178,7 @@
           <t>eye_open</t>
         </is>
       </c>
-      <c r="D152" s="12" t="n">
+      <c r="D152" s="15" t="n">
         <v>21</v>
       </c>
     </row>
@@ -19830,7 +20198,7 @@
           <t>torito</t>
         </is>
       </c>
-      <c r="D153" s="12" t="n">
+      <c r="D153" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -19850,7 +20218,7 @@
           <t>tarjeta de crédito</t>
         </is>
       </c>
-      <c r="D154" s="12" t="n">
+      <c r="D154" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -19870,7 +20238,7 @@
           <t>asset_promo</t>
         </is>
       </c>
-      <c r="D155" s="12" t="n">
+      <c r="D155" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19890,7 +20258,7 @@
           <t>Indicator Mobile</t>
         </is>
       </c>
-      <c r="D156" s="12" t="n">
+      <c r="D156" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19910,7 +20278,7 @@
           <t>Image Frame</t>
         </is>
       </c>
-      <c r="D157" s="12" t="n">
+      <c r="D157" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19930,7 +20298,7 @@
           <t>Step 01</t>
         </is>
       </c>
-      <c r="D158" s="12" t="n">
+      <c r="D158" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -19950,7 +20318,7 @@
           <t>Step 02</t>
         </is>
       </c>
-      <c r="D159" s="12" t="n">
+      <c r="D159" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -19970,7 +20338,7 @@
           <t>Step 03</t>
         </is>
       </c>
-      <c r="D160" s="12" t="n">
+      <c r="D160" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -19990,7 +20358,7 @@
           <t>BtnAyuda</t>
         </is>
       </c>
-      <c r="D161" s="12" t="n">
+      <c r="D161" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20010,7 +20378,7 @@
           <t>add</t>
         </is>
       </c>
-      <c r="D162" s="12" t="n">
+      <c r="D162" s="15" t="n">
         <v>109</v>
       </c>
     </row>
@@ -20030,7 +20398,7 @@
           <t>02</t>
         </is>
       </c>
-      <c r="D163" s="12" t="n">
+      <c r="D163" s="15" t="n">
         <v>107</v>
       </c>
     </row>
@@ -20050,7 +20418,7 @@
           <t>Title</t>
         </is>
       </c>
-      <c r="D164" s="12" t="n">
+      <c r="D164" s="15" t="n">
         <v>78</v>
       </c>
     </row>
@@ -20070,7 +20438,7 @@
           <t>Toast</t>
         </is>
       </c>
-      <c r="D165" s="12" t="n">
+      <c r="D165" s="15" t="n">
         <v>72</v>
       </c>
     </row>
@@ -20090,7 +20458,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="D166" s="12" t="n">
+      <c r="D166" s="15" t="n">
         <v>60</v>
       </c>
     </row>
@@ -20110,7 +20478,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="D167" s="12" t="n">
+      <c r="D167" s="15" t="n">
         <v>40</v>
       </c>
     </row>
@@ -20130,7 +20498,7 @@
           <t>Smile</t>
         </is>
       </c>
-      <c r="D168" s="12" t="n">
+      <c r="D168" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -20150,7 +20518,7 @@
           <t>Car</t>
         </is>
       </c>
-      <c r="D169" s="12" t="n">
+      <c r="D169" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -20170,7 +20538,7 @@
           <t>Indicator Mobile</t>
         </is>
       </c>
-      <c r="D170" s="12" t="n">
+      <c r="D170" s="15" t="n">
         <v>24</v>
       </c>
     </row>
@@ -20190,7 +20558,7 @@
           <t>mail</t>
         </is>
       </c>
-      <c r="D171" s="12" t="n">
+      <c r="D171" s="15" t="n">
         <v>22</v>
       </c>
     </row>
@@ -20210,7 +20578,7 @@
           <t>Step 01</t>
         </is>
       </c>
-      <c r="D172" s="12" t="n">
+      <c r="D172" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -20230,7 +20598,7 @@
           <t>Step 02</t>
         </is>
       </c>
-      <c r="D173" s="12" t="n">
+      <c r="D173" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -20250,7 +20618,7 @@
           <t>Step 03</t>
         </is>
       </c>
-      <c r="D174" s="12" t="n">
+      <c r="D174" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -20270,7 +20638,7 @@
           <t>choque</t>
         </is>
       </c>
-      <c r="D175" s="12" t="n">
+      <c r="D175" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -20290,7 +20658,7 @@
           <t>Espejos</t>
         </is>
       </c>
-      <c r="D176" s="12" t="n">
+      <c r="D176" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -20310,7 +20678,7 @@
           <t>support</t>
         </is>
       </c>
-      <c r="D177" s="12" t="n">
+      <c r="D177" s="15" t="n">
         <v>20</v>
       </c>
     </row>
@@ -20330,7 +20698,7 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="D178" s="12" t="n">
+      <c r="D178" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -20350,7 +20718,7 @@
           <t>Image</t>
         </is>
       </c>
-      <c r="D179" s="12" t="n">
+      <c r="D179" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -20370,7 +20738,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="D180" s="12" t="n">
+      <c r="D180" s="15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -20390,7 +20758,7 @@
           <t>BtnAyuda</t>
         </is>
       </c>
-      <c r="D181" s="12" t="n">
+      <c r="D181" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -20410,7 +20778,7 @@
           <t>celda</t>
         </is>
       </c>
-      <c r="D182" s="12" t="n">
+      <c r="D182" s="15" t="n">
         <v>312</v>
       </c>
     </row>
@@ -20430,7 +20798,7 @@
           <t>Component 120</t>
         </is>
       </c>
-      <c r="D183" s="12" t="n">
+      <c r="D183" s="15" t="n">
         <v>56</v>
       </c>
     </row>
@@ -20450,7 +20818,7 @@
           <t>directionLeft</t>
         </is>
       </c>
-      <c r="D184" s="12" t="n">
+      <c r="D184" s="15" t="n">
         <v>53</v>
       </c>
     </row>
@@ -20470,7 +20838,7 @@
           <t>whatsapp</t>
         </is>
       </c>
-      <c r="D185" s="12" t="n">
+      <c r="D185" s="15" t="n">
         <v>28</v>
       </c>
     </row>
@@ -20490,7 +20858,7 @@
           <t>DirectionDown</t>
         </is>
       </c>
-      <c r="D186" s="12" t="n">
+      <c r="D186" s="15" t="n">
         <v>27</v>
       </c>
     </row>
@@ -20510,7 +20878,7 @@
           <t>Indicator Mobile</t>
         </is>
       </c>
-      <c r="D187" s="12" t="n">
+      <c r="D187" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20530,7 +20898,7 @@
           <t>Step 01</t>
         </is>
       </c>
-      <c r="D188" s="12" t="n">
+      <c r="D188" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20550,7 +20918,7 @@
           <t>Step 02</t>
         </is>
       </c>
-      <c r="D189" s="12" t="n">
+      <c r="D189" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20570,7 +20938,7 @@
           <t>torito</t>
         </is>
       </c>
-      <c r="D190" s="12" t="n">
+      <c r="D190" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20590,7 +20958,7 @@
           <t>A.white</t>
         </is>
       </c>
-      <c r="D191" s="12" t="n">
+      <c r="D191" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -20610,7 +20978,7 @@
           <t>mail</t>
         </is>
       </c>
-      <c r="D192" s="12" t="n">
+      <c r="D192" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -20630,7 +20998,7 @@
           <t>iaSpark</t>
         </is>
       </c>
-      <c r="D193" s="12" t="n">
+      <c r="D193" s="15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -20650,7 +21018,7 @@
           <t>DirectionRight</t>
         </is>
       </c>
-      <c r="D194" s="12" t="n">
+      <c r="D194" s="15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -20670,7 +21038,7 @@
           <t>Viajeros</t>
         </is>
       </c>
-      <c r="D195" s="12" t="n">
+      <c r="D195" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -20690,7 +21058,7 @@
           <t>advertencia</t>
         </is>
       </c>
-      <c r="D196" s="12" t="n">
+      <c r="D196" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -20710,7 +21078,7 @@
           <t>hiking</t>
         </is>
       </c>
-      <c r="D197" s="12" t="n">
+      <c r="D197" s="15" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20730,7 +21098,7 @@
           <t>Viajeros Mobile</t>
         </is>
       </c>
-      <c r="D198" s="12" t="n">
+      <c r="D198" s="15" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20750,7 +21118,7 @@
           <t>Cancel Icon</t>
         </is>
       </c>
-      <c r="D199" s="12" t="n">
+      <c r="D199" s="15" t="n">
         <v>6</v>
       </c>
     </row>
@@ -20770,7 +21138,7 @@
           <t>Pasajeros</t>
         </is>
       </c>
-      <c r="D200" s="12" t="n">
+      <c r="D200" s="15" t="n">
         <v>4</v>
       </c>
     </row>
@@ -20790,7 +21158,7 @@
           <t>Spinner mesagge</t>
         </is>
       </c>
-      <c r="D201" s="12" t="n">
+      <c r="D201" s="15" t="n">
         <v>4</v>
       </c>
     </row>
@@ -20810,7 +21178,7 @@
           <t>Option</t>
         </is>
       </c>
-      <c r="D202" s="12" t="n">
+      <c r="D202" s="15" t="n">
         <v>174</v>
       </c>
     </row>
@@ -20830,7 +21198,7 @@
           <t>01 Info</t>
         </is>
       </c>
-      <c r="D203" s="12" t="n">
+      <c r="D203" s="15" t="n">
         <v>70</v>
       </c>
     </row>
@@ -20850,7 +21218,7 @@
           <t>ArrowLeft</t>
         </is>
       </c>
-      <c r="D204" s="12" t="n">
+      <c r="D204" s="15" t="n">
         <v>58</v>
       </c>
     </row>
@@ -20870,7 +21238,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="D205" s="12" t="n">
+      <c r="D205" s="15" t="n">
         <v>54</v>
       </c>
     </row>
@@ -20890,7 +21258,7 @@
           <t>whatsapp</t>
         </is>
       </c>
-      <c r="D206" s="12" t="n">
+      <c r="D206" s="15" t="n">
         <v>50</v>
       </c>
     </row>
@@ -20910,7 +21278,7 @@
           <t>Complex</t>
         </is>
       </c>
-      <c r="D207" s="12" t="n">
+      <c r="D207" s="15" t="n">
         <v>47</v>
       </c>
     </row>
@@ -20930,7 +21298,7 @@
           <t>Trend</t>
         </is>
       </c>
-      <c r="D208" s="12" t="n">
+      <c r="D208" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -20950,7 +21318,7 @@
           <t>A.white</t>
         </is>
       </c>
-      <c r="D209" s="12" t="n">
+      <c r="D209" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -20970,7 +21338,7 @@
           <t>Cancel Icon</t>
         </is>
       </c>
-      <c r="D210" s="12" t="n">
+      <c r="D210" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20990,7 +21358,7 @@
           <t>Toast</t>
         </is>
       </c>
-      <c r="D211" s="12" t="n">
+      <c r="D211" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21010,7 +21378,7 @@
           <t>eye_open</t>
         </is>
       </c>
-      <c r="D212" s="12" t="n">
+      <c r="D212" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21030,7 +21398,7 @@
           <t>torito</t>
         </is>
       </c>
-      <c r="D213" s="12" t="n">
+      <c r="D213" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21050,7 +21418,7 @@
           <t>Tooltip</t>
         </is>
       </c>
-      <c r="D214" s="12" t="n">
+      <c r="D214" s="15" t="n">
         <v>13</v>
       </c>
     </row>
@@ -21070,7 +21438,7 @@
           <t>send</t>
         </is>
       </c>
-      <c r="D215" s="12" t="n">
+      <c r="D215" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21090,7 +21458,7 @@
           <t>mail</t>
         </is>
       </c>
-      <c r="D216" s="12" t="n">
+      <c r="D216" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21110,7 +21478,7 @@
           <t>resumen</t>
         </is>
       </c>
-      <c r="D217" s="12" t="n">
+      <c r="D217" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21130,7 +21498,7 @@
           <t>Botón primario</t>
         </is>
       </c>
-      <c r="D218" s="12" t="n">
+      <c r="D218" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -21150,7 +21518,7 @@
           <t>Scroll</t>
         </is>
       </c>
-      <c r="D219" s="12" t="n">
+      <c r="D219" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -21170,7 +21538,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D220" s="12" t="n">
+      <c r="D220" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -21190,7 +21558,7 @@
           <t>Lock</t>
         </is>
       </c>
-      <c r="D221" s="12" t="n">
+      <c r="D221" s="15" t="n">
         <v>7</v>
       </c>
     </row>
@@ -21210,7 +21578,7 @@
           <t>Line Tracking Vertical</t>
         </is>
       </c>
-      <c r="D222" s="12" t="n">
+      <c r="D222" s="15" t="n">
         <v>155</v>
       </c>
     </row>
@@ -21230,7 +21598,7 @@
           <t>Step 3</t>
         </is>
       </c>
-      <c r="D223" s="12" t="n">
+      <c r="D223" s="15" t="n">
         <v>31</v>
       </c>
     </row>
@@ -21250,7 +21618,7 @@
           <t>Step 1</t>
         </is>
       </c>
-      <c r="D224" s="12" t="n">
+      <c r="D224" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -21270,7 +21638,7 @@
           <t>Step 2</t>
         </is>
       </c>
-      <c r="D225" s="12" t="n">
+      <c r="D225" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -21290,7 +21658,7 @@
           <t>Step 4</t>
         </is>
       </c>
-      <c r="D226" s="12" t="n">
+      <c r="D226" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -21310,7 +21678,7 @@
           <t>Step 5</t>
         </is>
       </c>
-      <c r="D227" s="12" t="n">
+      <c r="D227" s="15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -21330,7 +21698,7 @@
           <t>title_+_badges_download</t>
         </is>
       </c>
-      <c r="D228" s="12" t="n">
+      <c r="D228" s="15" t="n">
         <v>29</v>
       </c>
     </row>
@@ -21350,7 +21718,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D229" s="12" t="n">
+      <c r="D229" s="15" t="n">
         <v>29</v>
       </c>
     </row>
@@ -21370,7 +21738,7 @@
           <t>Indicator Mobile</t>
         </is>
       </c>
-      <c r="D230" s="12" t="n">
+      <c r="D230" s="15" t="n">
         <v>27</v>
       </c>
     </row>
@@ -21390,7 +21758,7 @@
           <t>Cancel Icon</t>
         </is>
       </c>
-      <c r="D231" s="12" t="n">
+      <c r="D231" s="15" t="n">
         <v>26</v>
       </c>
     </row>
@@ -21410,7 +21778,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="D232" s="12" t="n">
+      <c r="D232" s="15" t="n">
         <v>23</v>
       </c>
     </row>
@@ -21430,7 +21798,7 @@
           <t>Cargador circular</t>
         </is>
       </c>
-      <c r="D233" s="12" t="n">
+      <c r="D233" s="15" t="n">
         <v>16</v>
       </c>
     </row>
@@ -21450,7 +21818,7 @@
           <t>advertencia</t>
         </is>
       </c>
-      <c r="D234" s="12" t="n">
+      <c r="D234" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -21470,7 +21838,7 @@
           <t>add</t>
         </is>
       </c>
-      <c r="D235" s="12" t="n">
+      <c r="D235" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21490,7 +21858,7 @@
           <t>Close Icon</t>
         </is>
       </c>
-      <c r="D236" s="12" t="n">
+      <c r="D236" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21510,7 +21878,7 @@
           <t>cloudupload</t>
         </is>
       </c>
-      <c r="D237" s="12" t="n">
+      <c r="D237" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21530,7 +21898,7 @@
           <t>card-selector</t>
         </is>
       </c>
-      <c r="D238" s="12" t="n">
+      <c r="D238" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21550,7 +21918,7 @@
           <t>[SCTR] Planes cotizador</t>
         </is>
       </c>
-      <c r="D239" s="12" t="n">
+      <c r="D239" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21570,7 +21938,7 @@
           <t>description</t>
         </is>
       </c>
-      <c r="D240" s="12" t="n">
+      <c r="D240" s="15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -21590,7 +21958,7 @@
           <t>Bullet Icon</t>
         </is>
       </c>
-      <c r="D241" s="12" t="n">
+      <c r="D241" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -21610,7 +21978,7 @@
           <t>Icon</t>
         </is>
       </c>
-      <c r="D242" s="12" t="n">
+      <c r="D242" s="15" t="n">
         <v>221</v>
       </c>
     </row>
@@ -21630,7 +21998,7 @@
           <t>CardProductPromo</t>
         </is>
       </c>
-      <c r="D243" s="12" t="n">
+      <c r="D243" s="15" t="n">
         <v>206</v>
       </c>
     </row>
@@ -21650,7 +22018,7 @@
           <t>Cotizar</t>
         </is>
       </c>
-      <c r="D244" s="12" t="n">
+      <c r="D244" s="15" t="n">
         <v>110</v>
       </c>
     </row>
@@ -21670,7 +22038,7 @@
           <t>Video</t>
         </is>
       </c>
-      <c r="D245" s="12" t="n">
+      <c r="D245" s="15" t="n">
         <v>110</v>
       </c>
     </row>
@@ -21690,7 +22058,7 @@
           <t>Close Icon</t>
         </is>
       </c>
-      <c r="D246" s="12" t="n">
+      <c r="D246" s="15" t="n">
         <v>101</v>
       </c>
     </row>
@@ -21710,7 +22078,7 @@
           <t>Scroll</t>
         </is>
       </c>
-      <c r="D247" s="12" t="n">
+      <c r="D247" s="15" t="n">
         <v>83</v>
       </c>
     </row>
@@ -21730,7 +22098,7 @@
           <t>CardMenúMobile</t>
         </is>
       </c>
-      <c r="D248" s="12" t="n">
+      <c r="D248" s="15" t="n">
         <v>79</v>
       </c>
     </row>
@@ -21750,7 +22118,7 @@
           <t>CardMenú</t>
         </is>
       </c>
-      <c r="D249" s="12" t="n">
+      <c r="D249" s="15" t="n">
         <v>77</v>
       </c>
     </row>
@@ -21770,7 +22138,7 @@
           <t>WithoutShieldHeart</t>
         </is>
       </c>
-      <c r="D250" s="12" t="n">
+      <c r="D250" s="15" t="n">
         <v>74</v>
       </c>
     </row>
@@ -21790,7 +22158,7 @@
           <t>ShieldHeart</t>
         </is>
       </c>
-      <c r="D251" s="12" t="n">
+      <c r="D251" s="15" t="n">
         <v>71</v>
       </c>
     </row>
@@ -21810,7 +22178,7 @@
           <t>BotónCategoría</t>
         </is>
       </c>
-      <c r="D252" s="12" t="n">
+      <c r="D252" s="15" t="n">
         <v>69</v>
       </c>
     </row>
@@ -21830,7 +22198,7 @@
           <t>Slider</t>
         </is>
       </c>
-      <c r="D253" s="12" t="n">
+      <c r="D253" s="15" t="n">
         <v>64</v>
       </c>
     </row>
@@ -21850,7 +22218,7 @@
           <t>_Link Icon</t>
         </is>
       </c>
-      <c r="D254" s="12" t="n">
+      <c r="D254" s="15" t="n">
         <v>54</v>
       </c>
     </row>
@@ -21870,7 +22238,7 @@
           <t>_Button Icon</t>
         </is>
       </c>
-      <c r="D255" s="12" t="n">
+      <c r="D255" s="15" t="n">
         <v>54</v>
       </c>
     </row>
@@ -21890,7 +22258,7 @@
           <t>submenu</t>
         </is>
       </c>
-      <c r="D256" s="12" t="n">
+      <c r="D256" s="15" t="n">
         <v>48</v>
       </c>
     </row>
@@ -21910,7 +22278,7 @@
           <t>Car</t>
         </is>
       </c>
-      <c r="D257" s="12" t="n">
+      <c r="D257" s="15" t="n">
         <v>48</v>
       </c>
     </row>
@@ -21930,7 +22298,7 @@
           <t>Trend</t>
         </is>
       </c>
-      <c r="D258" s="12" t="n">
+      <c r="D258" s="15" t="n">
         <v>46</v>
       </c>
     </row>
@@ -21950,7 +22318,7 @@
           <t>MedicalService</t>
         </is>
       </c>
-      <c r="D259" s="12" t="n">
+      <c r="D259" s="15" t="n">
         <v>46</v>
       </c>
     </row>
@@ -21970,7 +22338,7 @@
           <t>Link Stamp</t>
         </is>
       </c>
-      <c r="D260" s="12" t="n">
+      <c r="D260" s="15" t="n">
         <v>36</v>
       </c>
     </row>
@@ -21990,7 +22358,7 @@
           <t>title_+_badges_download</t>
         </is>
       </c>
-      <c r="D261" s="12" t="n">
+      <c r="D261" s="15" t="n">
         <v>35</v>
       </c>
     </row>
@@ -22010,7 +22378,7 @@
           <t>icon</t>
         </is>
       </c>
-      <c r="D262" s="12" t="n">
+      <c r="D262" s="15" t="n">
         <v>24</v>
       </c>
     </row>
@@ -22030,7 +22398,7 @@
           <t>SecciónDescripción</t>
         </is>
       </c>
-      <c r="D263" s="12" t="n">
+      <c r="D263" s="15" t="n">
         <v>21</v>
       </c>
     </row>
@@ -22050,7 +22418,7 @@
           <t>Icon</t>
         </is>
       </c>
-      <c r="D264" s="12" t="n">
+      <c r="D264" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -22070,7 +22438,7 @@
           <t>Image</t>
         </is>
       </c>
-      <c r="D265" s="12" t="n">
+      <c r="D265" s="15" t="n">
         <v>18</v>
       </c>
     </row>
@@ -22090,7 +22458,7 @@
           <t>WithoutShieldHeart</t>
         </is>
       </c>
-      <c r="D266" s="12" t="n">
+      <c r="D266" s="15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -22110,7 +22478,7 @@
           <t>SeccionCanales</t>
         </is>
       </c>
-      <c r="D267" s="12" t="n">
+      <c r="D267" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -22130,7 +22498,7 @@
           <t>PersonalInjuy</t>
         </is>
       </c>
-      <c r="D268" s="12" t="n">
+      <c r="D268" s="15" t="n">
         <v>12</v>
       </c>
     </row>
@@ -22150,7 +22518,7 @@
           <t>Information</t>
         </is>
       </c>
-      <c r="D269" s="12" t="n">
+      <c r="D269" s="15" t="n">
         <v>11</v>
       </c>
     </row>
@@ -22170,7 +22538,7 @@
           <t>LogosCollab</t>
         </is>
       </c>
-      <c r="D270" s="12" t="n">
+      <c r="D270" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -22190,7 +22558,7 @@
           <t>CoberturasIconos</t>
         </is>
       </c>
-      <c r="D271" s="12" t="n">
+      <c r="D271" s="15" t="n">
         <v>10</v>
       </c>
     </row>
@@ -22210,7 +22578,7 @@
           <t>Scroll</t>
         </is>
       </c>
-      <c r="D272" s="12" t="n">
+      <c r="D272" s="15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -22230,7 +22598,7 @@
           <t>Complex</t>
         </is>
       </c>
-      <c r="D273" s="12" t="n">
+      <c r="D273" s="15" t="n">
         <v>6</v>
       </c>
     </row>
@@ -22250,7 +22618,7 @@
           <t>title_+_badges_download</t>
         </is>
       </c>
-      <c r="D274" s="12" t="n">
+      <c r="D274" s="15" t="n">
         <v>6</v>
       </c>
     </row>
@@ -22270,7 +22638,7 @@
           <t>problema eléctrico</t>
         </is>
       </c>
-      <c r="D275" s="12" t="n">
+      <c r="D275" s="15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -22290,7 +22658,7 @@
           <t>robo de autopartes</t>
         </is>
       </c>
-      <c r="D276" s="12" t="n">
+      <c r="D276" s="15" t="n">
         <v>4</v>
       </c>
     </row>
@@ -22310,7 +22678,7 @@
           <t>avión</t>
         </is>
       </c>
-      <c r="D277" s="12" t="n">
+      <c r="D277" s="15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22330,7 +22698,7 @@
           <t>generales</t>
         </is>
       </c>
-      <c r="D278" s="12" t="n">
+      <c r="D278" s="15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22350,7 +22718,7 @@
           <t>download</t>
         </is>
       </c>
-      <c r="D279" s="12" t="n">
+      <c r="D279" s="15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22370,7 +22738,7 @@
           <t>fractura</t>
         </is>
       </c>
-      <c r="D280" s="12" t="n">
+      <c r="D280" s="15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22390,7 +22758,7 @@
           <t>doctor</t>
         </is>
       </c>
-      <c r="D281" s="12" t="n">
+      <c r="D281" s="15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22399,13 +22767,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -22413,9 +22781,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22446,15 +22815,20 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
+          <t>Detach %</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
           <t>Frames RFD</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Inst. DS</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -22478,7 +22852,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -22486,13 +22860,18 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="H2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="I2" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22522,13 +22901,18 @@
           <t>64%</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="H3" s="7" t="n">
         <v>9789</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="I3" s="6" t="n">
         <v>15276</v>
       </c>
     </row>
@@ -22550,7 +22934,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -22558,13 +22942,18 @@
           <t>88%</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="H4" s="7" t="n">
         <v>1424</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="I4" s="6" t="n">
         <v>1625</v>
       </c>
     </row>
@@ -22586,7 +22975,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -22594,13 +22983,18 @@
           <t>51%</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="H5" s="7" t="n">
         <v>3018</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>5891</v>
       </c>
     </row>
@@ -22622,7 +23016,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -22630,14 +23024,19 @@
           <t>65%</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G6" s="7" t="n">
-        <v>14386</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>22040</v>
+      <c r="H6" s="7" t="n">
+        <v>14419</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>22099</v>
       </c>
     </row>
     <row r="7">
@@ -22658,7 +23057,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -22666,13 +23065,18 @@
           <t>94%</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="H7" s="7" t="n">
         <v>172970</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>184326</v>
       </c>
     </row>
@@ -22694,7 +23098,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -22702,13 +23106,18 @@
           <t>84%</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="H8" s="7" t="n">
         <v>8539</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="I8" s="6" t="n">
         <v>10226</v>
       </c>
     </row>
@@ -22730,7 +23139,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -22738,13 +23147,18 @@
           <t>90%</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="H9" s="7" t="n">
         <v>7739</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>8560</v>
       </c>
     </row>
@@ -22766,7 +23180,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -22774,13 +23188,18 @@
           <t>75%</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="H10" s="7" t="n">
         <v>1583</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="I10" s="6" t="n">
         <v>2109</v>
       </c>
     </row>
@@ -22802,7 +23221,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -22810,13 +23229,18 @@
           <t>87%</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="H11" s="7" t="n">
         <v>3852</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>4452</v>
       </c>
     </row>
@@ -22838,7 +23262,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -22846,13 +23270,18 @@
           <t>85%</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="H12" s="7" t="n">
         <v>3906</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="I12" s="6" t="n">
         <v>4593</v>
       </c>
     </row>
@@ -22874,7 +23303,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -22882,13 +23311,18 @@
           <t>73%</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="H13" s="7" t="n">
         <v>2286</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="I13" s="6" t="n">
         <v>3132</v>
       </c>
     </row>
@@ -22910,7 +23344,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -22918,13 +23352,18 @@
           <t>69%</t>
         </is>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="H14" s="7" t="n">
         <v>2650</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="I14" s="6" t="n">
         <v>3813</v>
       </c>
     </row>
@@ -22946,7 +23385,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -22954,14 +23393,19 @@
           <t>94%</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="7" t="n">
-        <v>11371</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>12077</v>
+      <c r="H15" s="7" t="n">
+        <v>11370</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>12076</v>
       </c>
     </row>
     <row r="16">
@@ -22982,7 +23426,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -22990,13 +23434,18 @@
           <t>85%</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="H16" s="7" t="n">
         <v>3566</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="I16" s="6" t="n">
         <v>4204</v>
       </c>
     </row>
@@ -23018,7 +23467,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -23026,13 +23475,18 @@
           <t>84%</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
         <v>73</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="H17" s="7" t="n">
         <v>11472</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="I17" s="6" t="n">
         <v>13594</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: adoption report 2026-06-30 22:33 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -1207,20 +1207,20 @@
         <v>1</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0</v>
+        <v>1424</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>19</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>88%</t>
         </is>
       </c>
       <c r="I19" s="10" t="n">
@@ -2135,20 +2135,20 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>0</v>
+        <v>1424</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="12" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>19</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>88%</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E571"/>
+  <dimension ref="A1:E590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17035,6 +17035,481 @@
         <v>2</v>
       </c>
     </row>
+    <row r="572">
+      <c r="A572" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B572" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C572" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D572" s="5" t="inlineStr">
+        <is>
+          <t>type_option</t>
+        </is>
+      </c>
+      <c r="E572" s="7" t="n">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B573" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C573" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D573" s="5" t="inlineStr">
+        <is>
+          <t>Átomo</t>
+        </is>
+      </c>
+      <c r="E573" s="7" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B574" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C574" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D574" s="5" t="inlineStr">
+        <is>
+          <t>Accordion</t>
+        </is>
+      </c>
+      <c r="E574" s="7" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B575" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C575" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D575" s="5" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E575" s="7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B576" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C576" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D576" s="5" t="inlineStr">
+        <is>
+          <t>section_footer</t>
+        </is>
+      </c>
+      <c r="E576" s="7" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B577" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C577" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D577" s="5" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E577" s="7" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B578" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C578" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D578" s="5" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="E578" s="7" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B579" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C579" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D579" s="5" t="inlineStr">
+        <is>
+          <t>src_option_redes</t>
+        </is>
+      </c>
+      <c r="E579" s="7" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B580" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C580" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D580" s="5" t="inlineStr">
+        <is>
+          <t>reemplazar slot</t>
+        </is>
+      </c>
+      <c r="E580" s="7" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B581" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C581" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D581" s="5" t="inlineStr">
+        <is>
+          <t>title_+_options</t>
+        </is>
+      </c>
+      <c r="E581" s="7" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B582" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C582" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D582" s="5" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+      <c r="E582" s="7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B583" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C583" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D583" s="5" t="inlineStr">
+        <is>
+          <t>src_option_stores_download</t>
+        </is>
+      </c>
+      <c r="E583" s="7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B584" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C584" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D584" s="5" t="inlineStr">
+        <is>
+          <t>Hero</t>
+        </is>
+      </c>
+      <c r="E584" s="7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B585" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C585" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D585" s="5" t="inlineStr">
+        <is>
+          <t>Breadcrumb</t>
+        </is>
+      </c>
+      <c r="E585" s="7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B586" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C586" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D586" s="5" t="inlineStr">
+        <is>
+          <t>title_+_phones</t>
+        </is>
+      </c>
+      <c r="E586" s="7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B587" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C587" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D587" s="5" t="inlineStr">
+        <is>
+          <t>title_+_social media</t>
+        </is>
+      </c>
+      <c r="E587" s="7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B588" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C588" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D588" s="5" t="inlineStr">
+        <is>
+          <t>Logo Horizontal</t>
+        </is>
+      </c>
+      <c r="E588" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B589" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C589" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D589" s="5" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="E589" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B590" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C590" s="4" t="inlineStr">
+        <is>
+          <t>Landing Alianzas</t>
+        </is>
+      </c>
+      <c r="D590" s="5" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E590" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17046,7 +17521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D261"/>
+  <dimension ref="A1:D281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22275,6 +22750,406 @@
       </c>
       <c r="D261" s="16" t="n">
         <v>35</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B262" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C262" s="4" t="inlineStr">
+        <is>
+          <t>icon</t>
+        </is>
+      </c>
+      <c r="D262" s="16" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B263" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C263" s="4" t="inlineStr">
+        <is>
+          <t>SecciónDescripción</t>
+        </is>
+      </c>
+      <c r="D263" s="16" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D264" s="16" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D265" s="16" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>WithoutShieldHeart</t>
+        </is>
+      </c>
+      <c r="D266" s="16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C267" s="4" t="inlineStr">
+        <is>
+          <t>SeccionCanales</t>
+        </is>
+      </c>
+      <c r="D267" s="16" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B268" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>PersonalInjuy</t>
+        </is>
+      </c>
+      <c r="D268" s="16" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C269" s="4" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="D269" s="16" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B270" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C270" s="4" t="inlineStr">
+        <is>
+          <t>LogosCollab</t>
+        </is>
+      </c>
+      <c r="D270" s="16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C271" s="4" t="inlineStr">
+        <is>
+          <t>CoberturasIconos</t>
+        </is>
+      </c>
+      <c r="D271" s="16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B272" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>Scroll</t>
+        </is>
+      </c>
+      <c r="D272" s="16" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C273" s="4" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="D273" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C274" s="4" t="inlineStr">
+        <is>
+          <t>title_+_badges_download</t>
+        </is>
+      </c>
+      <c r="D274" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C275" s="4" t="inlineStr">
+        <is>
+          <t>problema eléctrico</t>
+        </is>
+      </c>
+      <c r="D275" s="16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B276" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C276" s="4" t="inlineStr">
+        <is>
+          <t>robo de autopartes</t>
+        </is>
+      </c>
+      <c r="D276" s="16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="inlineStr">
+        <is>
+          <t>avión</t>
+        </is>
+      </c>
+      <c r="D277" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B278" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
+        <is>
+          <t>generales</t>
+        </is>
+      </c>
+      <c r="D278" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C279" s="4" t="inlineStr">
+        <is>
+          <t>download</t>
+        </is>
+      </c>
+      <c r="D279" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>fractura</t>
+        </is>
+      </c>
+      <c r="D280" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t>Embebidos</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr">
+        <is>
+          <t>doctor</t>
+        </is>
+      </c>
+      <c r="D281" s="16" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -22452,24 +23327,24 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
       <c r="G4" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>0</v>
+        <v>1424</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-01 16:43 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -1105,20 +1105,20 @@
         <v>3</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>10590</v>
+        <v>5448</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>2027</v>
+        <v>787</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
@@ -1997,20 +1997,20 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>4605</v>
+        <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>1163</v>
+        <v>0</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>80%</t>
+        <v>0</v>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -2031,20 +2031,20 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>537</v>
+        <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="H25" s="11" t="inlineStr">
-        <is>
-          <t>87%</t>
+        <v>0</v>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E568"/>
+  <dimension ref="A1:E533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15886,881 +15886,6 @@
       </c>
       <c r="E533" s="7" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="534">
-      <c r="A534" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B534" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C534" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D534" s="5" t="inlineStr">
-        <is>
-          <t>type_option</t>
-        </is>
-      </c>
-      <c r="E534" s="7" t="n">
-        <v>1995</v>
-      </c>
-    </row>
-    <row r="535">
-      <c r="A535" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B535" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C535" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D535" s="5" t="inlineStr">
-        <is>
-          <t>Tag</t>
-        </is>
-      </c>
-      <c r="E535" s="7" t="n">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="536">
-      <c r="A536" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B536" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C536" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D536" s="5" t="inlineStr">
-        <is>
-          <t>Button</t>
-        </is>
-      </c>
-      <c r="E536" s="7" t="n">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="537">
-      <c r="A537" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B537" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C537" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D537" s="5" t="inlineStr">
-        <is>
-          <t>section_footer</t>
-        </is>
-      </c>
-      <c r="E537" s="7" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="538">
-      <c r="A538" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B538" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C538" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D538" s="5" t="inlineStr">
-        <is>
-          <t>Tab</t>
-        </is>
-      </c>
-      <c r="E538" s="7" t="n">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="539">
-      <c r="A539" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B539" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C539" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D539" s="5" t="inlineStr">
-        <is>
-          <t>Átomo</t>
-        </is>
-      </c>
-      <c r="E539" s="7" t="n">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="540">
-      <c r="A540" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B540" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C540" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D540" s="5" t="inlineStr">
-        <is>
-          <t>src_option_redes</t>
-        </is>
-      </c>
-      <c r="E540" s="7" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="541">
-      <c r="A541" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B541" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C541" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D541" s="5" t="inlineStr">
-        <is>
-          <t>reemplazar slot</t>
-        </is>
-      </c>
-      <c r="E541" s="7" t="n">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="542">
-      <c r="A542" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B542" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C542" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D542" s="5" t="inlineStr">
-        <is>
-          <t>Header</t>
-        </is>
-      </c>
-      <c r="E542" s="7" t="n">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="543">
-      <c r="A543" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B543" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C543" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D543" s="5" t="inlineStr">
-        <is>
-          <t>Alert</t>
-        </is>
-      </c>
-      <c r="E543" s="7" t="n">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="544">
-      <c r="A544" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B544" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C544" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D544" s="5" t="inlineStr">
-        <is>
-          <t>Slider Controls</t>
-        </is>
-      </c>
-      <c r="E544" s="7" t="n">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="545">
-      <c r="A545" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B545" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C545" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D545" s="5" t="inlineStr">
-        <is>
-          <t>Status Control</t>
-        </is>
-      </c>
-      <c r="E545" s="7" t="n">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="546">
-      <c r="A546" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B546" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C546" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D546" s="5" t="inlineStr">
-        <is>
-          <t>title_+_options</t>
-        </is>
-      </c>
-      <c r="E546" s="7" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="547">
-      <c r="A547" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B547" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C547" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D547" s="5" t="inlineStr">
-        <is>
-          <t>src_option_stores_download</t>
-        </is>
-      </c>
-      <c r="E547" s="7" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="548">
-      <c r="A548" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B548" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C548" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D548" s="5" t="inlineStr">
-        <is>
-          <t>title_+_phones</t>
-        </is>
-      </c>
-      <c r="E548" s="7" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="549">
-      <c r="A549" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B549" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C549" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D549" s="5" t="inlineStr">
-        <is>
-          <t>title_+_social media</t>
-        </is>
-      </c>
-      <c r="E549" s="7" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="550">
-      <c r="A550" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B550" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C550" s="4" t="inlineStr">
-        <is>
-          <t>Menú / Home</t>
-        </is>
-      </c>
-      <c r="D550" s="5" t="inlineStr">
-        <is>
-          <t>Hero</t>
-        </is>
-      </c>
-      <c r="E550" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="551">
-      <c r="A551" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B551" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C551" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D551" s="5" t="inlineStr">
-        <is>
-          <t>type_option</t>
-        </is>
-      </c>
-      <c r="E551" s="7" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="552">
-      <c r="A552" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B552" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C552" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D552" s="5" t="inlineStr">
-        <is>
-          <t>Átomo</t>
-        </is>
-      </c>
-      <c r="E552" s="7" t="n">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="553">
-      <c r="A553" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B553" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C553" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D553" s="5" t="inlineStr">
-        <is>
-          <t>Accordion</t>
-        </is>
-      </c>
-      <c r="E553" s="7" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="554">
-      <c r="A554" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B554" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C554" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D554" s="5" t="inlineStr">
-        <is>
-          <t>Tab</t>
-        </is>
-      </c>
-      <c r="E554" s="7" t="n">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="555">
-      <c r="A555" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B555" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C555" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D555" s="5" t="inlineStr">
-        <is>
-          <t>Tag</t>
-        </is>
-      </c>
-      <c r="E555" s="7" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="556">
-      <c r="A556" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B556" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C556" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D556" s="5" t="inlineStr">
-        <is>
-          <t>Button</t>
-        </is>
-      </c>
-      <c r="E556" s="7" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="557">
-      <c r="A557" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B557" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C557" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D557" s="5" t="inlineStr">
-        <is>
-          <t>Alert</t>
-        </is>
-      </c>
-      <c r="E557" s="7" t="n">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="558">
-      <c r="A558" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B558" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C558" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D558" s="5" t="inlineStr">
-        <is>
-          <t>section_footer</t>
-        </is>
-      </c>
-      <c r="E558" s="7" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="559">
-      <c r="A559" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B559" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C559" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D559" s="5" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="E559" s="7" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="560">
-      <c r="A560" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B560" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C560" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D560" s="5" t="inlineStr">
-        <is>
-          <t>Calendar</t>
-        </is>
-      </c>
-      <c r="E560" s="7" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="561">
-      <c r="A561" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B561" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C561" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D561" s="5" t="inlineStr">
-        <is>
-          <t>reemplazar slot</t>
-        </is>
-      </c>
-      <c r="E561" s="7" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="562">
-      <c r="A562" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B562" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C562" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D562" s="5" t="inlineStr">
-        <is>
-          <t>Discount Badge</t>
-        </is>
-      </c>
-      <c r="E562" s="7" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="563">
-      <c r="A563" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B563" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C563" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D563" s="5" t="inlineStr">
-        <is>
-          <t>title_+_options</t>
-        </is>
-      </c>
-      <c r="E563" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="564">
-      <c r="A564" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B564" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C564" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D564" s="5" t="inlineStr">
-        <is>
-          <t>Breadcrumb</t>
-        </is>
-      </c>
-      <c r="E564" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="565">
-      <c r="A565" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B565" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C565" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D565" s="5" t="inlineStr">
-        <is>
-          <t>Slider Controls</t>
-        </is>
-      </c>
-      <c r="E565" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="566">
-      <c r="A566" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B566" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C566" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D566" s="5" t="inlineStr">
-        <is>
-          <t>title_+_phones</t>
-        </is>
-      </c>
-      <c r="E566" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="567">
-      <c r="A567" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B567" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C567" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D567" s="5" t="inlineStr">
-        <is>
-          <t>title_+_social media</t>
-        </is>
-      </c>
-      <c r="E567" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="568">
-      <c r="A568" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="B568" s="4" t="inlineStr">
-        <is>
-          <t>Web Corporativa</t>
-        </is>
-      </c>
-      <c r="C568" s="4" t="inlineStr">
-        <is>
-          <t>Productos Líneas Personales</t>
-        </is>
-      </c>
-      <c r="D568" s="5" t="inlineStr">
-        <is>
-          <t>Status Control</t>
-        </is>
-      </c>
-      <c r="E568" s="7" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -21618,11 +20743,11 @@
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Cotizar</t>
         </is>
       </c>
       <c r="D242" s="18" t="n">
-        <v>217</v>
+        <v>91</v>
       </c>
     </row>
     <row r="243">
@@ -21638,11 +20763,11 @@
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>CardProductPromo</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="D243" s="18" t="n">
-        <v>206</v>
+        <v>91</v>
       </c>
     </row>
     <row r="244">
@@ -21658,11 +20783,11 @@
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>Cotizar</t>
+          <t>Close Icon</t>
         </is>
       </c>
       <c r="D244" s="18" t="n">
-        <v>102</v>
+        <v>73</v>
       </c>
     </row>
     <row r="245">
@@ -21678,11 +20803,11 @@
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Scroll</t>
         </is>
       </c>
       <c r="D245" s="18" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
     </row>
     <row r="246">
@@ -21698,11 +20823,11 @@
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>Close Icon</t>
+          <t>_Link Icon</t>
         </is>
       </c>
       <c r="D246" s="18" t="n">
-        <v>84</v>
+        <v>54</v>
       </c>
     </row>
     <row r="247">
@@ -21718,11 +20843,11 @@
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>CardMenúMobile</t>
+          <t>ShieldHeart</t>
         </is>
       </c>
       <c r="D247" s="18" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
     </row>
     <row r="248">
@@ -21738,11 +20863,11 @@
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>CardMenú</t>
+          <t>WithoutShieldHeart</t>
         </is>
       </c>
       <c r="D248" s="18" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
     </row>
     <row r="249">
@@ -21758,11 +20883,11 @@
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>Scroll</t>
+          <t>_Button Icon</t>
         </is>
       </c>
       <c r="D249" s="18" t="n">
-        <v>71</v>
+        <v>50</v>
       </c>
     </row>
     <row r="250">
@@ -21778,11 +20903,11 @@
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>BotónCategoría</t>
+          <t>submenu</t>
         </is>
       </c>
       <c r="D250" s="18" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
     </row>
     <row r="251">
@@ -21798,11 +20923,11 @@
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>Slider</t>
+          <t>Link Stamp</t>
         </is>
       </c>
       <c r="D251" s="18" t="n">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="252">
@@ -21818,11 +20943,11 @@
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>WithoutShieldHeart</t>
+          <t>link</t>
         </is>
       </c>
       <c r="D252" s="18" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
     </row>
     <row r="253">
@@ -21838,11 +20963,11 @@
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
-          <t>ShieldHeart</t>
+          <t>support</t>
         </is>
       </c>
       <c r="D253" s="18" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
     </row>
     <row r="254">
@@ -21858,11 +20983,11 @@
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>_Link Icon</t>
+          <t>download</t>
         </is>
       </c>
       <c r="D254" s="18" t="n">
-        <v>54</v>
+        <v>20</v>
       </c>
     </row>
     <row r="255">
@@ -21878,11 +21003,11 @@
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>_Button Icon</t>
+          <t>Link Details</t>
         </is>
       </c>
       <c r="D255" s="18" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="256">
@@ -21898,11 +21023,11 @@
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>Car</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D256" s="18" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="257">
@@ -21918,11 +21043,11 @@
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>vida inversión</t>
         </is>
       </c>
       <c r="D257" s="18" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
     </row>
     <row r="258">
@@ -21938,11 +21063,11 @@
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>MedicalService</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="D258" s="18" t="n">
-        <v>46</v>
+        <v>11</v>
       </c>
     </row>
     <row r="259">
@@ -21958,11 +21083,11 @@
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>submenu</t>
+          <t>user</t>
         </is>
       </c>
       <c r="D259" s="18" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
     </row>
     <row r="260">
@@ -21978,11 +21103,11 @@
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>Link Stamp</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="D260" s="18" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
     </row>
     <row r="261">
@@ -21998,11 +21123,11 @@
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
-          <t>ProductTabs</t>
+          <t>title_+_badges_download</t>
         </is>
       </c>
       <c r="D261" s="18" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -23272,7 +22397,7 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
@@ -23281,13 +22406,13 @@
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>10590</v>
+        <v>5448</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>12617</v>
+        <v>6235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-07-02 17:20 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-01</t>
+          <t>Quarter: Q3 2026  |  2026-07-02</t>
         </is>
       </c>
     </row>
@@ -761,13 +761,13 @@
         <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>172970</v>
+        <v>214056</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>11356</v>
+        <v>13745</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -835,13 +835,13 @@
         <v>3</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>14419</v>
+        <v>14380</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7680</v>
+        <v>7668</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>36</v>
@@ -1583,13 +1583,13 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>157765</v>
+        <v>198851</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>10490</v>
+        <v>12879</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -1651,13 +1651,13 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>7895</v>
+        <v>7856</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>2414</v>
+        <v>2402</v>
       </c>
       <c r="G13" s="8" t="n">
         <v>34</v>
@@ -2224,11 +2224,11 @@
         <v>485</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2351</v>
+        <v>2366</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.01%</t>
         </is>
       </c>
     </row>
@@ -2242,11 +2242,11 @@
         <v>86</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4229</v>
+        <v>4256</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>1.99%</t>
+          <t>1.98%</t>
         </is>
       </c>
     </row>
@@ -2260,11 +2260,11 @@
         <v>58</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.95%</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
         <v>53</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>71255</v>
+        <v>72256</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         <v>40</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3758</v>
+        <v>3782</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
@@ -2332,11 +2332,11 @@
         <v>34</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>891</v>
+        <v>908</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>3.61%</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>8726</v>
+        <v>8910</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
@@ -2368,11 +2368,11 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>11044</v>
+        <v>11256</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.2%</t>
         </is>
       </c>
     </row>
@@ -2386,11 +2386,11 @@
         <v>23</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1408</v>
+        <v>1417</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.6%</t>
         </is>
       </c>
     </row>
@@ -2404,11 +2404,11 @@
         <v>21</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>1000</v>
+        <v>1008</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>2.06%</t>
+          <t>2.04%</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
         <v>20</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>17659</v>
+        <v>18026</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
@@ -2440,11 +2440,11 @@
         <v>16</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>4138</v>
+        <v>4184</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>0.38%</t>
         </is>
       </c>
     </row>
@@ -2458,11 +2458,11 @@
         <v>13</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1261</v>
+        <v>1414</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>1.02%</t>
+          <t>0.91%</t>
         </is>
       </c>
     </row>
@@ -2476,11 +2476,11 @@
         <v>11</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3791</v>
+        <v>3863</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.28%</t>
         </is>
       </c>
     </row>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="E175" s="7" t="n">
-        <v>87113</v>
+        <v>110447</v>
       </c>
     </row>
     <row r="176">
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="E176" s="7" t="n">
-        <v>15407</v>
+        <v>19407</v>
       </c>
     </row>
     <row r="177">
@@ -6933,7 +6933,7 @@
         </is>
       </c>
       <c r="E177" s="7" t="n">
-        <v>8152</v>
+        <v>10336</v>
       </c>
     </row>
     <row r="178">
@@ -6958,7 +6958,7 @@
         </is>
       </c>
       <c r="E178" s="7" t="n">
-        <v>7872</v>
+        <v>9872</v>
       </c>
     </row>
     <row r="179">
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>7423</v>
+        <v>9268</v>
       </c>
     </row>
     <row r="180">
@@ -7008,7 +7008,7 @@
         </is>
       </c>
       <c r="E180" s="7" t="n">
-        <v>5251</v>
+        <v>6266</v>
       </c>
     </row>
     <row r="181">
@@ -7033,7 +7033,7 @@
         </is>
       </c>
       <c r="E181" s="7" t="n">
-        <v>3935</v>
+        <v>4935</v>
       </c>
     </row>
     <row r="182">
@@ -7058,7 +7058,7 @@
         </is>
       </c>
       <c r="E182" s="7" t="n">
-        <v>3067</v>
+        <v>3651</v>
       </c>
     </row>
     <row r="183">
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="E183" s="7" t="n">
-        <v>2281</v>
+        <v>2914</v>
       </c>
     </row>
     <row r="184">
@@ -7108,7 +7108,7 @@
         </is>
       </c>
       <c r="E184" s="7" t="n">
-        <v>1676</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="185">
@@ -7133,7 +7133,7 @@
         </is>
       </c>
       <c r="E185" s="7" t="n">
-        <v>1554</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="186">
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="E186" s="7" t="n">
-        <v>1536</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="187">
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="E187" s="7" t="n">
-        <v>1278</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="188">
@@ -7204,11 +7204,11 @@
       </c>
       <c r="D188" s="5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Indicator step</t>
         </is>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1241</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="189">
@@ -7229,11 +7229,11 @@
       </c>
       <c r="D189" s="5" t="inlineStr">
         <is>
-          <t>Indicator step</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E189" s="7" t="n">
-        <v>1166</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="190">
@@ -7258,7 +7258,7 @@
         </is>
       </c>
       <c r="E190" s="7" t="n">
-        <v>1095</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="191">
@@ -7279,11 +7279,11 @@
       </c>
       <c r="D191" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Discount Badge</t>
         </is>
       </c>
       <c r="E191" s="7" t="n">
-        <v>984</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="192">
@@ -7304,11 +7304,11 @@
       </c>
       <c r="D192" s="5" t="inlineStr">
         <is>
-          <t>title_+_social media</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E192" s="7" t="n">
-        <v>984</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="193">
@@ -7329,11 +7329,11 @@
       </c>
       <c r="D193" s="5" t="inlineStr">
         <is>
-          <t>Discount Badge</t>
+          <t>title_+_social media</t>
         </is>
       </c>
       <c r="E193" s="7" t="n">
-        <v>948</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="194">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E194" s="7" t="n">
-        <v>780</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="195">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="E195" s="7" t="n">
-        <v>762</v>
+        <v>990</v>
       </c>
     </row>
     <row r="196">
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="E196" s="7" t="n">
-        <v>759</v>
+        <v>921</v>
       </c>
     </row>
     <row r="197">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>397</v>
+        <v>514</v>
       </c>
     </row>
     <row r="198">
@@ -7454,11 +7454,11 @@
       </c>
       <c r="D198" s="5" t="inlineStr">
         <is>
-          <t>Loader</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E198" s="7" t="n">
-        <v>364</v>
+        <v>503</v>
       </c>
     </row>
     <row r="199">
@@ -7479,11 +7479,11 @@
       </c>
       <c r="D199" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Loader</t>
         </is>
       </c>
       <c r="E199" s="7" t="n">
-        <v>329</v>
+        <v>477</v>
       </c>
     </row>
     <row r="200">
@@ -7508,7 +7508,7 @@
         </is>
       </c>
       <c r="E200" s="7" t="n">
-        <v>280</v>
+        <v>316</v>
       </c>
     </row>
     <row r="201">
@@ -7529,11 +7529,11 @@
       </c>
       <c r="D201" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E201" s="7" t="n">
-        <v>222</v>
+        <v>245</v>
       </c>
     </row>
     <row r="202">
@@ -7554,11 +7554,11 @@
       </c>
       <c r="D202" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E202" s="7" t="n">
-        <v>217</v>
+        <v>236</v>
       </c>
     </row>
     <row r="203">
@@ -7579,11 +7579,11 @@
       </c>
       <c r="D203" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E203" s="7" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="204">
@@ -7608,7 +7608,7 @@
         </is>
       </c>
       <c r="E204" s="7" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
     </row>
     <row r="205">
@@ -7633,7 +7633,7 @@
         </is>
       </c>
       <c r="E205" s="7" t="n">
-        <v>77</v>
+        <v>88</v>
       </c>
     </row>
     <row r="206">
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="E208" s="7" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="209">
@@ -8783,7 +8783,7 @@
         </is>
       </c>
       <c r="E251" s="7" t="n">
-        <v>685</v>
+        <v>681</v>
       </c>
     </row>
     <row r="252">
@@ -8833,7 +8833,7 @@
         </is>
       </c>
       <c r="E253" s="7" t="n">
-        <v>553</v>
+        <v>545</v>
       </c>
     </row>
     <row r="254">
@@ -8858,7 +8858,7 @@
         </is>
       </c>
       <c r="E254" s="7" t="n">
-        <v>551</v>
+        <v>545</v>
       </c>
     </row>
     <row r="255">
@@ -8883,7 +8883,7 @@
         </is>
       </c>
       <c r="E255" s="7" t="n">
-        <v>512</v>
+        <v>506</v>
       </c>
     </row>
     <row r="256">
@@ -8908,7 +8908,7 @@
         </is>
       </c>
       <c r="E256" s="7" t="n">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="257">
@@ -9008,7 +9008,7 @@
         </is>
       </c>
       <c r="E260" s="7" t="n">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="261">
@@ -9108,7 +9108,7 @@
         </is>
       </c>
       <c r="E264" s="7" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="265">
@@ -18520,7 +18520,7 @@
         </is>
       </c>
       <c r="D62" s="17" t="n">
-        <v>2366</v>
+        <v>2870</v>
       </c>
     </row>
     <row r="63">
@@ -18540,7 +18540,7 @@
         </is>
       </c>
       <c r="D63" s="17" t="n">
-        <v>699</v>
+        <v>945</v>
       </c>
     </row>
     <row r="64">
@@ -18560,7 +18560,7 @@
         </is>
       </c>
       <c r="D64" s="17" t="n">
-        <v>550</v>
+        <v>683</v>
       </c>
     </row>
     <row r="65">
@@ -18580,7 +18580,7 @@
         </is>
       </c>
       <c r="D65" s="17" t="n">
-        <v>512</v>
+        <v>645</v>
       </c>
     </row>
     <row r="66">
@@ -18596,11 +18596,11 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Action 1</t>
+          <t>Menu_Mobile</t>
         </is>
       </c>
       <c r="D66" s="17" t="n">
-        <v>496</v>
+        <v>609</v>
       </c>
     </row>
     <row r="67">
@@ -18616,11 +18616,11 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Action 2</t>
+          <t>Action 1</t>
         </is>
       </c>
       <c r="D67" s="17" t="n">
-        <v>496</v>
+        <v>600</v>
       </c>
     </row>
     <row r="68">
@@ -18636,11 +18636,11 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Menu_Mobile</t>
+          <t>Action 2</t>
         </is>
       </c>
       <c r="D68" s="17" t="n">
-        <v>482</v>
+        <v>600</v>
       </c>
     </row>
     <row r="69">
@@ -18660,7 +18660,7 @@
         </is>
       </c>
       <c r="D69" s="17" t="n">
-        <v>433</v>
+        <v>545</v>
       </c>
     </row>
     <row r="70">
@@ -18680,7 +18680,7 @@
         </is>
       </c>
       <c r="D70" s="17" t="n">
-        <v>398</v>
+        <v>513</v>
       </c>
     </row>
     <row r="71">
@@ -18700,7 +18700,7 @@
         </is>
       </c>
       <c r="D71" s="17" t="n">
-        <v>398</v>
+        <v>513</v>
       </c>
     </row>
     <row r="72">
@@ -18720,7 +18720,7 @@
         </is>
       </c>
       <c r="D72" s="17" t="n">
-        <v>390</v>
+        <v>503</v>
       </c>
     </row>
     <row r="73">
@@ -18740,7 +18740,7 @@
         </is>
       </c>
       <c r="D73" s="17" t="n">
-        <v>382</v>
+        <v>497</v>
       </c>
     </row>
     <row r="74">
@@ -18760,7 +18760,7 @@
         </is>
       </c>
       <c r="D74" s="17" t="n">
-        <v>328</v>
+        <v>388</v>
       </c>
     </row>
     <row r="75">
@@ -18776,11 +18776,11 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D75" s="17" t="n">
-        <v>324</v>
+        <v>360</v>
       </c>
     </row>
     <row r="76">
@@ -18796,11 +18796,11 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="D76" s="17" t="n">
-        <v>312</v>
+        <v>360</v>
       </c>
     </row>
     <row r="77">
@@ -18816,11 +18816,11 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Line Tracking Vertical</t>
+          <t>medios de pago</t>
         </is>
       </c>
       <c r="D77" s="17" t="n">
-        <v>295</v>
+        <v>320</v>
       </c>
     </row>
     <row r="78">
@@ -18836,11 +18836,11 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>medios de pago</t>
+          <t>Line Tracking Vertical</t>
         </is>
       </c>
       <c r="D78" s="17" t="n">
-        <v>280</v>
+        <v>295</v>
       </c>
     </row>
     <row r="79">
@@ -18860,7 +18860,7 @@
         </is>
       </c>
       <c r="D79" s="17" t="n">
-        <v>116</v>
+        <v>156</v>
       </c>
     </row>
     <row r="80">
@@ -18880,7 +18880,7 @@
         </is>
       </c>
       <c r="D80" s="17" t="n">
-        <v>104</v>
+        <v>130</v>
       </c>
     </row>
     <row r="81">
@@ -18896,11 +18896,11 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>width fixed pagination</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D81" s="17" t="n">
-        <v>104</v>
+        <v>126</v>
       </c>
     </row>
     <row r="82">
@@ -23032,7 +23032,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -23233,7 +23233,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -23313,7 +23313,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -23327,13 +23327,13 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>14419</v>
+        <v>14380</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>22099</v>
+        <v>22048</v>
       </c>
     </row>
     <row r="11">
@@ -23393,7 +23393,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -23407,13 +23407,13 @@
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>172970</v>
+        <v>214056</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>184326</v>
+        <v>227801</v>
       </c>
     </row>
     <row r="13">
@@ -23473,7 +23473,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -23553,7 +23553,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -23633,7 +23633,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -23713,7 +23713,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -23873,7 +23873,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -23953,7 +23953,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -24033,7 +24033,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -24113,7 +24113,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -24193,7 +24193,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-02 22:34 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -764,10 +764,10 @@
         <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>214056</v>
+        <v>213533</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>13745</v>
+        <v>13703</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -1586,10 +1586,10 @@
         <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>198851</v>
+        <v>198328</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>12879</v>
+        <v>12837</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="E175" s="7" t="n">
-        <v>110447</v>
+        <v>110159</v>
       </c>
     </row>
     <row r="176">
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="E176" s="7" t="n">
-        <v>19407</v>
+        <v>19359</v>
       </c>
     </row>
     <row r="177">
@@ -6933,7 +6933,7 @@
         </is>
       </c>
       <c r="E177" s="7" t="n">
-        <v>10336</v>
+        <v>10306</v>
       </c>
     </row>
     <row r="178">
@@ -6958,7 +6958,7 @@
         </is>
       </c>
       <c r="E178" s="7" t="n">
-        <v>9872</v>
+        <v>9848</v>
       </c>
     </row>
     <row r="179">
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>9268</v>
+        <v>9234</v>
       </c>
     </row>
     <row r="180">
@@ -7008,7 +7008,7 @@
         </is>
       </c>
       <c r="E180" s="7" t="n">
-        <v>6266</v>
+        <v>6259</v>
       </c>
     </row>
     <row r="181">
@@ -7033,7 +7033,7 @@
         </is>
       </c>
       <c r="E181" s="7" t="n">
-        <v>4935</v>
+        <v>4923</v>
       </c>
     </row>
     <row r="182">
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="E183" s="7" t="n">
-        <v>2914</v>
+        <v>2904</v>
       </c>
     </row>
     <row r="184">
@@ -7108,7 +7108,7 @@
         </is>
       </c>
       <c r="E184" s="7" t="n">
-        <v>2126</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="185">
@@ -7133,7 +7133,7 @@
         </is>
       </c>
       <c r="E185" s="7" t="n">
-        <v>1953</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="186">
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="E186" s="7" t="n">
-        <v>1935</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="187">
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="E187" s="7" t="n">
-        <v>1690</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="188">
@@ -7208,7 +7208,7 @@
         </is>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1508</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="189">
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="E189" s="7" t="n">
-        <v>1493</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="190">
@@ -7258,7 +7258,7 @@
         </is>
       </c>
       <c r="E190" s="7" t="n">
-        <v>1361</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="191">
@@ -7283,7 +7283,7 @@
         </is>
       </c>
       <c r="E191" s="7" t="n">
-        <v>1276</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="192">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="E192" s="7" t="n">
-        <v>1234</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="193">
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="E193" s="7" t="n">
-        <v>1234</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="194">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E194" s="7" t="n">
-        <v>1010</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="195">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="E195" s="7" t="n">
-        <v>990</v>
+        <v>986</v>
       </c>
     </row>
     <row r="196">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="198">
@@ -7483,7 +7483,7 @@
         </is>
       </c>
       <c r="E199" s="7" t="n">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="200">
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="E208" s="7" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="209">
@@ -18540,7 +18540,7 @@
         </is>
       </c>
       <c r="D63" s="17" t="n">
-        <v>945</v>
+        <v>933</v>
       </c>
     </row>
     <row r="64">
@@ -18560,7 +18560,7 @@
         </is>
       </c>
       <c r="D64" s="17" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="65">
@@ -18580,7 +18580,7 @@
         </is>
       </c>
       <c r="D65" s="17" t="n">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="66">
@@ -18600,7 +18600,7 @@
         </is>
       </c>
       <c r="D66" s="17" t="n">
-        <v>609</v>
+        <v>607</v>
       </c>
     </row>
     <row r="67">
@@ -18680,7 +18680,7 @@
         </is>
       </c>
       <c r="D70" s="17" t="n">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="71">
@@ -18700,7 +18700,7 @@
         </is>
       </c>
       <c r="D71" s="17" t="n">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="72">
@@ -18720,7 +18720,7 @@
         </is>
       </c>
       <c r="D72" s="17" t="n">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="73">
@@ -18740,7 +18740,7 @@
         </is>
       </c>
       <c r="D73" s="17" t="n">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="74">
@@ -18860,7 +18860,7 @@
         </is>
       </c>
       <c r="D79" s="17" t="n">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="80">
@@ -18896,11 +18896,11 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>width fixed pagination</t>
         </is>
       </c>
       <c r="D81" s="17" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="82">
@@ -23410,10 +23410,10 @@
         <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>214056</v>
+        <v>213533</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>227801</v>
+        <v>227236</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-03 16:57 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-02</t>
+          <t>Quarter: Q3 2026  |  2026-07-03</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>73</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>11472</v>
+        <v>11453</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>2122</v>
@@ -2062,7 +2062,7 @@
         <v>14</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>1419</v>
+        <v>1400</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>172</v>
@@ -2224,11 +2224,11 @@
         <v>485</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2366</v>
+        <v>2436</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>17.01%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
@@ -2242,11 +2242,11 @@
         <v>86</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4256</v>
+        <v>4382</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>1.98%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
@@ -2260,11 +2260,11 @@
         <v>58</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>776</v>
+        <v>811</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>6.95%</t>
+          <t>6.67%</t>
         </is>
       </c>
     </row>
@@ -2275,10 +2275,10 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>72256</v>
+        <v>76698</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2314,11 +2314,11 @@
         <v>40</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3782</v>
+        <v>3894</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>1.02%</t>
         </is>
       </c>
     </row>
@@ -2332,11 +2332,11 @@
         <v>34</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>908</v>
+        <v>1005</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>3.61%</t>
+          <t>3.27%</t>
         </is>
       </c>
     </row>
@@ -2350,11 +2350,11 @@
         <v>24</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>8910</v>
+        <v>10521</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>0.27%</t>
+          <t>0.23%</t>
         </is>
       </c>
     </row>
@@ -2368,11 +2368,11 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>11256</v>
+        <v>12673</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>0.18%</t>
         </is>
       </c>
     </row>
@@ -2386,47 +2386,47 @@
         <v>23</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1417</v>
+        <v>1459</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>1.6%</t>
+          <t>1.55%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Accordion</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
         <v>21</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>1008</v>
+        <v>19785</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>0.11%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Accordion</t>
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>18026</v>
+        <v>1108</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>1.86%</t>
         </is>
       </c>
     </row>
@@ -2440,11 +2440,11 @@
         <v>16</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>4184</v>
+        <v>4904</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>0.38%</t>
+          <t>0.33%</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
         <v>13</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1414</v>
+        <v>1420</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         <v>11</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3863</v>
+        <v>3892</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
@@ -16354,11 +16354,11 @@
       </c>
       <c r="D554" s="5" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E554" s="7" t="n">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="555">
@@ -16379,11 +16379,11 @@
       </c>
       <c r="D555" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Tab</t>
         </is>
       </c>
       <c r="E555" s="7" t="n">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="556">
@@ -16408,7 +16408,7 @@
         </is>
       </c>
       <c r="E556" s="7" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="557">
@@ -23032,7 +23032,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -23233,7 +23233,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -23313,7 +23313,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -23393,7 +23393,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -23473,7 +23473,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -23553,7 +23553,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -23633,7 +23633,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -23713,7 +23713,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -23873,7 +23873,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -23953,7 +23953,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -24033,7 +24033,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -24113,7 +24113,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -24193,7 +24193,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -24210,10 +24210,10 @@
         <v>73</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>11472</v>
+        <v>11453</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>13594</v>
+        <v>13575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: adoption report 2026-07-03 22:35 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -764,10 +764,10 @@
         <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>213533</v>
+        <v>214825</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>13703</v>
+        <v>13740</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -1586,10 +1586,10 @@
         <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>198328</v>
+        <v>199620</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>12837</v>
+        <v>12874</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="E175" s="7" t="n">
-        <v>110159</v>
+        <v>110927</v>
       </c>
     </row>
     <row r="176">
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="E176" s="7" t="n">
-        <v>19359</v>
+        <v>19487</v>
       </c>
     </row>
     <row r="177">
@@ -6933,7 +6933,7 @@
         </is>
       </c>
       <c r="E177" s="7" t="n">
-        <v>10306</v>
+        <v>10350</v>
       </c>
     </row>
     <row r="178">
@@ -6958,7 +6958,7 @@
         </is>
       </c>
       <c r="E178" s="7" t="n">
-        <v>9848</v>
+        <v>9912</v>
       </c>
     </row>
     <row r="179">
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>9234</v>
+        <v>9288</v>
       </c>
     </row>
     <row r="180">
@@ -7008,7 +7008,7 @@
         </is>
       </c>
       <c r="E180" s="7" t="n">
-        <v>6259</v>
+        <v>6270</v>
       </c>
     </row>
     <row r="181">
@@ -7033,7 +7033,7 @@
         </is>
       </c>
       <c r="E181" s="7" t="n">
-        <v>4923</v>
+        <v>4955</v>
       </c>
     </row>
     <row r="182">
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="E183" s="7" t="n">
-        <v>2904</v>
+        <v>2939</v>
       </c>
     </row>
     <row r="184">
@@ -7108,7 +7108,7 @@
         </is>
       </c>
       <c r="E184" s="7" t="n">
-        <v>2120</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="185">
@@ -7133,7 +7133,7 @@
         </is>
       </c>
       <c r="E185" s="7" t="n">
-        <v>1947</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="186">
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="E186" s="7" t="n">
-        <v>1929</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="187">
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="E187" s="7" t="n">
-        <v>1682</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="188">
@@ -7208,7 +7208,7 @@
         </is>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1502</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="189">
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="E189" s="7" t="n">
-        <v>1487</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="190">
@@ -7258,7 +7258,7 @@
         </is>
       </c>
       <c r="E190" s="7" t="n">
-        <v>1357</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="191">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="E192" s="7" t="n">
-        <v>1231</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="193">
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="E193" s="7" t="n">
-        <v>1231</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="194">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E194" s="7" t="n">
-        <v>1006</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="195">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="E195" s="7" t="n">
-        <v>986</v>
+        <v>994</v>
       </c>
     </row>
     <row r="196">
@@ -7429,11 +7429,11 @@
       </c>
       <c r="D197" s="5" t="inlineStr">
         <is>
-          <t>Breadcrumb</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="198">
@@ -7454,11 +7454,11 @@
       </c>
       <c r="D198" s="5" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Breadcrumb</t>
         </is>
       </c>
       <c r="E198" s="7" t="n">
-        <v>503</v>
+        <v>519</v>
       </c>
     </row>
     <row r="199">
@@ -7483,7 +7483,7 @@
         </is>
       </c>
       <c r="E199" s="7" t="n">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="200">
@@ -18560,7 +18560,7 @@
         </is>
       </c>
       <c r="D64" s="17" t="n">
-        <v>681</v>
+        <v>682</v>
       </c>
     </row>
     <row r="65">
@@ -18580,7 +18580,7 @@
         </is>
       </c>
       <c r="D65" s="17" t="n">
-        <v>643</v>
+        <v>650</v>
       </c>
     </row>
     <row r="66">
@@ -18600,7 +18600,7 @@
         </is>
       </c>
       <c r="D66" s="17" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
     </row>
     <row r="67">
@@ -18680,7 +18680,7 @@
         </is>
       </c>
       <c r="D70" s="17" t="n">
-        <v>511</v>
+        <v>518</v>
       </c>
     </row>
     <row r="71">
@@ -18700,7 +18700,7 @@
         </is>
       </c>
       <c r="D71" s="17" t="n">
-        <v>511</v>
+        <v>518</v>
       </c>
     </row>
     <row r="72">
@@ -18720,7 +18720,7 @@
         </is>
       </c>
       <c r="D72" s="17" t="n">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="73">
@@ -18740,7 +18740,7 @@
         </is>
       </c>
       <c r="D73" s="17" t="n">
-        <v>495</v>
+        <v>502</v>
       </c>
     </row>
     <row r="74">
@@ -18896,11 +18896,11 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>width fixed pagination</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D81" s="17" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82">
@@ -23410,10 +23410,10 @@
         <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>213533</v>
+        <v>214825</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>227236</v>
+        <v>228565</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-06 18:14 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-03</t>
+          <t>Quarter: Q3 2026  |  2026-07-06</t>
         </is>
       </c>
     </row>
@@ -727,10 +727,10 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7739</v>
+        <v>7804</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>821</v>
+        <v>844</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>38</v>
@@ -764,10 +764,10 @@
         <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>214825</v>
+        <v>215167</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>13740</v>
+        <v>13747</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -1484,10 +1484,10 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>704</v>
+        <v>769</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>187</v>
+        <v>210</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>20</v>
@@ -1586,10 +1586,10 @@
         <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>199620</v>
+        <v>199962</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>12874</v>
+        <v>12881</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -2260,11 +2260,11 @@
         <v>58</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>6.67%</t>
+          <t>6.62%</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
         <v>56</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>76698</v>
+        <v>77514</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2332,11 +2332,11 @@
         <v>34</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1005</v>
+        <v>1065</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>3.27%</t>
+          <t>3.09%</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>10521</v>
+        <v>10569</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>12673</v>
+        <v>12732</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
@@ -2404,7 +2404,7 @@
         <v>21</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>19785</v>
+        <v>19828</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
@@ -2440,11 +2440,11 @@
         <v>16</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>4904</v>
+        <v>4955</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.32%</t>
         </is>
       </c>
     </row>
@@ -2458,11 +2458,11 @@
         <v>13</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1420</v>
+        <v>1434</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.9%</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
         <v>11</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3892</v>
+        <v>3893</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
@@ -4733,7 +4733,7 @@
         </is>
       </c>
       <c r="E89" s="7" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="90">
@@ -4754,11 +4754,11 @@
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
-        <v>73</v>
+        <v>85</v>
       </c>
     </row>
     <row r="91">
@@ -4779,11 +4779,11 @@
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="92">
@@ -4808,7 +4808,7 @@
         </is>
       </c>
       <c r="E92" s="7" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="93">
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="E93" s="7" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="94">
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="E94" s="7" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="95">
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="E95" s="7" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="96">
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="E100" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="101">
@@ -5058,7 +5058,7 @@
         </is>
       </c>
       <c r="E102" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="103">
@@ -5083,7 +5083,7 @@
         </is>
       </c>
       <c r="E103" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="E175" s="7" t="n">
-        <v>110927</v>
+        <v>111119</v>
       </c>
     </row>
     <row r="176">
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="E176" s="7" t="n">
-        <v>19487</v>
+        <v>19519</v>
       </c>
     </row>
     <row r="177">
@@ -6933,7 +6933,7 @@
         </is>
       </c>
       <c r="E177" s="7" t="n">
-        <v>10350</v>
+        <v>10370</v>
       </c>
     </row>
     <row r="178">
@@ -6958,7 +6958,7 @@
         </is>
       </c>
       <c r="E178" s="7" t="n">
-        <v>9912</v>
+        <v>9928</v>
       </c>
     </row>
     <row r="179">
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>9288</v>
+        <v>9300</v>
       </c>
     </row>
     <row r="180">
@@ -7008,7 +7008,7 @@
         </is>
       </c>
       <c r="E180" s="7" t="n">
-        <v>6270</v>
+        <v>6275</v>
       </c>
     </row>
     <row r="181">
@@ -7033,7 +7033,7 @@
         </is>
       </c>
       <c r="E181" s="7" t="n">
-        <v>4955</v>
+        <v>4963</v>
       </c>
     </row>
     <row r="182">
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="E183" s="7" t="n">
-        <v>2939</v>
+        <v>2944</v>
       </c>
     </row>
     <row r="184">
@@ -7108,7 +7108,7 @@
         </is>
       </c>
       <c r="E184" s="7" t="n">
-        <v>2136</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="185">
@@ -7133,7 +7133,7 @@
         </is>
       </c>
       <c r="E185" s="7" t="n">
-        <v>1968</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="186">
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="E186" s="7" t="n">
-        <v>1950</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="187">
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="E187" s="7" t="n">
-        <v>1686</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="188">
@@ -7208,7 +7208,7 @@
         </is>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1523</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="189">
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="E189" s="7" t="n">
-        <v>1490</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="190">
@@ -7258,7 +7258,7 @@
         </is>
       </c>
       <c r="E190" s="7" t="n">
-        <v>1365</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="191">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="E192" s="7" t="n">
-        <v>1239</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="193">
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="E193" s="7" t="n">
-        <v>1239</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="194">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E194" s="7" t="n">
-        <v>1020</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="195">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="E195" s="7" t="n">
-        <v>994</v>
+        <v>996</v>
       </c>
     </row>
     <row r="196">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>519</v>
+        <v>539</v>
       </c>
     </row>
     <row r="198">
@@ -7458,7 +7458,7 @@
         </is>
       </c>
       <c r="E198" s="7" t="n">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="199">
@@ -7483,7 +7483,7 @@
         </is>
       </c>
       <c r="E199" s="7" t="n">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="200">
@@ -18160,7 +18160,7 @@
         </is>
       </c>
       <c r="D44" s="17" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45">
@@ -18176,11 +18176,11 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Atajos | Beneficios (new)</t>
+          <t>NorthEast</t>
         </is>
       </c>
       <c r="D45" s="17" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46">
@@ -18196,11 +18196,11 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Menu_Mobile</t>
+          <t>Atajos | Beneficios (new)</t>
         </is>
       </c>
       <c r="D46" s="17" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47">
@@ -18216,11 +18216,11 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>NorthEast</t>
+          <t>Menu_Mobile</t>
         </is>
       </c>
       <c r="D47" s="17" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48">
@@ -18416,7 +18416,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Infotip</t>
+          <t>PersonalInjuy</t>
         </is>
       </c>
       <c r="D57" s="17" t="n">
@@ -18436,7 +18436,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>trofeo</t>
+          <t>Infotip</t>
         </is>
       </c>
       <c r="D58" s="17" t="n">
@@ -18456,11 +18456,11 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>vida ley</t>
+          <t>trofeo</t>
         </is>
       </c>
       <c r="D59" s="17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60">
@@ -18476,7 +18476,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>tratamiento</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D60" s="17" t="n">
@@ -18496,7 +18496,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Right Label</t>
+          <t>vida ley</t>
         </is>
       </c>
       <c r="D61" s="17" t="n">
@@ -18560,7 +18560,7 @@
         </is>
       </c>
       <c r="D64" s="17" t="n">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="65">
@@ -18580,7 +18580,7 @@
         </is>
       </c>
       <c r="D65" s="17" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
     </row>
     <row r="66">
@@ -18600,7 +18600,7 @@
         </is>
       </c>
       <c r="D66" s="17" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
     </row>
     <row r="67">
@@ -18680,7 +18680,7 @@
         </is>
       </c>
       <c r="D70" s="17" t="n">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="71">
@@ -18700,7 +18700,7 @@
         </is>
       </c>
       <c r="D71" s="17" t="n">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="72">
@@ -18720,7 +18720,7 @@
         </is>
       </c>
       <c r="D72" s="17" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="73">
@@ -18740,7 +18740,7 @@
         </is>
       </c>
       <c r="D73" s="17" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="74">
@@ -23032,7 +23032,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -23233,7 +23233,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -23313,7 +23313,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -23393,7 +23393,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -23410,10 +23410,10 @@
         <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>214825</v>
+        <v>215167</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>228565</v>
+        <v>228914</v>
       </c>
     </row>
     <row r="13">
@@ -23473,7 +23473,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -23553,7 +23553,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -23570,10 +23570,10 @@
         <v>8</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>7739</v>
+        <v>7804</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>8560</v>
+        <v>8648</v>
       </c>
     </row>
     <row r="17">
@@ -23633,7 +23633,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -23713,7 +23713,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -23873,7 +23873,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -23953,7 +23953,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -24033,7 +24033,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -24113,7 +24113,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -24193,7 +24193,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-07 17:44 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-06</t>
+          <t>Quarter: Q3 2026  |  2026-07-07</t>
         </is>
       </c>
     </row>
@@ -690,10 +690,10 @@
         <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3704</v>
+        <v>3712</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>27</v>
@@ -1450,10 +1450,10 @@
         <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2511</v>
+        <v>2519</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>25</v>
@@ -2224,11 +2224,11 @@
         <v>485</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2436</v>
+        <v>2461</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.46%</t>
         </is>
       </c>
     </row>
@@ -2242,11 +2242,11 @@
         <v>86</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4382</v>
+        <v>4427</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>1.92%</t>
+          <t>1.91%</t>
         </is>
       </c>
     </row>
@@ -2260,11 +2260,11 @@
         <v>58</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>818</v>
+        <v>823</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>6.58%</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
         <v>56</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>77514</v>
+        <v>78461</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2314,11 +2314,11 @@
         <v>40</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3894</v>
+        <v>3934</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1.02%</t>
+          <t>1.01%</t>
         </is>
       </c>
     </row>
@@ -2332,11 +2332,11 @@
         <v>34</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1065</v>
+        <v>1102</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>3.09%</t>
+          <t>2.99%</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>10569</v>
+        <v>10578</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>12732</v>
+        <v>12788</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
@@ -2386,11 +2386,11 @@
         <v>23</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1459</v>
+        <v>1474</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>1.54%</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
         <v>21</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>19828</v>
+        <v>19885</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
         <v>21</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>1.86%</t>
+          <t>1.85%</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>4955</v>
+        <v>5062</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
@@ -2458,11 +2458,11 @@
         <v>13</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1434</v>
+        <v>1449</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>0.9%</t>
+          <t>0.89%</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
         <v>11</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3893</v>
+        <v>3895</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="63">
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65">
@@ -4133,7 +4133,7 @@
         </is>
       </c>
       <c r="E65" s="7" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="66">
@@ -4433,7 +4433,7 @@
         </is>
       </c>
       <c r="E77" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="78">
@@ -17780,7 +17780,7 @@
         </is>
       </c>
       <c r="D30" s="17" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31">
@@ -22932,7 +22932,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -23053,7 +23053,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -23133,7 +23133,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -23293,7 +23293,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -23453,7 +23453,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -23533,7 +23533,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -23613,7 +23613,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -23630,10 +23630,10 @@
         <v>12</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>3704</v>
+        <v>3712</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>4291</v>
+        <v>4302</v>
       </c>
     </row>
     <row r="21">
@@ -23693,7 +23693,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -23773,7 +23773,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -23853,7 +23853,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -23933,7 +23933,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -24013,7 +24013,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -24093,7 +24093,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-08 17:04 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-07</t>
+          <t>Quarter: Q3 2026  |  2026-07-08</t>
         </is>
       </c>
     </row>
@@ -690,10 +690,10 @@
         <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3634</v>
+        <v>3653</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>27</v>
@@ -764,7 +764,7 @@
         <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>215167</v>
+        <v>215415</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>13747</v>
@@ -1450,10 +1450,10 @@
         <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2441</v>
+        <v>2460</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>26</v>
@@ -1586,7 +1586,7 @@
         <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>199962</v>
+        <v>200210</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>12881</v>
@@ -2224,11 +2224,11 @@
         <v>485</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2461</v>
+        <v>2471</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>16.41%</t>
         </is>
       </c>
     </row>
@@ -2242,11 +2242,11 @@
         <v>86</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4427</v>
+        <v>4454</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.89%</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
         <v>58</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
         <v>56</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>78461</v>
+        <v>78975</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2314,11 +2314,11 @@
         <v>40</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3934</v>
+        <v>3958</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.0%</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>12788</v>
+        <v>12816</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
@@ -2386,11 +2386,11 @@
         <v>23</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1474</v>
+        <v>1484</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>1.53%</t>
         </is>
       </c>
     </row>
@@ -2404,11 +2404,11 @@
         <v>21</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>19885</v>
+        <v>20008</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.1%</t>
         </is>
       </c>
     </row>
@@ -2422,11 +2422,11 @@
         <v>21</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>1112</v>
+        <v>1119</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>1.85%</t>
+          <t>1.84%</t>
         </is>
       </c>
     </row>
@@ -2440,11 +2440,11 @@
         <v>16</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>5062</v>
+        <v>5185</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>0.32%</t>
+          <t>0.31%</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
         <v>11</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3895</v>
+        <v>3899</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63">
@@ -4083,7 +4083,7 @@
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="64">
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65">
@@ -4133,7 +4133,7 @@
         </is>
       </c>
       <c r="E65" s="7" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="66">
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="E66" s="7" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="67">
@@ -4208,7 +4208,7 @@
         </is>
       </c>
       <c r="E68" s="7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69">
@@ -4283,7 +4283,7 @@
         </is>
       </c>
       <c r="E71" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="72">
@@ -4354,11 +4354,11 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="75">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4404,11 +4404,11 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="77">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E194" s="7" t="n">
-        <v>539</v>
+        <v>787</v>
       </c>
     </row>
     <row r="195">
@@ -17645,7 +17645,7 @@
         </is>
       </c>
       <c r="D22" s="17" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23">
@@ -17665,7 +17665,7 @@
         </is>
       </c>
       <c r="D23" s="17" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24">
@@ -17685,7 +17685,7 @@
         </is>
       </c>
       <c r="D24" s="17" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25">
@@ -22957,7 +22957,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -23078,7 +23078,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -23158,7 +23158,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -23238,7 +23238,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -23318,7 +23318,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -23335,10 +23335,10 @@
         <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>215167</v>
+        <v>215415</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>228914</v>
+        <v>229162</v>
       </c>
     </row>
     <row r="13">
@@ -23398,7 +23398,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -23478,7 +23478,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -23558,7 +23558,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -23638,7 +23638,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -23655,10 +23655,10 @@
         <v>12</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>3634</v>
+        <v>3653</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>4262</v>
+        <v>4284</v>
       </c>
     </row>
     <row r="21">
@@ -23718,7 +23718,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -23798,7 +23798,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -23878,7 +23878,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -23958,7 +23958,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -24038,7 +24038,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -24118,7 +24118,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-08 22:37 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -690,10 +690,10 @@
         <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3653</v>
+        <v>3634</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>27</v>
@@ -1171,10 +1171,10 @@
         <v>6</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G19" s="8" t="n">
         <v>19</v>
@@ -1450,10 +1450,10 @@
         <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2460</v>
+        <v>2441</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>26</v>
@@ -2096,10 +2096,10 @@
         <v>6</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>19</v>
@@ -4058,7 +4058,7 @@
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="63">
@@ -4083,7 +4083,7 @@
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="64">
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="65">
@@ -4133,7 +4133,7 @@
         </is>
       </c>
       <c r="E65" s="7" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="66">
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="E66" s="7" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67">
@@ -4208,7 +4208,7 @@
         </is>
       </c>
       <c r="E68" s="7" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="69">
@@ -4283,7 +4283,7 @@
         </is>
       </c>
       <c r="E71" s="7" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="72">
@@ -4354,11 +4354,11 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Text Area</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="75">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>title_+_phones</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>title_+_phones</t>
+          <t>Text Area</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -16858,7 +16858,7 @@
         </is>
       </c>
       <c r="E574" s="7" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="575">
@@ -17645,7 +17645,7 @@
         </is>
       </c>
       <c r="D22" s="17" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23">
@@ -17665,7 +17665,7 @@
         </is>
       </c>
       <c r="D23" s="17" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24">
@@ -17685,7 +17685,7 @@
         </is>
       </c>
       <c r="D24" s="17" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25">
@@ -22465,7 +22465,7 @@
         </is>
       </c>
       <c r="D263" s="17" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="264">
@@ -22585,7 +22585,7 @@
         </is>
       </c>
       <c r="D269" s="17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="270">
@@ -23095,10 +23095,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1625</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="7">
@@ -23655,10 +23655,10 @@
         <v>12</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>3653</v>
+        <v>3634</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>4284</v>
+        <v>4262</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-09 17:56 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-08</t>
+          <t>Quarter: Q3 2026  |  2026-07-09</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7804</v>
+        <v>7808</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>844</v>
@@ -764,7 +764,7 @@
         <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>215415</v>
+        <v>215429</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>13747</v>
@@ -1174,7 +1174,7 @@
         <v>1425</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G19" s="8" t="n">
         <v>19</v>
@@ -1484,7 +1484,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>210</v>
@@ -1586,7 +1586,7 @@
         <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>200210</v>
+        <v>200224</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>12881</v>
@@ -2099,7 +2099,7 @@
         <v>1425</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>19</v>
@@ -2224,11 +2224,11 @@
         <v>485</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2471</v>
+        <v>2476</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>16.38%</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
         <v>86</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4454</v>
+        <v>4463</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
         <v>56</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>78975</v>
+        <v>79894</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         <v>40</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3958</v>
+        <v>3966</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
@@ -2332,11 +2332,11 @@
         <v>34</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1102</v>
+        <v>1130</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>2.99%</t>
+          <t>2.92%</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>10578</v>
+        <v>10630</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>12816</v>
+        <v>12873</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
@@ -2386,11 +2386,11 @@
         <v>23</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1484</v>
+        <v>1487</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.52%</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
         <v>21</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>20008</v>
+        <v>20317</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
         <v>21</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>1119</v>
+        <v>1134</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>1.84%</t>
+          <t>1.82%</t>
         </is>
       </c>
     </row>
@@ -2440,11 +2440,11 @@
         <v>16</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>5185</v>
+        <v>5443</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.29%</t>
         </is>
       </c>
     </row>
@@ -2458,29 +2458,29 @@
         <v>13</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1449</v>
+        <v>1463</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>0.88%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Checkbox Atom</t>
+          <t>Option Group</t>
         </is>
       </c>
       <c r="B19" s="12" t="n">
         <v>11</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3899</v>
+        <v>351</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>3.04%</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
         </is>
       </c>
       <c r="E87" s="7" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="88">
@@ -4983,7 +4983,7 @@
         </is>
       </c>
       <c r="E99" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="100">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E194" s="7" t="n">
-        <v>787</v>
+        <v>801</v>
       </c>
     </row>
     <row r="195">
@@ -22461,7 +22461,7 @@
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>SecciónDescripción</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="D263" s="17" t="n">
@@ -22481,7 +22481,7 @@
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="D264" s="17" t="n">
@@ -22501,11 +22501,11 @@
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>SecciónDescripción</t>
         </is>
       </c>
       <c r="D265" s="17" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="266">
@@ -22957,7 +22957,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -23078,7 +23078,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -23098,7 +23098,7 @@
         <v>1425</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1624</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="7">
@@ -23158,7 +23158,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -23238,7 +23238,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -23318,7 +23318,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -23335,10 +23335,10 @@
         <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>215415</v>
+        <v>215429</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>229162</v>
+        <v>229176</v>
       </c>
     </row>
     <row r="13">
@@ -23398,7 +23398,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -23478,7 +23478,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -23495,10 +23495,10 @@
         <v>8</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>7804</v>
+        <v>7808</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>8648</v>
+        <v>8652</v>
       </c>
     </row>
     <row r="17">
@@ -23558,7 +23558,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -23638,7 +23638,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -23718,7 +23718,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -23798,7 +23798,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -23878,7 +23878,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -23958,7 +23958,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -24038,7 +24038,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -24118,7 +24118,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-09 22:52 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -727,10 +727,10 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7808</v>
+        <v>7743</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>844</v>
+        <v>821</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>38</v>
@@ -1484,10 +1484,10 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>773</v>
+        <v>708</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>210</v>
+        <v>187</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>20</v>
@@ -4658,7 +4658,7 @@
         </is>
       </c>
       <c r="E86" s="7" t="n">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="87">
@@ -4679,11 +4679,11 @@
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Átomo</t>
+          <t>Alert</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="88">
@@ -4704,11 +4704,11 @@
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Átomo</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="89">
@@ -4733,7 +4733,7 @@
         </is>
       </c>
       <c r="E89" s="7" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="90">
@@ -4758,7 +4758,7 @@
         </is>
       </c>
       <c r="E90" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="91">
@@ -4783,7 +4783,7 @@
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="92">
@@ -4808,7 +4808,7 @@
         </is>
       </c>
       <c r="E92" s="7" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="93">
@@ -4933,7 +4933,7 @@
         </is>
       </c>
       <c r="E97" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98">
@@ -4983,7 +4983,7 @@
         </is>
       </c>
       <c r="E99" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100">
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="E100" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="101">
@@ -18085,7 +18085,7 @@
         </is>
       </c>
       <c r="D44" s="17" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45">
@@ -18101,11 +18101,11 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>NorthEast</t>
+          <t>Atajos | Beneficios (new)</t>
         </is>
       </c>
       <c r="D45" s="17" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46">
@@ -18121,11 +18121,11 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Atajos | Beneficios (new)</t>
+          <t>Menu_Mobile</t>
         </is>
       </c>
       <c r="D46" s="17" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47">
@@ -18141,11 +18141,11 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Menu_Mobile</t>
+          <t>NorthEast</t>
         </is>
       </c>
       <c r="D47" s="17" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48">
@@ -18341,7 +18341,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>PersonalInjuy</t>
+          <t>Infotip</t>
         </is>
       </c>
       <c r="D57" s="17" t="n">
@@ -18361,7 +18361,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Infotip</t>
+          <t>trofeo</t>
         </is>
       </c>
       <c r="D58" s="17" t="n">
@@ -18381,11 +18381,11 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>trofeo</t>
+          <t>vida ley</t>
         </is>
       </c>
       <c r="D59" s="17" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="60">
@@ -18401,7 +18401,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>tratamiento</t>
         </is>
       </c>
       <c r="D60" s="17" t="n">
@@ -18421,7 +18421,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>vida ley</t>
+          <t>Right Label</t>
         </is>
       </c>
       <c r="D61" s="17" t="n">
@@ -23495,10 +23495,10 @@
         <v>8</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>7808</v>
+        <v>7743</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>8652</v>
+        <v>8564</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-10 22:31 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -764,10 +764,10 @@
         <v>50</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>215429</v>
+        <v>216174</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>13747</v>
+        <v>13778</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>47</v>
@@ -1586,10 +1586,10 @@
         <v>43</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>200224</v>
+        <v>200969</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>12881</v>
+        <v>12912</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>42</v>
@@ -6758,7 +6758,7 @@
         </is>
       </c>
       <c r="E170" s="7" t="n">
-        <v>111119</v>
+        <v>111599</v>
       </c>
     </row>
     <row r="171">
@@ -6783,7 +6783,7 @@
         </is>
       </c>
       <c r="E171" s="7" t="n">
-        <v>19519</v>
+        <v>19599</v>
       </c>
     </row>
     <row r="172">
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="E172" s="7" t="n">
-        <v>10370</v>
+        <v>10420</v>
       </c>
     </row>
     <row r="173">
@@ -6833,7 +6833,7 @@
         </is>
       </c>
       <c r="E173" s="7" t="n">
-        <v>9928</v>
+        <v>9968</v>
       </c>
     </row>
     <row r="174">
@@ -6858,7 +6858,7 @@
         </is>
       </c>
       <c r="E174" s="7" t="n">
-        <v>9300</v>
+        <v>9320</v>
       </c>
     </row>
     <row r="175">
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="E175" s="7" t="n">
-        <v>6275</v>
+        <v>6285</v>
       </c>
     </row>
     <row r="176">
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="E176" s="7" t="n">
-        <v>4963</v>
+        <v>4983</v>
       </c>
     </row>
     <row r="177">
@@ -6933,7 +6933,7 @@
         </is>
       </c>
       <c r="E177" s="7" t="n">
-        <v>3651</v>
+        <v>3656</v>
       </c>
     </row>
     <row r="178">
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>2140</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="180">
@@ -7133,7 +7133,7 @@
         </is>
       </c>
       <c r="E185" s="7" t="n">
-        <v>1367</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="186">
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="E187" s="7" t="n">
-        <v>1241</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="188">
@@ -7208,7 +7208,7 @@
         </is>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1241</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="189">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="E196" s="7" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="197">
@@ -7429,11 +7429,11 @@
       </c>
       <c r="D197" s="5" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>236</v>
+        <v>245</v>
       </c>
     </row>
     <row r="198">
@@ -7679,7 +7679,7 @@
       </c>
       <c r="D207" s="5" t="inlineStr">
         <is>
-          <t>Menu title</t>
+          <t>Dropdown Input</t>
         </is>
       </c>
       <c r="E207" s="7" t="n">
@@ -7704,11 +7704,11 @@
       </c>
       <c r="D208" s="5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Menu title</t>
         </is>
       </c>
       <c r="E208" s="7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="209">
@@ -7729,11 +7729,11 @@
       </c>
       <c r="D209" s="5" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E209" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="210">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="D210" s="5" t="inlineStr">
         <is>
-          <t>Dropdown Input</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="E210" s="7" t="n">
@@ -23285,10 +23285,10 @@
         <v>50</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>215429</v>
+        <v>216174</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>229176</v>
+        <v>229952</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-14 16:11 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-13</t>
+          <t>Quarter: Q3 2026  |  2026-07-14</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-15 16:17 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-14</t>
+          <t>Quarter: Q3 2026  |  2026-07-15</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-16 16:14 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-15</t>
+          <t>Quarter: Q3 2026  |  2026-07-16</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-17 16:11 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-16</t>
+          <t>Quarter: Q3 2026  |  2026-07-17</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-20 16:23 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-17</t>
+          <t>Quarter: Q3 2026  |  2026-07-20</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-21 16:20 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-20</t>
+          <t>Quarter: Q3 2026  |  2026-07-21</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-22 16:18 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-21</t>
+          <t>Quarter: Q3 2026  |  2026-07-22</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-23 16:24 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-22</t>
+          <t>Quarter: Q3 2026  |  2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-24 16:34 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-23</t>
+          <t>Quarter: Q3 2026  |  2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-27 16:55 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-24</t>
+          <t>Quarter: Q3 2026  |  2026-07-27</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-28 16:39 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-27</t>
+          <t>Quarter: Q3 2026  |  2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-29 16:18 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-28</t>
+          <t>Quarter: Q3 2026  |  2026-07-29</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-30 16:24 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-29</t>
+          <t>Quarter: Q3 2026  |  2026-07-30</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-07-31 16:42 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-30</t>
+          <t>Quarter: Q3 2026  |  2026-07-31</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-03 17:07 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-07-31</t>
+          <t>Quarter: Q3 2026  |  2026-08-03</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-04 16:49 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-03</t>
+          <t>Quarter: Q3 2026  |  2026-08-04</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-05 16:29 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-04</t>
+          <t>Quarter: Q3 2026  |  2026-08-05</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-07 01:00 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-05</t>
+          <t>Quarter: Q3 2026  |  2026-08-07</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-10 15:56 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-07</t>
+          <t>Quarter: Q3 2026  |  2026-08-10</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-11 15:57 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-10</t>
+          <t>Quarter: Q3 2026  |  2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-12 15:55 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-11</t>
+          <t>Quarter: Q3 2026  |  2026-08-12</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-13 15:55 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-12</t>
+          <t>Quarter: Q3 2026  |  2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-14 15:46 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-13</t>
+          <t>Quarter: Q3 2026  |  2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-17 15:20 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-14</t>
+          <t>Quarter: Q3 2026  |  2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-18 15:26 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-17</t>
+          <t>Quarter: Q3 2026  |  2026-08-18</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-19 15:26 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-18</t>
+          <t>Quarter: Q3 2026  |  2026-08-19</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-20 15:29 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-19</t>
+          <t>Quarter: Q3 2026  |  2026-08-20</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-21 15:28 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-20</t>
+          <t>Quarter: Q3 2026  |  2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-24 15:35 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-21</t>
+          <t>Quarter: Q3 2026  |  2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-25 15:38 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-24</t>
+          <t>Quarter: Q3 2026  |  2026-08-25</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-26 16:14 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-25</t>
+          <t>Quarter: Q3 2026  |  2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-27 00:22 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-26</t>
+          <t>Quarter: Q3 2026  |  2026-08-27</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-28 00:13 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-27</t>
+          <t>Quarter: Q3 2026  |  2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-29 02:59 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-28</t>
+          <t>Quarter: Q3 2026  |  2026-08-29</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-08-31 20:36 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-29</t>
+          <t>Quarter: Q3 2026  |  2026-08-31</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-01 00:16 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-08-31</t>
+          <t>Quarter: Q3 2026  |  2026-09-01</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-02 18:23 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-01</t>
+          <t>Quarter: Q3 2026  |  2026-09-02</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-03 18:18 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-02</t>
+          <t>Quarter: Q3 2026  |  2026-09-03</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-04 18:01 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-03</t>
+          <t>Quarter: Q3 2026  |  2026-09-04</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-07 18:58 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-04</t>
+          <t>Quarter: Q3 2026  |  2026-09-07</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-08 18:16 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-07</t>
+          <t>Quarter: Q3 2026  |  2026-09-08</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-09 18:16 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-08</t>
+          <t>Quarter: Q3 2026  |  2026-09-09</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-10 18:01 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-09</t>
+          <t>Quarter: Q3 2026  |  2026-09-10</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-11 18:08 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-10</t>
+          <t>Quarter: Q3 2026  |  2026-09-11</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>